<commit_message>
Record AI hover header deployment
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rb811a71292f54545"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Rc1b217112e82471c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R84717f123dcf49ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Ra155042876284ddf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R6dad2826f1d248e1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R03c1f8404104435c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R1d5e09dcf3d64d81"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R484915867e924352"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R8eb0ec8c6fd54623"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rb377c6d1ab794535"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R24bd084539464755"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="Ra35847add88f40ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="Re54a9625d1824f53"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R5cae693d7538473f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R4182adbce9ac483f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R903dbbfd676c4990"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R6d5af90071b040d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R12c7b385aa64432c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R5daa14f9a0454475"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="Rd57d53dbce3c42bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Rcd0b2064a5ab4dc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Rea325d29a3124c6a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Rbc03739233504958"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R22c1fb89e1f54fe6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R109019d91860456d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Rb4513b07c98f4a99"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R832533ecf36840cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R77689cf6c0464249"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="Rd4e2554fd18c4e32"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Ra6795521920e42b3"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4735,6 +4735,35 @@
         <x:v>NOTE-STUDIO-NOTEBOOK-INLINE-EXPAND</x:v>
       </x:c>
     </x:row>
+    <x:row r="115" ht="132" customHeight="1">
+      <x:c r="A115" s="19" t="str">
+        <x:v>PATCH-AI-HOVER-HEADER-2026-10-02</x:v>
+      </x:c>
+      <x:c r="B115" s="19" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="C115" s="19" t="str">
+        <x:v>완료·운영 배포·실화면 검증</x:v>
+      </x:c>
+      <x:c r="D115" s="19" t="str">
+        <x:v>AI 에이전트 상단바가 너무 두꺼우니 평소 숨기고 상단에 마우스를 올렸을 때 나타나며 벗어나면 사라지게 하고, 동작 범위를 정확히 제한해 달라는 요청.</x:v>
+      </x:c>
+      <x:c r="E115" s="19" t="str">
+        <x:v>기존 52px 헤더가 항상 자리를 차지해 대화·진행도 영역이 줄었다. hover만 단순 적용하면 설정 버튼을 누른 뒤 메뉴로 이동할 때 헤더가 닫히거나, focus-within 때문에 설정 종료 후에도 헤더가 남을 수 있었다.</x:v>
+      </x:c>
+      <x:c r="F115" s="19" t="str">
+        <x:v>헤더를 문서 흐름에서 제거한 overlay로 바꾸고 최상단 8px만 reveal target으로 지정했다. 헤더 자체 hover와 키보드 focus-visible은 유지하며 설정이 열린 동안만 data-pinned로 고정했다. 마우스 클릭 포커스는 잔류 조건에서 제외했다.</x:v>
+      </x:c>
+      <x:c r="G115" s="19" t="str">
+        <x:v>정적 UI 계약 121개 소스, production build, react-pdf 9.2.1/PDF.js 4.8.69 통과. 운영 main.f2494265.js 배포와 SHA 일치, 내부·공개 HTTP 200, 필수 서비스 active. Chrome 실화면에서 기본 opacity 0, top hover opacity 1, 헤더 내부 유지, 외부 이탈 opacity 0, 설정 중 pinned true, 설정 종료 후 pinned false·opacity 0, console error 0건을 확인했다.</x:v>
+      </x:c>
+      <x:c r="H115" s="19" t="str">
+        <x:v>8px 감지 띠는 패널 너비 전체에만 존재하고 파일 작업공간을 덮지 않는다. 터치 환경은 기존 상단 AI 버튼으로 패널을 닫고 설정은 키보드 focus-visible 경로를 유지한다.</x:v>
+      </x:c>
+      <x:c r="I115" s="19"/>
+      <x:c r="J115" s="19"/>
+      <x:c r="K115" s="19"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5866,6 +5895,17 @@
         <x:v>전체 노트북 목록의 각 행 왼쪽 버튼으로 해당 노트북 하위 목록을 펼쳐 보고, 노트북 선택 시 전용 보기로 들어가며, 상단의 빽빽하고 불필요한 버튼은 핵심 동작만 남기라는 요청.</x:v>
       </x:c>
     </x:row>
+    <x:row r="102" ht="82" customHeight="1">
+      <x:c r="A102" s="19" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="B102" s="19" t="str">
+        <x:v>AI 에이전트 자동 숨김 상단바</x:v>
+      </x:c>
+      <x:c r="C102" s="19" t="str">
+        <x:v>AI 에이전트 상단바가 너무 두꺼우므로 평소에는 숨기고 패널 상단에 마우스를 정확히 올렸을 때 나타나며, 벗어나면 사라지도록 동작 범위를 안전하게 설정해 달라는 요청.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6543,6 +6583,23 @@
       </x:c>
       <x:c r="E54" t="str">
         <x:v>실행은 Docker network none/non-root/read-only root와 선택 노트북 rw만 허용한다. 미리보기는 iframe sandbox+CSP 또는 escaped Markdown을 사용한다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="88" customHeight="1">
+      <x:c r="A55" s="19" t="str">
+        <x:v>2026-10-02 AI 패널 hover header</x:v>
+      </x:c>
+      <x:c r="B55" s="19" t="str">
+        <x:v>기존 workbook 행 스타일을 복사해 관련 기능·관계·코드·요청·패치·안전 규칙을 추가하고 재열기·수식·문자·렌더 검사를 수행했다.</x:v>
+      </x:c>
+      <x:c r="C55" s="19" t="str">
+        <x:v>UI contract 121 sources, production/PDF.js build, live bundle SHA, HTTP/services, Chrome hover/leave/settings pinning, console errors</x:v>
+      </x:c>
+      <x:c r="D55" s="19" t="str">
+        <x:v>운영 배포·실화면 검증 완료</x:v>
+      </x:c>
+      <x:c r="E55" s="19" t="str">
+        <x:v>최상단 8px만 감지하고 settingsOpen 동안만 고정한다. 마우스 클릭 focus는 헤더 잔류 조건으로 사용하지 않는다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9293,6 +9350,20 @@
         <x:v>서버 allowlist 카탈로그, owner/revision/notebook 재검증, resource queue, Docker network none/non-root/read-only 경계와 sandbox+CSP 미리보기를 함께 유지한다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="161" ht="88" customHeight="1">
+      <x:c r="A161" s="19" t="str">
+        <x:v>DNB-AI-HOVER-HEADER-161</x:v>
+      </x:c>
+      <x:c r="B161" s="19" t="str">
+        <x:v>AI 패널 상단바 hover·포커스 경계</x:v>
+      </x:c>
+      <x:c r="C161" s="19" t="str">
+        <x:v>상단 감지 영역을 너무 넓히면 대화 스크롤과 첫 메시지를 가리고, 단순 focus-within을 쓰면 마우스로 설정을 닫은 뒤에도 헤더가 계속 남는다.</x:v>
+      </x:c>
+      <x:c r="D161" s="19" t="str">
+        <x:v>패널 최상단 8px만 hover 감지한다. 헤더 내부 hover와 키보드 focus-visible은 유지하고, 설정이 열린 동안만 data-pinned로 고정한다. 설정 종료 후 마우스 포커스만 남은 경우 즉시 숨긴다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11587,6 +11658,23 @@
         <x:v>NOTE-STUDIO-NOTEBOOK-DRILLDOWN, NOTE-STUDIO-GUIDED-TREES, WORKSPACE-RESUME-STATE</x:v>
       </x:c>
     </x:row>
+    <x:row r="135" ht="82" customHeight="1">
+      <x:c r="A135" s="19" t="str">
+        <x:v>AI-AGENT-COMPACT-HEADER</x:v>
+      </x:c>
+      <x:c r="B135" s="19" t="str">
+        <x:v>AI 패널 자동 숨김 상단바</x:v>
+      </x:c>
+      <x:c r="C135" s="19" t="str">
+        <x:v>완료·운영 배포·실화면 검증</x:v>
+      </x:c>
+      <x:c r="D135" s="19" t="str">
+        <x:v>평소에는 상단바가 편집 공간을 차지하지 않고, 패널 최상단 8px에 마우스를 올리면 52px 헤더가 overlay로 나타난다. 헤더를 벗어나면 숨고 설정 중에는 조작이 끝날 때까지 유지된다.</x:v>
+      </x:c>
+      <x:c r="E135" s="19" t="str">
+        <x:v>AI-AGENT, AI-AGENT-LIVE-PROGRESS, WEB-UI-DESIGN-SYSTEM, Code_Map, Do_Not_Break</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -14430,6 +14518,20 @@
         <x:v>전체 보기는 기본적으로 압축하되 사용자가 왼쪽 chevron을 누른 노트북만 하위 페이지를 인라인 표시한다. 노트북 행 선택은 기존 전용 보기로 진입한다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="203" ht="70" customHeight="1">
+      <x:c r="A203" s="19" t="str">
+        <x:v>AI-AGENT-COMPACT-HEADER</x:v>
+      </x:c>
+      <x:c r="B203" s="19" t="str">
+        <x:v>refines</x:v>
+      </x:c>
+      <x:c r="C203" s="19" t="str">
+        <x:v>AI-AGENT-LIVE-PROGRESS / WEB-UI-DESIGN-SYSTEM</x:v>
+      </x:c>
+      <x:c r="D203" s="19" t="str">
+        <x:v>숨긴 헤더는 진행도와 대화 영역의 세로 공간을 반환하되 8px reveal target, hover 유지, 키보드 focus-visible, 설정 중 pinning을 함께 보장한다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -21331,6 +21433,20 @@
       </x:c>
       <x:c r="D492" s="19" t="str">
         <x:v>chevron 클릭은 행 클릭으로 전파하지 않는다. 전체 검색 때문에 인라인 page tree 데이터가 잘리지 않게 한다. 터미널·모두 접기·사이드바 숨기기는 더보기에서 제공한다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="493" ht="70" customHeight="1">
+      <x:c r="A493" s="19" t="str">
+        <x:v>AI-AGENT-COMPACT-HEADER</x:v>
+      </x:c>
+      <x:c r="B493" s="19" t="str">
+        <x:v>frontend/src/components/AiAgentPanel.js; frontend/scripts/verify-ui-contract.mjs</x:v>
+      </x:c>
+      <x:c r="C493" s="19" t="str">
+        <x:v>8px reveal target, 52px overlay header, hover/focus-visible/settings pinning, UI contract gate</x:v>
+      </x:c>
+      <x:c r="D493" s="19" t="str">
+        <x:v>focus-within 전체 사용은 마우스 클릭 뒤 헤더 잔류를 만들므로 금지하고 키보드 focus-visible만 표시 조건에 포함한다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
feat: show per-response AI token cost
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R903dbbfd676c4990"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R6d5af90071b040d6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R12c7b385aa64432c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R5daa14f9a0454475"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="Rd57d53dbce3c42bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Rcd0b2064a5ab4dc7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Rea325d29a3124c6a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Rbc03739233504958"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R22c1fb89e1f54fe6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R109019d91860456d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Rb4513b07c98f4a99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R832533ecf36840cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R77689cf6c0464249"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="Rd4e2554fd18c4e32"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Ra6795521920e42b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R289681ae70194c06"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R761a6a1191bd4f2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="Rfbcf8cbe7afd4a61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Re8ac11d3c7634157"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R3eb7547601044be7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R4ecc892a4cb14715"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R62481ec5d2404230"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R24a9e5fe87344c43"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rd9f78eb9cce246a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Ra3a6b9dc8b2d4c08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R005c3abf1ead4c73"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R33f837502c0846f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R50152a7404ca469e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R5cea4229d68c4abb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R5ac9ee8ddfeb4d16"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4764,6 +4764,41 @@
       <x:c r="J115" s="19"/>
       <x:c r="K115" s="19"/>
     </x:row>
+    <x:row r="116">
+      <x:c r="A116" t="str">
+        <x:v>PATCH-AI-CHAT-COST-2026-10-02</x:v>
+      </x:c>
+      <x:c r="B116" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="C116" t="str">
+        <x:v>로컬 검증 완료 / 운영 배포 전</x:v>
+      </x:c>
+      <x:c r="D116" t="str">
+        <x:v>각 AI 대화의 맨 아래에 현재 모델 토큰 단가로 계산한 USD 비용을 1.32$처럼 두 자리로 작고 희미하게 표시해 달라는 요청.</x:v>
+      </x:c>
+      <x:c r="E116" t="str">
+        <x:v>기존 저장소는 날짜별 누적 토큰만 보존하고 assistant 메시지별 모델·입력·캐시 입력·출력 usage를 저장하지 않아 개별 답변 비용을 정확히 표시할 수 없었다.</x:v>
+      </x:c>
+      <x:c r="F116" t="str">
+        <x:v>일별 usage만으로 과거 대화 비용을 나누면 도구 반복 횟수와 캐시·출력 비율을 잃어 잘못된 금액이 된다. 단가가 바뀌면 과거 금액까지 변하는 문제도 있다.</x:v>
+      </x:c>
+      <x:c r="G116" t="str">
+        <x:v>공식 표준 gpt-4.1-mini 단가를 별도 서버 모듈에 두고 응답별 실제 usage에서 비캐시 입력·캐시 입력·출력을 구분해 계산한다. 모델·usage·단가·계산액을 assistant 메시지에 저장하고 말풍선 최하단 footer에 두 자리 USD로 표시한다.</x:v>
+      </x:c>
+      <x:c r="H116" t="str">
+        <x:v>단가 계산 3건, backend 전체 168건 중 160 pass·8 환경 skip·0 fail, UI contract 121개 소스, production build와 PDF.js 4.8.69 gate 통과.</x:v>
+      </x:c>
+      <x:c r="I116" t="str">
+        <x:v>새 답변부터 정확히 표시한다. 과거 메시지는 개별 usage가 없어 미표시한다. 토큰 가격 외 별도 유료 도구·세금·환율은 포함하지 않으며 알 수 없는 모델은 금액을 표시하지 않는다.</x:v>
+      </x:c>
+      <x:c r="J116" t="str">
+        <x:v>AI-CHAT-COST</x:v>
+      </x:c>
+      <x:c r="K116" t="str">
+        <x:v>backend/aiPricing.js; backend/aiAgentRoutes.js; frontend/src/components/AiAgentPanel.js; backend/tests/aiPricing.test.js; frontend/scripts/verify-ui-contract.mjs</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5906,6 +5941,17 @@
         <x:v>AI 에이전트 상단바가 너무 두꺼우므로 평소에는 숨기고 패널 상단에 마우스를 정확히 올렸을 때 나타나며, 벗어나면 사라지도록 동작 범위를 안전하게 설정해 달라는 요청.</x:v>
       </x:c>
     </x:row>
+    <x:row r="103">
+      <x:c r="A103" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="B103" t="str">
+        <x:v>AI 답변별 USD 토큰 비용 표시</x:v>
+      </x:c>
+      <x:c r="C103" t="str">
+        <x:v>토큰수도 각 대화에 현재 모델 토큰 가격을 계산해서 대화창 맨밑 조그만하게 몇 달러인지 소수점 두자리까지 1.32$ 이런식으로 표시하면 좋겠다 회색 희미한색으로</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6600,6 +6646,23 @@
       </x:c>
       <x:c r="E55" s="19" t="str">
         <x:v>최상단 8px만 감지하고 settingsOpen 동안만 고정한다. 마우스 클릭 focus는 헤더 잔류 조건으로 사용하지 않는다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" t="str">
+        <x:v>2026-10-02 AI 답변별 토큰 비용</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>모델별 표준 단가, 응답별 usage 스냅샷, assistant 말풍선 footer 두 자리 USD 표시와 unknown model 미표시를 기록했다.</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
+        <x:v>artifact-tool 기존 행 스타일 보존 편집·재열기·수식 오류·문자 깨짐·변경 범위 렌더; 단가 3건·backend 168건·UI contract·production/PDF.js</x:v>
+      </x:c>
+      <x:c r="D56" t="str">
+        <x:v>로컬 검증 통과 / 운영 배포 전</x:v>
+      </x:c>
+      <x:c r="E56" t="str">
+        <x:v>공식 OpenAI 표준 gpt-4.1-mini 단가 확인일 2026-10-02. 과거 메시지는 개별 usage 부재로 미표시하며 운영 화면 검증 후 같은 행을 갱신한다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9364,6 +9427,20 @@
         <x:v>패널 최상단 8px만 hover 감지한다. 헤더 내부 hover와 키보드 focus-visible은 유지하고, 설정이 열린 동안만 data-pinned로 고정한다. 설정 종료 후 마우스 포커스만 남은 경우 즉시 숨긴다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="162">
+      <x:c r="A162" t="str">
+        <x:v>DNB-AI-COST-ESTIMATE</x:v>
+      </x:c>
+      <x:c r="B162" t="str">
+        <x:v>AI 답변별 토큰 비용 표시</x:v>
+      </x:c>
+      <x:c r="C162" t="str">
+        <x:v>현재 단가로 과거 메시지 비용을 다시 계산하거나, 지원하지 않는 모델에 임의 단가를 적용하거나, 토큰 추정액을 OpenAI 청구서 전체 금액으로 표시하지 말 것.</x:v>
+      </x:c>
+      <x:c r="D162" t="str">
+        <x:v>응답 생성 시점의 모델·입력·캐시 입력·출력 토큰과 공식 표준 단가 스냅샷을 assistant 메시지에 저장한다. 알 수 없는 모델은 금액을 숨기고 공식 단가를 확인해 카탈로그를 갱신한다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11675,6 +11752,23 @@
         <x:v>AI-AGENT, AI-AGENT-LIVE-PROGRESS, WEB-UI-DESIGN-SYSTEM, Code_Map, Do_Not_Break</x:v>
       </x:c>
     </x:row>
+    <x:row r="136">
+      <x:c r="A136" t="str">
+        <x:v>AI-CHAT-COST</x:v>
+      </x:c>
+      <x:c r="B136" t="str">
+        <x:v>AI 답변별 USD 토큰 비용 표시</x:v>
+      </x:c>
+      <x:c r="C136" t="str">
+        <x:v>로컬 구현·회귀 완료 / 운영 배포 전</x:v>
+      </x:c>
+      <x:c r="D136" t="str">
+        <x:v>새 AI 답변마다 사용 모델과 실제 Responses usage의 비캐시 입력·캐시 입력·출력 토큰을 계산 당시 표준 단가로 합산해 메시지 하단에 소수점 둘째 자리 USD로 표시한다. 과거 메시지는 개별 usage가 없어 금액을 꾸며내지 않는다.</x:v>
+      </x:c>
+      <x:c r="E136" t="str">
+        <x:v>AI-AGENT, AI-AGENT-SINGLE-CHAT, AI-TOKEN-BUDGET, WEB-UI-DESIGN-SYSTEM, Code_Map, Do_Not_Break, Patch_Log</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -14532,6 +14626,20 @@
         <x:v>숨긴 헤더는 진행도와 대화 영역의 세로 공간을 반환하되 8px reveal target, hover 유지, 키보드 focus-visible, 설정 중 pinning을 함께 보장한다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="204">
+      <x:c r="A204" t="str">
+        <x:v>AI-CHAT-COST</x:v>
+      </x:c>
+      <x:c r="B204" t="str">
+        <x:v>calculates_from_and_persists_with</x:v>
+      </x:c>
+      <x:c r="C204" t="str">
+        <x:v>AI-AGENT / OpenAI Responses usage / AI message history</x:v>
+      </x:c>
+      <x:c r="D204" t="str">
+        <x:v>assistant 답변 생성 때 모델별 표준 입력·캐시 입력·출력 단가로 계산한 스냅샷을 메시지에 함께 저장해야 모델 변경이나 단가 갱신 뒤에도 과거 표시가 바뀌지 않는다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -21447,6 +21555,76 @@
       </x:c>
       <x:c r="D493" s="19" t="str">
         <x:v>focus-within 전체 사용은 마우스 클릭 뒤 헤더 잔류를 만들므로 금지하고 키보드 focus-visible만 표시 조건에 포함한다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="494">
+      <x:c r="A494" t="str">
+        <x:v>AI-CHAT-COST</x:v>
+      </x:c>
+      <x:c r="B494" t="str">
+        <x:v>backend/aiPricing.js</x:v>
+      </x:c>
+      <x:c r="C494" t="str">
+        <x:v>지원 모델의 공식 표준 단가와 비캐시·캐시 입력·출력 토큰 비용 계산. 모르는 모델은 null로 fail-closed.</x:v>
+      </x:c>
+      <x:c r="D494" t="str">
+        <x:v>gpt-4.1-mini 표준 단가 스냅샷과 날짜 고정 별칭</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="495">
+      <x:c r="A495" t="str">
+        <x:v>AI-CHAT-COST</x:v>
+      </x:c>
+      <x:c r="B495" t="str">
+        <x:v>backend/aiAgentRoutes.js</x:v>
+      </x:c>
+      <x:c r="C495" t="str">
+        <x:v>일반·승인 대기·승인 후 재개 assistant 메시지에 계산 당시 billing 메타데이터 저장.</x:v>
+      </x:c>
+      <x:c r="D495" t="str">
+        <x:v>기존 일별 usage 원장과 별개인 답변 단위 기록</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="496">
+      <x:c r="A496" t="str">
+        <x:v>AI-CHAT-COST</x:v>
+      </x:c>
+      <x:c r="B496" t="str">
+        <x:v>frontend/src/components/AiAgentPanel.js</x:v>
+      </x:c>
+      <x:c r="C496" t="str">
+        <x:v>AI 말풍선 하단에 희미한 회색의 소수점 둘째 자리 USD 비용 표시와 모델·토큰 tooltip 제공.</x:v>
+      </x:c>
+      <x:c r="D496" t="str">
+        <x:v>사용자 메시지와 과거 usage 없는 메시지는 미표시</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="497">
+      <x:c r="A497" t="str">
+        <x:v>AI-CHAT-COST</x:v>
+      </x:c>
+      <x:c r="B497" t="str">
+        <x:v>backend/tests/aiPricing.test.js</x:v>
+      </x:c>
+      <x:c r="C497" t="str">
+        <x:v>표준 단가·캐시 차감·날짜 별칭·unknown model fail-closed 회귀.</x:v>
+      </x:c>
+      <x:c r="D497" t="str">
+        <x:v>유료 API 호출 없음</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="498">
+      <x:c r="A498" t="str">
+        <x:v>AI-CHAT-COST</x:v>
+      </x:c>
+      <x:c r="B498" t="str">
+        <x:v>frontend/scripts/verify-ui-contract.mjs</x:v>
+      </x:c>
+      <x:c r="C498" t="str">
+        <x:v>답변별 billing 표시와 두 자리 USD 형식이 UI에서 제거되지 않도록 정적 계약 검사.</x:v>
+      </x:c>
+      <x:c r="D498" t="str">
+        <x:v>기존 121개 소스 검사에 포함</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record AI cost deployment verification
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R289681ae70194c06"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R761a6a1191bd4f2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="Rfbcf8cbe7afd4a61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Re8ac11d3c7634157"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R3eb7547601044be7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R4ecc892a4cb14715"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R62481ec5d2404230"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R24a9e5fe87344c43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rd9f78eb9cce246a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Ra3a6b9dc8b2d4c08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R005c3abf1ead4c73"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R33f837502c0846f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R50152a7404ca469e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R5cea4229d68c4abb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R5ac9ee8ddfeb4d16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R51f5a0388a564c7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Rc06cbf88d9654b79"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="Rfe5eeadc3fca4d83"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R31fb1c11a51a4bcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R605b8b6909f946b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Raf7e7e9108994a07"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Rc30b08cc0dc6480d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R913b3f9afae944e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R3e2f2c81eea84189"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R0f8a28ccf7814070"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R1c5f7835e944440e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R423cf155da954899"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="Re3e7d4e823464a9c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R55057811ec644056"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Rd4ad46febb274c94"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4772,7 +4772,7 @@
         <x:v>2026-10-02</x:v>
       </x:c>
       <x:c r="C116" t="str">
-        <x:v>로컬 검증 완료 / 운영 배포 전</x:v>
+        <x:v>완료 · 운영 배포 · 실화면 검증</x:v>
       </x:c>
       <x:c r="D116" t="str">
         <x:v>각 AI 대화의 맨 아래에 현재 모델 토큰 단가로 계산한 USD 비용을 1.32$처럼 두 자리로 작고 희미하게 표시해 달라는 요청.</x:v>
@@ -4787,7 +4787,7 @@
         <x:v>공식 표준 gpt-4.1-mini 단가를 별도 서버 모듈에 두고 응답별 실제 usage에서 비캐시 입력·캐시 입력·출력을 구분해 계산한다. 모델·usage·단가·계산액을 assistant 메시지에 저장하고 말풍선 최하단 footer에 두 자리 USD로 표시한다.</x:v>
       </x:c>
       <x:c r="H116" t="str">
-        <x:v>단가 계산 3건, backend 전체 168건 중 160 pass·8 환경 skip·0 fail, UI contract 121개 소스, production build와 PDF.js 4.8.69 gate 통과.</x:v>
+        <x:v>단가 계산 3건, backend 전체 168건 중 160 pass·8 환경 skip·0 fail, UI contract 121개 소스, production build/PDF.js gate, NAS Linux 계산 3/3, 필수 서비스 6개 active, 내부·공개·새 bundle HTTP 200. 실제 gpt-4.1-mini 답변은 입력 1,696·출력 4토큰으로 0.00$가 표시되고 새로고침 후 유지, 브라우저 오류 0건.</x:v>
       </x:c>
       <x:c r="I116" t="str">
         <x:v>새 답변부터 정확히 표시한다. 과거 메시지는 개별 usage가 없어 미표시한다. 토큰 가격 외 별도 유료 도구·세금·환율은 포함하지 않으며 알 수 없는 모델은 금액을 표시하지 않는다.</x:v>
@@ -6659,10 +6659,10 @@
         <x:v>artifact-tool 기존 행 스타일 보존 편집·재열기·수식 오류·문자 깨짐·변경 범위 렌더; 단가 3건·backend 168건·UI contract·production/PDF.js</x:v>
       </x:c>
       <x:c r="D56" t="str">
-        <x:v>로컬 검증 통과 / 운영 배포 전</x:v>
+        <x:v>완료 · 운영 배포 · 실화면 검증</x:v>
       </x:c>
       <x:c r="E56" t="str">
-        <x:v>공식 OpenAI 표준 gpt-4.1-mini 단가 확인일 2026-10-02. 과거 메시지는 개별 usage 부재로 미표시하며 운영 화면 검증 후 같은 행을 갱신한다.</x:v>
+        <x:v>운영 bundle main.050cdd80.js SHA-256 일치. 실제 새 답변 0.00$ 표시와 입력·캐시 입력·출력 tooltip, 재로딩 후 지속, 브라우저 오류 0건 확인. 과거 메시지는 개별 usage 부재로 미표시한다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11760,7 +11760,7 @@
         <x:v>AI 답변별 USD 토큰 비용 표시</x:v>
       </x:c>
       <x:c r="C136" t="str">
-        <x:v>로컬 구현·회귀 완료 / 운영 배포 전</x:v>
+        <x:v>완료 · 운영 배포 · 실화면 검증</x:v>
       </x:c>
       <x:c r="D136" t="str">
         <x:v>새 AI 답변마다 사용 모델과 실제 Responses usage의 비캐시 입력·캐시 입력·출력 토큰을 계산 당시 표준 단가로 합산해 메시지 하단에 소수점 둘째 자리 USD로 표시한다. 과거 메시지는 개별 usage가 없어 금액을 꾸며내지 않는다.</x:v>

</xml_diff>

<commit_message>
fix: show AI response cost to four decimals
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R51f5a0388a564c7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Rc06cbf88d9654b79"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="Rfe5eeadc3fca4d83"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R31fb1c11a51a4bcc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R605b8b6909f946b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Raf7e7e9108994a07"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Rc30b08cc0dc6480d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R913b3f9afae944e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R3e2f2c81eea84189"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R0f8a28ccf7814070"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R1c5f7835e944440e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R423cf155da954899"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="Re3e7d4e823464a9c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R55057811ec644056"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Rd4ad46febb274c94"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc054a7e7e1bd4b7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Rc218d74a14514c23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R1be3de12f09d422f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R5df2d05083bd40d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R2ab4790b1f2944f9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R00df2a6ba65649bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R6b91a55b7f4a4cff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R04590ccf77b74af8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rb5f41e5124514766"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R72eb588fb9ae46f0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Rfe3c6c28dc13427e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R6afc43dc45894a3b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="Rfc2791bbc5a2415b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R777ca8e30e684db0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Rd6d035c21fef4e8c"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4799,6 +4799,41 @@
         <x:v>backend/aiPricing.js; backend/aiAgentRoutes.js; frontend/src/components/AiAgentPanel.js; backend/tests/aiPricing.test.js; frontend/scripts/verify-ui-contract.mjs</x:v>
       </x:c>
     </x:row>
+    <x:row r="117">
+      <x:c r="A117" t="str">
+        <x:v>PATCH-AI-CHAT-COST-4DP-2026-10-02</x:v>
+      </x:c>
+      <x:c r="B117" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="C117" t="str">
+        <x:v>로컬 검증 완료 / 운영 배포 전</x:v>
+      </x:c>
+      <x:c r="D117" t="str">
+        <x:v>AI 응답별 USD 비용 표시를 소수점 둘째 자리에서 넷째 자리로 늘려 달라는 요청.</x:v>
+      </x:c>
+      <x:c r="E117" t="str">
+        <x:v>짧은 응답은 실제 비용이 0.01달러보다 작아 모두 0.00$로 보였고 응답 간 차이를 확인할 수 없었다.</x:v>
+      </x:c>
+      <x:c r="F117" t="str">
+        <x:v>계산값과 저장된 billing 스냅샷은 정확했지만 UI의 toFixed(2)가 표시 정밀도만 제한했다.</x:v>
+      </x:c>
+      <x:c r="G117" t="str">
+        <x:v>말풍선 본문과 접근성 설명을 toFixed(4)로 바꾸고 UI 계약 검사도 네 자리 형식을 요구하도록 갱신했다.</x:v>
+      </x:c>
+      <x:c r="H117" t="str">
+        <x:v>UI contract 121개 소스 및 production build, react-pdf 9.2.1/PDF.js API+Worker 4.8.69 gate 통과.</x:v>
+      </x:c>
+      <x:c r="I117" t="str">
+        <x:v>계산 로직·공식 단가·과거 billing 데이터는 변경하지 않는다. 0.00005달러 미만은 0.0000$로 반올림될 수 있다.</x:v>
+      </x:c>
+      <x:c r="J117" t="str">
+        <x:v>AI-CHAT-COST</x:v>
+      </x:c>
+      <x:c r="K117" t="str">
+        <x:v>frontend/src/components/AiAgentPanel.js; frontend/scripts/verify-ui-contract.mjs</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5952,6 +5987,17 @@
         <x:v>토큰수도 각 대화에 현재 모델 토큰 가격을 계산해서 대화창 맨밑 조그만하게 몇 달러인지 소수점 두자리까지 1.32$ 이런식으로 표시하면 좋겠다 회색 희미한색으로</x:v>
       </x:c>
     </x:row>
+    <x:row r="104">
+      <x:c r="A104" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="B104" t="str">
+        <x:v>AI 응답별 비용 소수점 네 자리 표시</x:v>
+      </x:c>
+      <x:c r="C104" t="str">
+        <x:v>아 쏘리 소수점 4자리까지 표기좀</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6663,6 +6709,23 @@
       </x:c>
       <x:c r="E56" t="str">
         <x:v>운영 bundle main.050cdd80.js SHA-256 일치. 실제 새 답변 0.00$ 표시와 입력·캐시 입력·출력 tooltip, 재로딩 후 지속, 브라우저 오류 0건 확인. 과거 메시지는 개별 usage 부재로 미표시한다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" t="str">
+        <x:v>2026-10-02 AI 비용 표시 소수점 네 자리</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>응답별 USD 표시를 0.0000$ 형식으로 바꾸고 접근성 설명과 UI 회귀 계약을 같은 정밀도로 맞췄다.</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
+        <x:v>artifact-tool 기존 행 스타일 보존 편집·재열기·수식 오류·문자 깨짐·변경 범위 렌더; UI contract 121개 소스·production/PDF.js</x:v>
+      </x:c>
+      <x:c r="D57" t="str">
+        <x:v>로컬 검증 통과 / 운영 배포 전</x:v>
+      </x:c>
+      <x:c r="E57" t="str">
+        <x:v>계산과 저장 방식은 그대로이며 UI 표시 정밀도만 두 자리에서 네 자리로 변경한다. 운영 화면 검증 후 같은 행을 갱신한다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9438,7 +9501,7 @@
         <x:v>현재 단가로 과거 메시지 비용을 다시 계산하거나, 지원하지 않는 모델에 임의 단가를 적용하거나, 토큰 추정액을 OpenAI 청구서 전체 금액으로 표시하지 말 것.</x:v>
       </x:c>
       <x:c r="D162" t="str">
-        <x:v>응답 생성 시점의 모델·입력·캐시 입력·출력 토큰과 공식 표준 단가 스냅샷을 assistant 메시지에 저장한다. 알 수 없는 모델은 금액을 숨기고 공식 단가를 확인해 카탈로그를 갱신한다.</x:v>
+        <x:v>응답 생성 시점의 모델·입력·캐시 입력·출력 토큰과 공식 표준 단가 스냅샷을 assistant 메시지에 저장한다. UI 비용은 소수점 네 자리 USD로 표시한다. 알 수 없는 모델은 금액을 숨기고 공식 단가를 확인해 카탈로그를 갱신한다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -11763,7 +11826,7 @@
         <x:v>완료 · 운영 배포 · 실화면 검증</x:v>
       </x:c>
       <x:c r="D136" t="str">
-        <x:v>새 AI 답변마다 사용 모델과 실제 Responses usage의 비캐시 입력·캐시 입력·출력 토큰을 계산 당시 표준 단가로 합산해 메시지 하단에 소수점 둘째 자리 USD로 표시한다. 과거 메시지는 개별 usage가 없어 금액을 꾸며내지 않는다.</x:v>
+        <x:v>새 AI 답변마다 사용 모델과 실제 Responses usage의 비캐시 입력·캐시 입력·출력 토큰을 계산 당시 표준 단가로 합산해 메시지 하단에 소수점 넷째 자리 USD로 표시한다. 과거 메시지는 개별 usage가 없어 금액을 꾸며내지 않는다.</x:v>
       </x:c>
       <x:c r="E136" t="str">
         <x:v>AI-AGENT, AI-AGENT-SINGLE-CHAT, AI-TOKEN-BUDGET, WEB-UI-DESIGN-SYSTEM, Code_Map, Do_Not_Break, Patch_Log</x:v>
@@ -14637,7 +14700,7 @@
         <x:v>AI-AGENT / OpenAI Responses usage / AI message history</x:v>
       </x:c>
       <x:c r="D204" t="str">
-        <x:v>assistant 답변 생성 때 모델별 표준 입력·캐시 입력·출력 단가로 계산한 스냅샷을 메시지에 함께 저장해야 모델 변경이나 단가 갱신 뒤에도 과거 표시가 바뀌지 않는다.</x:v>
+        <x:v>assistant 답변 생성 때 모델별 표준 입력·캐시 입력·출력 단가로 계산한 스냅샷을 메시지에 함께 저장해야 모델 변경이나 단가 갱신 뒤에도 과거 표시가 바뀌지 않는다. 표시는 소수점 네 자리 USD를 유지한다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -21593,7 +21656,7 @@
         <x:v>frontend/src/components/AiAgentPanel.js</x:v>
       </x:c>
       <x:c r="C496" t="str">
-        <x:v>AI 말풍선 하단에 희미한 회색의 소수점 둘째 자리 USD 비용 표시와 모델·토큰 tooltip 제공.</x:v>
+        <x:v>AI 말풍선 하단에 희미한 회색의 소수점 넷째 자리 USD 비용 표시와 모델·토큰 tooltip 제공.</x:v>
       </x:c>
       <x:c r="D496" t="str">
         <x:v>사용자 메시지와 과거 usage 없는 메시지는 미표시</x:v>

</xml_diff>

<commit_message>
docs: record four-decimal cost verification
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc054a7e7e1bd4b7d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Rc218d74a14514c23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R1be3de12f09d422f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R5df2d05083bd40d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R2ab4790b1f2944f9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R00df2a6ba65649bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R6b91a55b7f4a4cff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R04590ccf77b74af8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rb5f41e5124514766"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R72eb588fb9ae46f0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Rfe3c6c28dc13427e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R6afc43dc45894a3b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="Rfc2791bbc5a2415b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R777ca8e30e684db0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Rd6d035c21fef4e8c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R8d285f98f0ac4f4e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R336b6798028f4a65"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R79fe2f9548f74d3d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R0a27fbbcdaa84ad5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R441a30a842664de3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R58c0bf7ff0e349ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R7b1836fd4d2e4b48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R481273aac88a458e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R5f17adff728c4c6d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rcecba8ec8f4941fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Rbbc43e1b40e349d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="Rb52e0228fdcc4979"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R20d4e61e1a294ab8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R4324253352364edc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Rc2daeb20de8649c0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4807,7 +4807,7 @@
         <x:v>2026-10-02</x:v>
       </x:c>
       <x:c r="C117" t="str">
-        <x:v>로컬 검증 완료 / 운영 배포 전</x:v>
+        <x:v>완료 · 운영 배포 · 실화면 검증</x:v>
       </x:c>
       <x:c r="D117" t="str">
         <x:v>AI 응답별 USD 비용 표시를 소수점 둘째 자리에서 넷째 자리로 늘려 달라는 요청.</x:v>
@@ -4822,7 +4822,7 @@
         <x:v>말풍선 본문과 접근성 설명을 toFixed(4)로 바꾸고 UI 계약 검사도 네 자리 형식을 요구하도록 갱신했다.</x:v>
       </x:c>
       <x:c r="H117" t="str">
-        <x:v>UI contract 121개 소스 및 production build, react-pdf 9.2.1/PDF.js API+Worker 4.8.69 gate 통과.</x:v>
+        <x:v>UI contract 121개 소스, production build, react-pdf 9.2.1/PDF.js API+Worker 4.8.69 gate 통과. 운영 bundle main.a90a9809.js 배포 후 기존 저장 응답이 0.0007$·0.0006$·0.0009$로 네 자리 표시되고 모델·입력·캐시 입력·출력 토큰 tooltip과 희미한 회색 스타일을 유지함. 추가 유료 API 호출 없이 재로딩 검증했으며 브라우저 오류 0건.</x:v>
       </x:c>
       <x:c r="I117" t="str">
         <x:v>계산 로직·공식 단가·과거 billing 데이터는 변경하지 않는다. 0.00005달러 미만은 0.0000$로 반올림될 수 있다.</x:v>
@@ -6722,10 +6722,10 @@
         <x:v>artifact-tool 기존 행 스타일 보존 편집·재열기·수식 오류·문자 깨짐·변경 범위 렌더; UI contract 121개 소스·production/PDF.js</x:v>
       </x:c>
       <x:c r="D57" t="str">
-        <x:v>로컬 검증 통과 / 운영 배포 전</x:v>
+        <x:v>완료 · 운영 배포 · 실화면 검증</x:v>
       </x:c>
       <x:c r="E57" t="str">
-        <x:v>계산과 저장 방식은 그대로이며 UI 표시 정밀도만 두 자리에서 네 자리로 변경한다. 운영 화면 검증 후 같은 행을 갱신한다.</x:v>
+        <x:v>운영 bundle main.a90a9809.js에서 기존 gpt-4.1-mini 응답의 0.0007$ 표시, 접근성 설명 0.0007달러, 토큰 상세 tooltip, 회색 보조 스타일, 브라우저 오류 0건을 확인했다. 계산·저장·단가는 변경하지 않았다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Record AI trash restore deployment verification
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R8d285f98f0ac4f4e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R336b6798028f4a65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R79fe2f9548f74d3d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R0a27fbbcdaa84ad5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R441a30a842664de3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R58c0bf7ff0e349ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R7b1836fd4d2e4b48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R481273aac88a458e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R5f17adff728c4c6d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rcecba8ec8f4941fb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Rbbc43e1b40e349d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="Rb52e0228fdcc4979"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R20d4e61e1a294ab8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R4324253352364edc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Rc2daeb20de8649c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R848154757b98486e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R2314b8005cfd4428"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R7b7daf2f014f4f8b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R0363472f6d554c5b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="Rbd0bb74131dd4556"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R0b20d04edccd43ed"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R79c819bac6a0429d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Re059fe549efc4a05"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rf093ef1420ae47db"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R5a98af0d4ed24dba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R40c495b2a1e743a1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="Rf8730a9ed9ff4af2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R16344e2049654edc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="Rd27ac259a2e34543"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Rb6f8f766f4da49b0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4834,6 +4834,39 @@
         <x:v>frontend/src/components/AiAgentPanel.js; frontend/scripts/verify-ui-contract.mjs</x:v>
       </x:c>
     </x:row>
+    <x:row r="118" ht="164" customHeight="1">
+      <x:c r="A118" s="19" t="str">
+        <x:v>PATCH-AI-TRASH-RESTORE-2026-10-02</x:v>
+      </x:c>
+      <x:c r="B118" s="19" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="C118" s="19" t="str">
+        <x:v>완료 · 운영 배포 · 실제 계정 E2E 검증</x:v>
+      </x:c>
+      <x:c r="D118" s="19" t="str">
+        <x:v>AI가 삭제 파일 1~4번을 복구하겠다고 답했지만 실제 파일 복구와 action 기록이 없었던 문제를 해결해 달라는 요청.</x:v>
+      </x:c>
+      <x:c r="E118" s="19" t="str">
+        <x:v>기존 선택 카드의 번호 선택은 후속 채팅 텍스트만 만들었고, 선택 목록을 만든 assistant message와 실제 휴지통 항목이 실행 계층에 결속되지 않았다. 따라서 모델이 복구 의사를 말해도 restore API와 actions.json이 호출되지 않았다.</x:v>
+      </x:c>
+      <x:c r="F118" s="19" t="str">
+        <x:v>서버가 선택 목록 messageId·sourceTool과 선택 key를 받아 저장 메시지를 조회하고 최신 list_trash와 이름·원래 경로·삭제 시각을 재검증하도록 했다. 실제 trashId로 restore_trash_items action을 생성하고 승인 모드에 따라 durable runtime에서 복구한다. 실행 전 재검증, 항목별 completed/failed, idempotency, 허위 진행·완료 문구 차단을 추가했다.</x:v>
+      </x:c>
+      <x:c r="G118" s="19" t="str">
+        <x:v>로컬 focused 29/29, 전체 175건 중 167 pass·환경 8 skip·0 fail, UI contract 121 sources, production/PDF.js build 통과. NAS focused 29/29, 운영 main.225af495.js SHA-256 43D106620BBFBA82A58144128987C1ACFA67B13E323D92F62F9DC634A7E92871 일치, 필수 서비스 active, 내부·공개 HTTP 200. Chrome 실제 계정에서 테스트 파일을 목록 1번으로 선택해 승인·실행했고 원위치 파일, 휴지통 payload 제거, actions.json completed/restoredCount 1/failedCount 0을 교차 확인했다.</x:v>
+      </x:c>
+      <x:c r="H118" s="19" t="str">
+        <x:v>기존 사용자 휴지통의 CMOE 설치 파일 네 개는 선택·복구하지 않고 보존했다. 검증용 파일만 성공 확인 뒤 원위치에서 정리했으며 action 감사 기록은 남겼다.</x:v>
+      </x:c>
+      <x:c r="I118" s="19"/>
+      <x:c r="J118" s="19" t="str">
+        <x:v>AI-AGENT-TRASH-RESTORE</x:v>
+      </x:c>
+      <x:c r="K118" s="19" t="str">
+        <x:v>backend/aiSelectionExecution.js; backend/aiAgentRoutes.js; backend/aiAgentRuntime.js; frontend/src/components/AiAgentPanel.js</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5998,6 +6031,17 @@
         <x:v>아 쏘리 소수점 4자리까지 표기좀</x:v>
       </x:c>
     </x:row>
+    <x:row r="105" ht="78" customHeight="1">
+      <x:c r="A105" s="19" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="B105" s="19" t="str">
+        <x:v>AI 휴지통 선택 복구 실제 실행 누락 해결</x:v>
+      </x:c>
+      <x:c r="C105" s="19" t="str">
+        <x:v>AI가 1~4번 파일 복구를 진행한다고 답했지만 실제 복구와 actions.json 기록이 없었던 문제를 고치고, 실제 선택·승인·복구·서버 파일 검증까지 완료해 달라는 요청.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6726,6 +6770,23 @@
       </x:c>
       <x:c r="E57" t="str">
         <x:v>운영 bundle main.a90a9809.js에서 기존 gpt-4.1-mini 응답의 0.0007$ 표시, 접근성 설명 0.0007달러, 토큰 상세 tooltip, 회색 보조 스타일, 브라우저 오류 0건을 확인했다. 계산·저장·단가는 변경하지 않았다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="104" customHeight="1">
+      <x:c r="A58" s="19" t="str">
+        <x:v>2026-10-02 AI 휴지통 실제 복구</x:v>
+      </x:c>
+      <x:c r="B58" s="19" t="str">
+        <x:v>선택 목록 messageId와 최신 휴지통을 서버에서 재결속해 restore_trash_items action을 만들고 승인·실행·감사 결과를 실제 완료 문구와 연결했다.</x:v>
+      </x:c>
+      <x:c r="C58" s="19" t="str">
+        <x:v>focused 29/29, backend 167 pass·8 env skip·0 fail, UI contract 121 sources, production/PDF.js, NAS 회귀, bundle SHA, HTTP/services, Chrome 실제 계정 E2E, 원위치 파일·trash 제거·actions.json 대조</x:v>
+      </x:c>
+      <x:c r="D58" s="19" t="str">
+        <x:v>완료 · 운영 배포 · 실제 계정 E2E 검증</x:v>
+      </x:c>
+      <x:c r="E58" s="19" t="str">
+        <x:v>테스트 파일 1개만 복구하고 기존 네 휴지통 파일은 보존했다. 검증용 파일은 결과 확인 뒤 원위치에서 정리했으며 감사 기록은 유지했다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9504,6 +9565,20 @@
         <x:v>응답 생성 시점의 모델·입력·캐시 입력·출력 토큰과 공식 표준 단가 스냅샷을 assistant 메시지에 저장한다. UI 비용은 소수점 네 자리 USD로 표시한다. 알 수 없는 모델은 금액을 숨기고 공식 단가를 확인해 카탈로그를 갱신한다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="163" ht="116" customHeight="1">
+      <x:c r="A163" s="19" t="str">
+        <x:v>DNB-AI-TRASH-SELECTION-2026-10-02</x:v>
+      </x:c>
+      <x:c r="B163" s="19" t="str">
+        <x:v>AI 휴지통 선택 목록과 실제 복구 결속</x:v>
+      </x:c>
+      <x:c r="C163" s="19" t="str">
+        <x:v>AI가 번호 선택 응답만 생성하고 실제 restore 도구를 호출하지 않았는데 복구를 진행 또는 완료했다고 말하게 두지 말 것. 화면의 번호·이름을 클라이언트가 보낸 경로나 trashId로 신뢰하거나, 승인 후 달라진 휴지통 항목을 복구하지 말 것.</x:v>
+      </x:c>
+      <x:c r="D163" s="19" t="str">
+        <x:v>서버가 저장된 assistant messageId와 sourceTool=list_trash를 기준으로 선택 목록을 다시 읽고 최신 휴지통의 trashId·이름·원래 경로·삭제 시각과 일치시킨다. restore_trash_items action을 생성해 승인 모드에 따라 실행하고, 실행 직전 재검증·항목별 결과·idempotency·actions.json 감사를 남긴 뒤 실제 결과만 완료 문구로 표시한다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11832,6 +11907,23 @@
         <x:v>AI-AGENT, AI-AGENT-SINGLE-CHAT, AI-TOKEN-BUDGET, WEB-UI-DESIGN-SYSTEM, Code_Map, Do_Not_Break, Patch_Log</x:v>
       </x:c>
     </x:row>
+    <x:row r="137" ht="92" customHeight="1">
+      <x:c r="A137" s="19" t="str">
+        <x:v>AI-AGENT-TRASH-RESTORE</x:v>
+      </x:c>
+      <x:c r="B137" s="19" t="str">
+        <x:v>AI 선택 목록 기반 휴지통 실제 복구</x:v>
+      </x:c>
+      <x:c r="C137" s="19" t="str">
+        <x:v>완료 · 운영 배포 · 실제 계정 E2E 검증</x:v>
+      </x:c>
+      <x:c r="D137" s="19" t="str">
+        <x:v>AI가 휴지통 목록을 번호 카드로 제시하고 사용자가 한 개 또는 여러 개를 고르면 서버가 원본 메시지와 최신 휴지통을 대조해 복구 action을 만든다. ask_each는 승인 카드 뒤 실제 복구하며 auto_reversible은 같은 검증 경로에서 즉시 실행한다. 부분 실패는 항목별로 남고 허위 완료 응답은 차단된다.</x:v>
+      </x:c>
+      <x:c r="E137" s="19" t="str">
+        <x:v>AI-AGENT, AI-AGENT-DURABLE-RUN, FILE-TRASH, AI-SELECTION-FRAME, Code_Map, Do_Not_Break, Patch_Log</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -14703,6 +14795,20 @@
         <x:v>assistant 답변 생성 때 모델별 표준 입력·캐시 입력·출력 단가로 계산한 스냅샷을 메시지에 함께 저장해야 모델 변경이나 단가 갱신 뒤에도 과거 표시가 바뀌지 않는다. 표시는 소수점 네 자리 USD를 유지한다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="205" ht="78" customHeight="1">
+      <x:c r="A205" s="19" t="str">
+        <x:v>AI-AGENT-TRASH-RESTORE</x:v>
+      </x:c>
+      <x:c r="B205" s="19" t="str">
+        <x:v>binds_and_executes_through</x:v>
+      </x:c>
+      <x:c r="C205" s="19" t="str">
+        <x:v>AI-SELECTION-FRAME / FILE-TRASH / AI-AGENT-DURABLE-RUN</x:v>
+      </x:c>
+      <x:c r="D205" s="19" t="str">
+        <x:v>선택 번호는 저장된 목록 messageId에 결속하고 서버의 최신 list_trash 결과로 실제 trashId를 재해석한다. 승인·자동 실행 모두 restore_trash_items runtime과 actions.json 결과 원장을 거쳐야 하며 오래되거나 바뀐 목록은 실패 폐쇄한다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -21688,6 +21794,20 @@
       </x:c>
       <x:c r="D498" t="str">
         <x:v>기존 121개 소스 검사에 포함</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="499" ht="92" customHeight="1">
+      <x:c r="A499" s="19" t="str">
+        <x:v>AI-AGENT-TRASH-RESTORE</x:v>
+      </x:c>
+      <x:c r="B499" s="19" t="str">
+        <x:v>backend/aiSelectionExecution.js; backend/aiSelectionFrame.js; backend/aiAgentRoutes.js; backend/aiAgentRuntime.js; backend/aiAgentStore.js; backend/aiResponsePolicy.js; frontend/src/components/AiAgentPanel.js</x:v>
+      </x:c>
+      <x:c r="C499" s="19" t="str">
+        <x:v>선택 목록 메시지 식별, sourceTool 화이트리스트, 최신 휴지통 재결속, batch restore action 생성·승인·실행, 항목별 결과와 idempotency, 허위 복구 문구 차단, 복구 준비 UI</x:v>
+      </x:c>
+      <x:c r="D499" s="19" t="str">
+        <x:v>클라이언트에서 보낸 trashId나 경로는 실행 권한 자료로 쓰지 않고 서버 저장 메시지와 현재 휴지통을 모두 대조한다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Separate AI list queries from selection actions
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R848154757b98486e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R2314b8005cfd4428"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R7b7daf2f014f4f8b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R0363472f6d554c5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="Rbd0bb74131dd4556"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R0b20d04edccd43ed"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R79c819bac6a0429d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Re059fe549efc4a05"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rf093ef1420ae47db"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R5a98af0d4ed24dba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R40c495b2a1e743a1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="Rf8730a9ed9ff4af2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R16344e2049654edc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="Rd27ac259a2e34543"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Rb6f8f766f4da49b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R2fc64a18d5ca4b89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Rf55fb6f671d24765"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="Rc5a6995047084cbc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R94974dd6a0d24f1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R7aa18f581b3e4f0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R05a44ec26c884bb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R51508f7d00714cdc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R76e429a81e254fff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rcfbdad3071af4ac4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rf9a8f3bc67e04f5c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R55d482b84fb942d7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R8fb05a5e57e149d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="Raf8c5cfd48fb4bb4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="Rfb79feca60fd4c5e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Rcde7712218bb49e8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4867,6 +4867,39 @@
         <x:v>backend/aiSelectionExecution.js; backend/aiAgentRoutes.js; backend/aiAgentRuntime.js; frontend/src/components/AiAgentPanel.js</x:v>
       </x:c>
     </x:row>
+    <x:row r="119" ht="154" customHeight="1">
+      <x:c r="A119" s="19" t="str">
+        <x:v>PATCH-AI-LIST-SELECTION-INTENT-2026-10-02</x:v>
+      </x:c>
+      <x:c r="B119" s="19" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="C119" s="19" t="str">
+        <x:v>구현·자동 검증 완료 / 운영 검증 대기</x:v>
+      </x:c>
+      <x:c r="D119" s="19" t="str">
+        <x:v>“나 오늘 뭐 삭제했어?”라고 조회만 했는데 바로 복구 항목 선택 UI가 뜨는 하드코딩처럼 보이는 동작을 수정해 달라는 요청.</x:v>
+      </x:c>
+      <x:c r="E119" s="19" t="str">
+        <x:v>응답 후처리가 목록형 도구의 결과가 있으면 선택 필요 여부와 무관하게 selectionFrame을 항상 저장했다. 또한 이전 복구 작업이 collecting 상태이면 “삭제했어?” 같은 과거형 질문이 미완성 변경 권한을 승계할 여지가 있었다.</x:v>
+      </x:c>
+      <x:c r="F119" s="19" t="str">
+        <x:v>선택 프레임은 현재 요청이 선택 가능한 목록·번호 목록을 명시했거나 현재 요청에 승인된 변경 도구가 있는 경우에만 생성한다. 단순 조회에서는 모델의 텍스트 목록만 유지한다. 과거형 했어·됐어·지워졌나요를 변경 권한 승계 차단 질문으로 분류했다.</x:v>
+      </x:c>
+      <x:c r="G119" s="19" t="str">
+        <x:v>집중 41/41, Windows backend 전체 180건 중 172 pass·환경 8 skip·0 fail, git diff check 통과. 단순 삭제 내역 조회 4종은 selectionFrame=null이며 명시적 선택 목록·실제 복원 요청은 기존 선택 UI를 유지한다. 변경 권한이 있어도 모델이 선택을 요청하지 않은 무관한 목록에는 프레임을 붙이지 않는다.</x:v>
+      </x:c>
+      <x:c r="H119" s="19" t="str">
+        <x:v>운영 NAS 배포와 공개 Chrome의 실제 같은 문장 검증은 다음 단계에서 수행한다. 일반 목록 조회도 같은 공통 정책을 적용하므로 파일·사용자·노트 목록에서 불필요한 선택 카드가 제거된다.</x:v>
+      </x:c>
+      <x:c r="I119" s="19"/>
+      <x:c r="J119" s="19" t="str">
+        <x:v>AI-AGENT-TRASH-RESTORE</x:v>
+      </x:c>
+      <x:c r="K119" s="19" t="str">
+        <x:v>backend/aiResponsePolicy.js; backend/aiAgentRuntime.js; backend/tests/aiResponsePolicy.test.js; backend/tests/aiConversationContinuation.test.js</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6042,6 +6075,17 @@
         <x:v>AI가 1~4번 파일 복구를 진행한다고 답했지만 실제 복구와 actions.json 기록이 없었던 문제를 고치고, 실제 선택·승인·복구·서버 파일 검증까지 완료해 달라는 요청.</x:v>
       </x:c>
     </x:row>
+    <x:row r="106" ht="74" customHeight="1">
+      <x:c r="A106" s="19" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="B106" s="19" t="str">
+        <x:v>AI 단순 삭제 내역 조회의 복구 선택 UI 제거</x:v>
+      </x:c>
+      <x:c r="C106" s="19" t="str">
+        <x:v>나 오늘 뭐 삭제했어?라고만 물었는데 바로 복구 항목 선택이 뜨는 하드코딩 같은 동작을 고쳐 달라는 요청.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6787,6 +6831,23 @@
       </x:c>
       <x:c r="E58" s="19" t="str">
         <x:v>테스트 파일 1개만 복구하고 기존 네 휴지통 파일은 보존했다. 검증용 파일은 결과 확인 뒤 원위치에서 정리했으며 감사 기록은 유지했다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="96" customHeight="1">
+      <x:c r="A59" s="19" t="str">
+        <x:v>2026-10-02 AI 조회·선택 의도 분리</x:v>
+      </x:c>
+      <x:c r="B59" s="19" t="str">
+        <x:v>목록 도구 실행과 선택 UI 노출을 분리하고, 과거형 조회 질문이 이전 pending 변경 권한을 승계하지 않도록 했다.</x:v>
+      </x:c>
+      <x:c r="C59" s="19" t="str">
+        <x:v>집중 41/41, backend 172 pass·8 env skip·0 fail, 단순 조회 4종 selectionFrame null, 무관 목록 차단, 명시적 선택·복원 회귀 유지, diff check</x:v>
+      </x:c>
+      <x:c r="D59" s="19" t="str">
+        <x:v>구현·자동 검증 완료 / 운영 검증 대기</x:v>
+      </x:c>
+      <x:c r="E59" s="19" t="str">
+        <x:v>운영 배포 뒤 공개 Chrome에서 동일 문장으로 텍스트 목록만 보이고 선택 카드·복구 준비 버튼이 없는지 확인한다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9579,6 +9640,20 @@
         <x:v>서버가 저장된 assistant messageId와 sourceTool=list_trash를 기준으로 선택 목록을 다시 읽고 최신 휴지통의 trashId·이름·원래 경로·삭제 시각과 일치시킨다. restore_trash_items action을 생성해 승인 모드에 따라 실행하고, 실행 직전 재검증·항목별 결과·idempotency·actions.json 감사를 남긴 뒤 실제 결과만 완료 문구로 표시한다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="164" ht="110" customHeight="1">
+      <x:c r="A164" s="19" t="str">
+        <x:v>DNB-AI-LIST-SELECTION-INTENT-2026-10-02</x:v>
+      </x:c>
+      <x:c r="B164" s="19" t="str">
+        <x:v>AI 조회 목록과 작업 대상 선택 UI 분리</x:v>
+      </x:c>
+      <x:c r="C164" s="19" t="str">
+        <x:v>list_trash, search_files 등 목록 조회 도구가 결과를 반환했다는 이유만으로 선택 카드나 복구 준비 버튼을 붙이지 말 것. 과거 조회 질문이 이전 미완성 변경 작업의 권한을 이어받게 두지 말 것.</x:v>
+      </x:c>
+      <x:c r="D164" s="19" t="str">
+        <x:v>선택 프레임은 현재 사용자 요청이 선택 가능한 목록·번호 목록을 명시했거나 현재 요청에 승인된 변경 도구가 있을 때만 노출한다. 단순 조회는 텍스트 결과만 유지한다. 했어·됐어·지워졌나요 같은 과거형 질문은 이전 pending mutation을 승계하지 않는다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11918,7 +11993,7 @@
         <x:v>완료 · 운영 배포 · 실제 계정 E2E 검증</x:v>
       </x:c>
       <x:c r="D137" s="19" t="str">
-        <x:v>AI가 휴지통 목록을 번호 카드로 제시하고 사용자가 한 개 또는 여러 개를 고르면 서버가 원본 메시지와 최신 휴지통을 대조해 복구 action을 만든다. ask_each는 승인 카드 뒤 실제 복구하며 auto_reversible은 같은 검증 경로에서 즉시 실행한다. 부분 실패는 항목별로 남고 허위 완료 응답은 차단된다.</x:v>
+        <x:v>AI가 휴지통 목록을 번호 카드로 제시하는 것은 사용자가 복구 실행 또는 선택 가능한 목록을 명시한 경우에 한한다. 단순 삭제 내역 조회는 목록 답변만 제공한다. 사용자가 항목을 고르면 서버가 원본 메시지와 최신 휴지통을 대조해 복구 action을 만들고 승인 모드에 따라 실행한다.</x:v>
       </x:c>
       <x:c r="E137" s="19" t="str">
         <x:v>AI-AGENT, AI-AGENT-DURABLE-RUN, FILE-TRASH, AI-SELECTION-FRAME, Code_Map, Do_Not_Break, Patch_Log</x:v>
@@ -14806,7 +14881,7 @@
         <x:v>AI-SELECTION-FRAME / FILE-TRASH / AI-AGENT-DURABLE-RUN</x:v>
       </x:c>
       <x:c r="D205" s="19" t="str">
-        <x:v>선택 번호는 저장된 목록 messageId에 결속하고 서버의 최신 list_trash 결과로 실제 trashId를 재해석한다. 승인·자동 실행 모두 restore_trash_items runtime과 actions.json 결과 원장을 거쳐야 하며 오래되거나 바뀐 목록은 실패 폐쇄한다.</x:v>
+        <x:v>조회 결과 자체는 선택 의도가 아니다. 선택 프레임은 현재 요청의 명시적 선택 UI 요구 또는 승인된 변경 의도가 있을 때만 노출한다. 선택 뒤에는 저장된 목록 messageId와 최신 list_trash 결과를 대조해 실제 trashId를 재해석하고 restore_trash_items runtime과 actions.json을 거친다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -21804,10 +21879,10 @@
         <x:v>backend/aiSelectionExecution.js; backend/aiSelectionFrame.js; backend/aiAgentRoutes.js; backend/aiAgentRuntime.js; backend/aiAgentStore.js; backend/aiResponsePolicy.js; frontend/src/components/AiAgentPanel.js</x:v>
       </x:c>
       <x:c r="C499" s="19" t="str">
-        <x:v>선택 목록 메시지 식별, sourceTool 화이트리스트, 최신 휴지통 재결속, batch restore action 생성·승인·실행, 항목별 결과와 idempotency, 허위 복구 문구 차단, 복구 준비 UI</x:v>
+        <x:v>선택 목록 메시지 식별, 조회와 선택 UI 의도 분리, 과거형 질문의 pending 권한 승계 차단, 최신 휴지통 재결속, batch restore action 생성·승인·실행, 항목별 결과와 idempotency</x:v>
       </x:c>
       <x:c r="D499" s="19" t="str">
-        <x:v>클라이언트에서 보낸 trashId나 경로는 실행 권한 자료로 쓰지 않고 서버 저장 메시지와 현재 휴지통을 모두 대조한다.</x:v>
+        <x:v>클라이언트 경로·trashId는 실행 권한으로 쓰지 않는다. 목록 조회만 한 메시지에는 선택 프레임을 저장하지 않으며 선택을 명시한 현재 요청만 후속 실행 계약에 들어간다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Record AI query selection intent verification
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R2fc64a18d5ca4b89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Rf55fb6f671d24765"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="Rc5a6995047084cbc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R94974dd6a0d24f1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R7aa18f581b3e4f0a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R05a44ec26c884bb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R51508f7d00714cdc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R76e429a81e254fff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rcfbdad3071af4ac4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rf9a8f3bc67e04f5c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R55d482b84fb942d7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R8fb05a5e57e149d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="Raf8c5cfd48fb4bb4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="Rfb79feca60fd4c5e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Rcde7712218bb49e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R7c86f9086f004890"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R2588af745bf445cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R144d95fe25e34071"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Rd4d23aee90684b46"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R1333df969c024834"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Rceb80422f10647a4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R8f37025816fb4e42"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Rb37210e2fcbc45f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R129cffec71314e60"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Re04ed3b0114b4b9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Rb9044e8460644288"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="Rf27b82a867c14a19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="Ra52a88e198fe4f7a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R37be4f51ab6c4da7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R81c44c2db32d493b"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4875,7 +4875,7 @@
         <x:v>2026-10-02</x:v>
       </x:c>
       <x:c r="C119" s="19" t="str">
-        <x:v>구현·자동 검증 완료 / 운영 검증 대기</x:v>
+        <x:v>완료 · 운영 배포 · 실화면 검증</x:v>
       </x:c>
       <x:c r="D119" s="19" t="str">
         <x:v>“나 오늘 뭐 삭제했어?”라고 조회만 했는데 바로 복구 항목 선택 UI가 뜨는 하드코딩처럼 보이는 동작을 수정해 달라는 요청.</x:v>
@@ -4887,10 +4887,10 @@
         <x:v>선택 프레임은 현재 요청이 선택 가능한 목록·번호 목록을 명시했거나 현재 요청에 승인된 변경 도구가 있는 경우에만 생성한다. 단순 조회에서는 모델의 텍스트 목록만 유지한다. 과거형 했어·됐어·지워졌나요를 변경 권한 승계 차단 질문으로 분류했다.</x:v>
       </x:c>
       <x:c r="G119" s="19" t="str">
-        <x:v>집중 41/41, Windows backend 전체 180건 중 172 pass·환경 8 skip·0 fail, git diff check 통과. 단순 삭제 내역 조회 4종은 selectionFrame=null이며 명시적 선택 목록·실제 복원 요청은 기존 선택 UI를 유지한다. 변경 권한이 있어도 모델이 선택을 요청하지 않은 무관한 목록에는 프레임을 붙이지 않는다.</x:v>
+        <x:v>집중 41/41, Windows backend 전체 180건 중 172 pass·환경 8 skip·0 fail, NAS 집중 회귀 통과. 공개 Chrome에서 실제 “나 오늘 뭐 삭제했어?” 요청 후 삭제 파일 텍스트 목록만 표시되고 복구 선택 카드·복구 준비 버튼이 없는 것을 확인했다. 명시적 선택 목록·실제 복원 요청 회귀는 유지한다.</x:v>
       </x:c>
       <x:c r="H119" s="19" t="str">
-        <x:v>운영 NAS 배포와 공개 Chrome의 실제 같은 문장 검증은 다음 단계에서 수행한다. 일반 목록 조회도 같은 공통 정책을 적용하므로 파일·사용자·노트 목록에서 불필요한 선택 카드가 제거된다.</x:v>
+        <x:v>단순 조회는 선택 UI를 만들지 않는다. 복구 실행 또는 “선택 가능한 목록/번호로 보여줘”를 명시하면 기존 선택·승인 흐름을 사용한다.</x:v>
       </x:c>
       <x:c r="I119" s="19"/>
       <x:c r="J119" s="19" t="str">
@@ -6841,13 +6841,13 @@
         <x:v>목록 도구 실행과 선택 UI 노출을 분리하고, 과거형 조회 질문이 이전 pending 변경 권한을 승계하지 않도록 했다.</x:v>
       </x:c>
       <x:c r="C59" s="19" t="str">
-        <x:v>집중 41/41, backend 172 pass·8 env skip·0 fail, 단순 조회 4종 selectionFrame null, 무관 목록 차단, 명시적 선택·복원 회귀 유지, diff check</x:v>
+        <x:v>집중 41/41, backend 172 pass·8 env skip·0 fail, NAS 집중 회귀, 서비스·HTTP, 공개 Chrome 동일 문장 실화면, 선택 카드 부재 확인</x:v>
       </x:c>
       <x:c r="D59" s="19" t="str">
-        <x:v>구현·자동 검증 완료 / 운영 검증 대기</x:v>
+        <x:v>완료 · 운영 배포 · 실화면 검증</x:v>
       </x:c>
       <x:c r="E59" s="19" t="str">
-        <x:v>운영 배포 뒤 공개 Chrome에서 동일 문장으로 텍스트 목록만 보이고 선택 카드·복구 준비 버튼이 없는지 확인한다.</x:v>
+        <x:v>단순 조회에는 텍스트 목록만 표시하고, 명시적 복구·선택 요청에만 선택 프레임을 제공한다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Generalize AI query and selection intent
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R7c86f9086f004890"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R2588af745bf445cc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R144d95fe25e34071"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Rd4d23aee90684b46"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R1333df969c024834"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Rceb80422f10647a4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R8f37025816fb4e42"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Rb37210e2fcbc45f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R129cffec71314e60"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Re04ed3b0114b4b9f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Rb9044e8460644288"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="Rf27b82a867c14a19"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="Ra52a88e198fe4f7a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R37be4f51ab6c4da7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R81c44c2db32d493b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf460af104b5d4105"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R34d30a9280704cf7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="Red6c30a4d63247c6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Rb8d90dee55244a96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="Reb6826d4d9e54fc9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R16183195e3744a48"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Rbdc22961eeb44b68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Rf06e17ffe49945bc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rb255f6485fac4285"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rdb5f1a8f47764715"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R034d8b62d94741b5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="Rd11de93f89b94f1d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R085c905542ef4474"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R8250d6b4d82c4345"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Rf33cd7bf4b834f30"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4900,6 +4900,39 @@
         <x:v>backend/aiResponsePolicy.js; backend/aiAgentRuntime.js; backend/tests/aiResponsePolicy.test.js; backend/tests/aiConversationContinuation.test.js</x:v>
       </x:c>
     </x:row>
+    <x:row r="120" ht="170" customHeight="1">
+      <x:c r="A120" s="19" t="str">
+        <x:v>PATCH-AI-GLOBAL-INTENT-SELECTION-2026-10-02</x:v>
+      </x:c>
+      <x:c r="B120" s="19" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="C120" s="19" t="str">
+        <x:v>구현·자동 검증 완료 / 운영 검증 대기</x:v>
+      </x:c>
+      <x:c r="D120" s="19" t="str">
+        <x:v>“이런 거 말고도 다른 부분에 대해서도 마찬가지다”라는 요청에 따라 삭제·복구에 한정하지 않고 AI의 전체 조회·선택·실행 의도를 공통화한다.</x:v>
+      </x:c>
+      <x:c r="E120" s="19" t="str">
+        <x:v>알려줘가 전역 실행 어미라 변경 단어가 포함된 조회가 mutation 권한을 얻을 수 있었다. 또한 공통 선택 UI가 휴지통 외 항목도 구조화 selection으로 보내 휴지통 복구 전용 서버 경로에 잘못 진입할 수 있었다. 여러 조회 도구를 호출하면 현재 변경과 무관한 마지막 목록이 카드가 될 수도 있었다.</x:v>
+      </x:c>
+      <x:c r="F120" s="19" t="str">
+        <x:v>알려줘를 일반 실행 어미에서 제거하고 상대에게 알려줘·말해줘만 채팅 전송으로 분리했다. 선택 source와 mutation tool의 호환표를 추가해 현재 작업과 맞는 목록만 카드로 만든다. 휴지통만 결정적 서버 재결속을 사용하고 나머지 선택은 표시 문자열 후속 대화로 보내 최신 도구가 재검증한다.</x:v>
+      </x:c>
+      <x:c r="G120" s="19" t="str">
+        <x:v>집중 34/34, Windows backend 전체 185건 중 177 pass·환경 8 skip·0 fail, UI contract 121개 소스와 diff check가 통과했다. 로컬 production build는 기존 혼합 npm/pnpm eslint 경로 충돌로 중단되어 NAS에서 재검증한다.</x:v>
+      </x:c>
+      <x:c r="H120" s="19" t="str">
+        <x:v>운영 NAS 회귀·production/PDF.js build·서비스·HTTP·공개 Chrome 다영역 조회 검증이 남았다. 새 목록/변경 도구 추가 시 SOURCE_TO_MUTATIONS와 조회 문장 행렬을 같이 갱신한다.</x:v>
+      </x:c>
+      <x:c r="I120" s="19"/>
+      <x:c r="J120" s="19" t="str">
+        <x:v>AI-AGENT-INTENT-SELECTION</x:v>
+      </x:c>
+      <x:c r="K120" s="19" t="str">
+        <x:v>backend/aiAgentRuntime.js; backend/aiResponsePolicy.js; backend/aiSelectionFrame.js; frontend/src/components/AiAgentPanel.js</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6086,6 +6119,17 @@
         <x:v>나 오늘 뭐 삭제했어?라고만 물었는데 바로 복구 항목 선택이 뜨는 하드코딩 같은 동작을 고쳐 달라는 요청.</x:v>
       </x:c>
     </x:row>
+    <x:row r="107" ht="78" customHeight="1">
+      <x:c r="A107" s="19" t="str">
+        <x:v>2026-10-02</x:v>
+      </x:c>
+      <x:c r="B107" s="19" t="str">
+        <x:v>AI 전 영역 조회·선택·실행 의도 일반화</x:v>
+      </x:c>
+      <x:c r="C107" s="19" t="str">
+        <x:v>삭제·복구뿐 아니라 다른 부분도 같은 원칙을 적용해 단순 조회가 선택 UI나 변경 실행으로 바뀌지 않게 해 달라는 요청.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6848,6 +6892,23 @@
       </x:c>
       <x:c r="E59" s="19" t="str">
         <x:v>단순 조회에는 텍스트 목록만 표시하고, 명시적 복구·선택 요청에만 선택 프레임을 제공한다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60" ht="106" customHeight="1">
+      <x:c r="A60" s="19" t="str">
+        <x:v>2026-10-02 AI 전 영역 의도·선택 계약</x:v>
+      </x:c>
+      <x:c r="B60" s="19" t="str">
+        <x:v>정보 요청과 실행 명령, 선택 UI와 실제 변경, 휴지통 구조화 선택과 일반 선택 후속 대화를 공통 정책으로 분리했다.</x:v>
+      </x:c>
+      <x:c r="C60" s="19" t="str">
+        <x:v>집중 34/34, backend 177 pass·8 env skip·0 fail, UI contract 121 sources, diff check</x:v>
+      </x:c>
+      <x:c r="D60" s="19" t="str">
+        <x:v>구현·자동 검증 완료 / 운영 검증 대기</x:v>
+      </x:c>
+      <x:c r="E60" s="19" t="str">
+        <x:v>변경 단어가 포함된 조회도 mutation 권한 0개이며, 현재 변경과 무관한 목록은 선택 프레임 후보가 아니다. 휴지통 외 선택은 휴지통 복구 route를 호출하지 않는다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9654,6 +9715,20 @@
         <x:v>선택 프레임은 현재 사용자 요청이 선택 가능한 목록·번호 목록을 명시했거나 현재 요청에 승인된 변경 도구가 있을 때만 노출한다. 단순 조회는 텍스트 결과만 유지한다. 했어·됐어·지워졌나요 같은 과거형 질문은 이전 pending mutation을 승계하지 않는다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="165" ht="132" customHeight="1">
+      <x:c r="A165" s="19" t="str">
+        <x:v>DNB-AI-GLOBAL-INTENT-SELECTION-2026-10-02</x:v>
+      </x:c>
+      <x:c r="B165" s="19" t="str">
+        <x:v>AI 전 영역 조회·선택·실행 의도 분리</x:v>
+      </x:c>
+      <x:c r="C165" s="19" t="str">
+        <x:v>삭제·복구뿐 아니라 파일, 사용자, 친구, 채팅, 알림, 노트, 연동 PC, 공유, 회의, 관리자 기능에서 알려줘·보여줘·목록·상태·내역 같은 정보 요청을 변경 허가로 해석하지 말 것. 현재 작업과 무관한 조회 결과를 선택 카드로 붙이거나 휴지통 외 선택을 휴지통 복구 경로로 보내지 말 것.</x:v>
+      </x:c>
+      <x:c r="D165" s="19" t="str">
+        <x:v>변경 권한은 실제 실행 명령으로만 만든다. 누구에게 알려줘·말해줘는 채팅 전송으로 별도 식별한다. 선택 프레임은 승인된 변경 도구와 호환되는 최신 조회 결과에만 결속한다. 휴지통만 저장 메시지와 최신 trash를 결정적으로 재대조하고, 다른 선택은 표시 문자열을 새 대화로 보내 관련 조회 도구가 다시 검증한다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -11999,6 +12074,23 @@
         <x:v>AI-AGENT, AI-AGENT-DURABLE-RUN, FILE-TRASH, AI-SELECTION-FRAME, Code_Map, Do_Not_Break, Patch_Log</x:v>
       </x:c>
     </x:row>
+    <x:row r="138" ht="104" customHeight="1">
+      <x:c r="A138" s="19" t="str">
+        <x:v>AI-AGENT-INTENT-SELECTION</x:v>
+      </x:c>
+      <x:c r="B138" s="19" t="str">
+        <x:v>AI 전 영역 조회·선택·실행 계약</x:v>
+      </x:c>
+      <x:c r="C138" s="19" t="str">
+        <x:v>구현·자동 검증 완료 / 운영 검증 대기</x:v>
+      </x:c>
+      <x:c r="D138" s="19" t="str">
+        <x:v>파일·사용자·친구·채팅·알림·노트·연동 PC·공유·회의·관리자 영역의 조회를 변경 권한과 분리한다. 사용자가 선택 UI를 명시하거나 실제 변경 작업에 후보 선택이 필요할 때만 현재 작업과 호환되는 목록 카드를 표시한다.</x:v>
+      </x:c>
+      <x:c r="E138" s="19" t="str">
+        <x:v>AI-AGENT, AI-AGENT-TRASH-RESTORE, FILE, CHAT, NOTI, NOTE-STUDIO, WIN-PAIR, SHARE, MEET, USER-MGMT</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -14884,6 +14976,20 @@
         <x:v>조회 결과 자체는 선택 의도가 아니다. 선택 프레임은 현재 요청의 명시적 선택 UI 요구 또는 승인된 변경 의도가 있을 때만 노출한다. 선택 뒤에는 저장된 목록 messageId와 최신 list_trash 결과를 대조해 실제 trashId를 재해석하고 restore_trash_items runtime과 actions.json을 거친다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="206" ht="108" customHeight="1">
+      <x:c r="A206" s="19" t="str">
+        <x:v>AI-AGENT-INTENT-SELECTION</x:v>
+      </x:c>
+      <x:c r="B206" s="19" t="str">
+        <x:v>AI-AGENT-TRASH-RESTORE; FILE; CHAT; NOTI; NOTE-STUDIO; WIN-PAIR; SHARE; MEET; USER-MGMT</x:v>
+      </x:c>
+      <x:c r="C206" s="19" t="str">
+        <x:v>조회 질문은 실행 권한 0개다. 실제 실행 요청은 해당 mutation tool만 허가하고, 선택 프레임은 그 mutation과 호환되는 read tool 결과만 사용한다. 휴지통 외 선택은 휴지통 전용 구조화 실행 경로에 들어가지 않는다.</x:v>
+      </x:c>
+      <x:c r="D206" s="19" t="str">
+        <x:v>새 목록 도구나 변경 도구를 추가할 때 선택 호환 관계와 조회 문장 회귀를 함께 등록하지 않으면 선택 UI를 자동 노출하지 않는다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -21883,6 +21989,20 @@
       </x:c>
       <x:c r="D499" s="19" t="str">
         <x:v>클라이언트 경로·trashId는 실행 권한으로 쓰지 않는다. 목록 조회만 한 메시지에는 선택 프레임을 저장하지 않으며 선택을 명시한 현재 요청만 후속 실행 계약에 들어간다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="500" ht="112" customHeight="1">
+      <x:c r="A500" s="19" t="str">
+        <x:v>AI-AGENT-INTENT-SELECTION</x:v>
+      </x:c>
+      <x:c r="B500" s="19" t="str">
+        <x:v>backend/aiAgentRuntime.js; backend/aiResponsePolicy.js; backend/aiSelectionFrame.js; backend/aiAgentRoutes.js; frontend/src/components/AiAgentPanel.js; backend/tests/aiConversationContinuation.test.js; backend/tests/aiResponsePolicy.test.js; frontend/scripts/verify-ui-contract.mjs</x:v>
+      </x:c>
+      <x:c r="C500" s="19" t="str">
+        <x:v>정보 요청과 실행 명령 분리, mutation-to-list 호환표, 무관한 최신 목록 배제, 휴지통 전용 구조화 선택과 일반 선택 후속 대화 분리</x:v>
+      </x:c>
+      <x:c r="D500" s="19" t="str">
+        <x:v>알려줘를 전역 실행 어미로 사용하지 않는다. 외부 사용자에게 알려줘만 채팅 전송 의도로 유지하며, 선택 UI는 승인 작업과 source tool 호환성을 검사한다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Record global AI intent verification
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf460af104b5d4105"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R34d30a9280704cf7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="Red6c30a4d63247c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Rb8d90dee55244a96"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="Reb6826d4d9e54fc9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R16183195e3744a48"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Rbdc22961eeb44b68"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Rf06e17ffe49945bc"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rb255f6485fac4285"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rdb5f1a8f47764715"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R034d8b62d94741b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="Rd11de93f89b94f1d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R085c905542ef4474"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R8250d6b4d82c4345"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Rf33cd7bf4b834f30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra091fa9ba5a04cf8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Rf627a4244e2647d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="Rdcf8a5793acf4690"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R184b2c0bc8f7427b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R6fe0e51c30284254"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R6929e7f4757b4e5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R870bc74dbe354a6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Ra09da1cb1386486a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Racc77999139a4745"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rafeaff84203344ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R731eb19c52b5408f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="Rb56478229349411e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R129d9ebb97e84c14"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="Redfeae6a1c654e64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R904cc84289014e19"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4900,7 +4900,7 @@
         <x:v>backend/aiResponsePolicy.js; backend/aiAgentRuntime.js; backend/tests/aiResponsePolicy.test.js; backend/tests/aiConversationContinuation.test.js</x:v>
       </x:c>
     </x:row>
-    <x:row r="120" ht="170" customHeight="1">
+    <x:row r="120" ht="198" customHeight="1">
       <x:c r="A120" s="19" t="str">
         <x:v>PATCH-AI-GLOBAL-INTENT-SELECTION-2026-10-02</x:v>
       </x:c>
@@ -4908,7 +4908,7 @@
         <x:v>2026-10-02</x:v>
       </x:c>
       <x:c r="C120" s="19" t="str">
-        <x:v>구현·자동 검증 완료 / 운영 검증 대기</x:v>
+        <x:v>완료 · 운영 배포 · 실화면 검증</x:v>
       </x:c>
       <x:c r="D120" s="19" t="str">
         <x:v>“이런 거 말고도 다른 부분에 대해서도 마찬가지다”라는 요청에 따라 삭제·복구에 한정하지 않고 AI의 전체 조회·선택·실행 의도를 공통화한다.</x:v>
@@ -4920,10 +4920,10 @@
         <x:v>알려줘를 일반 실행 어미에서 제거하고 상대에게 알려줘·말해줘만 채팅 전송으로 분리했다. 선택 source와 mutation tool의 호환표를 추가해 현재 작업과 맞는 목록만 카드로 만든다. 휴지통만 결정적 서버 재결속을 사용하고 나머지 선택은 표시 문자열 후속 대화로 보내 최신 도구가 재검증한다.</x:v>
       </x:c>
       <x:c r="G120" s="19" t="str">
-        <x:v>집중 34/34, Windows backend 전체 185건 중 177 pass·환경 8 skip·0 fail, UI contract 121개 소스와 diff check가 통과했다. 로컬 production build는 기존 혼합 npm/pnpm eslint 경로 충돌로 중단되어 NAS에서 재검증한다.</x:v>
+        <x:v>집중 34/34, Windows backend 185건 중 177 pass·환경 8 skip·0 fail, NAS backend 185건 중 179 pass·런타임 6 skip·0 fail, UI contract 121개 소스, diff check 통과. NAS production build는 CI=false DISABLE_ESLINT_PLUGIN=true로 성공했고 PDF.js API/Worker 4.8.69 일치를 확인했다. 공개 Chrome에서 차단 사용자·연결 해제 PC·노트 목록 조회를 연속 실행해 기존 선택 카드 5개와 승인 안내 2개가 증가하지 않고 조회 답변만 표시됨을 확인했다. 서비스 전부 active, msp-backend online, 내부·공개 HTTP 200, 배포 bundle SHA-256 c27ae3e26a23085d016b18f2b9a87c694e7f3140ca95d79f11e1a6bd45c7217b.</x:v>
       </x:c>
       <x:c r="H120" s="19" t="str">
-        <x:v>운영 NAS 회귀·production/PDF.js build·서비스·HTTP·공개 Chrome 다영역 조회 검증이 남았다. 새 목록/변경 도구 추가 시 SOURCE_TO_MUTATIONS와 조회 문장 행렬을 같이 갱신한다.</x:v>
+        <x:v>새 조회·변경 도구를 추가할 때 SOURCE_TO_MUTATIONS 호환표와 정보요청 회귀 행렬을 함께 갱신해야 한다. 일반 선택은 표시 문자열 후속 대화에서 최신 목록을 재조회하므로 실제 변경 전 승인·대상 재검증 원칙을 유지한다.</x:v>
       </x:c>
       <x:c r="I120" s="19"/>
       <x:c r="J120" s="19" t="str">
@@ -6894,7 +6894,7 @@
         <x:v>단순 조회에는 텍스트 목록만 표시하고, 명시적 복구·선택 요청에만 선택 프레임을 제공한다.</x:v>
       </x:c>
     </x:row>
-    <x:row r="60" ht="106" customHeight="1">
+    <x:row r="60" ht="126" customHeight="1">
       <x:c r="A60" s="19" t="str">
         <x:v>2026-10-02 AI 전 영역 의도·선택 계약</x:v>
       </x:c>
@@ -6902,13 +6902,13 @@
         <x:v>정보 요청과 실행 명령, 선택 UI와 실제 변경, 휴지통 구조화 선택과 일반 선택 후속 대화를 공통 정책으로 분리했다.</x:v>
       </x:c>
       <x:c r="C60" s="19" t="str">
-        <x:v>집중 34/34, backend 177 pass·8 env skip·0 fail, UI contract 121 sources, diff check</x:v>
+        <x:v>집중 34/34; Windows 177 pass·8 skip; NAS 179 pass·6 skip; UI contract 121; production/PDF.js build; services/PM2/HTTP 200; 공개 Chrome 3개 영역에서 선택 카드·승인 안내 증가 0</x:v>
       </x:c>
       <x:c r="D60" s="19" t="str">
-        <x:v>구현·자동 검증 완료 / 운영 검증 대기</x:v>
+        <x:v>완료 · 운영 배포 · 실화면 검증</x:v>
       </x:c>
       <x:c r="E60" s="19" t="str">
-        <x:v>변경 단어가 포함된 조회도 mutation 권한 0개이며, 현재 변경과 무관한 목록은 선택 프레임 후보가 아니다. 휴지통 외 선택은 휴지통 복구 route를 호출하지 않는다.</x:v>
+        <x:v>차단 사용자·연결 해제 PC·노트 목록은 모두 텍스트 조회로 끝났고 새 선택·실행 UI를 만들지 않았다. 조회와 실행의 분리는 삭제·복구 전용 하드코딩이 아니라 공통 런타임·응답 정책으로 적용된다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12082,7 +12082,7 @@
         <x:v>AI 전 영역 조회·선택·실행 계약</x:v>
       </x:c>
       <x:c r="C138" s="19" t="str">
-        <x:v>구현·자동 검증 완료 / 운영 검증 대기</x:v>
+        <x:v>완료 · 운영 배포 · 실화면 검증</x:v>
       </x:c>
       <x:c r="D138" s="19" t="str">
         <x:v>파일·사용자·친구·채팅·알림·노트·연동 PC·공유·회의·관리자 영역의 조회를 변경 권한과 분리한다. 사용자가 선택 UI를 명시하거나 실제 변경 작업에 후보 선택이 필요할 때만 현재 작업과 호환되는 목록 카드를 표시한다.</x:v>

</xml_diff>

<commit_message>
feat: add Cresero organization mail control plane
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Ra091fa9ba5a04cf8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Rf627a4244e2647d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="Rdcf8a5793acf4690"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R184b2c0bc8f7427b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R6fe0e51c30284254"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R6929e7f4757b4e5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R870bc74dbe354a6c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Ra09da1cb1386486a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Racc77999139a4745"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rafeaff84203344ef"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R731eb19c52b5408f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="Rb56478229349411e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R129d9ebb97e84c14"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="Redfeae6a1c654e64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R904cc84289014e19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R3b26ba2f62414bc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Ra6590b597851469d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R52be0925cc82467d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Rc3f63732f2da409b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R32b40bf68cd24299"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R6b5ba280dc124096"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Raf706b1eb5654cae"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R88bb5117dc48414f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R527a92dbba6c4389"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rf40c27fe23ac4606"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R42195d1e47394805"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R26cfe267efa3428c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R3dd73f86d78e4e23"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R52685421fc1a424e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R077ecc3477ec4cea"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4933,6 +4933,41 @@
         <x:v>backend/aiAgentRuntime.js; backend/aiResponsePolicy.js; backend/aiSelectionFrame.js; frontend/src/components/AiAgentPanel.js</x:v>
       </x:c>
     </x:row>
+    <x:row r="121">
+      <x:c r="A121" s="19" t="str">
+        <x:v>PATCH-ORG-MAIL-CONTROL-2026-10-15</x:v>
+      </x:c>
+      <x:c r="B121" s="19" t="str">
+        <x:v>2026-10-15</x:v>
+      </x:c>
+      <x:c r="C121" s="19" t="str">
+        <x:v>로컬 구현·검증 완료 / 운영 배포·외부 연결 전</x:v>
+      </x:c>
+      <x:c r="D121" s="19" t="str">
+        <x:v>사용자@cresero.com 메일, 직책별 초기 계정, 회사 내·외부 회원가입과 명부·보안 설정을 알아서 구성.</x:v>
+      </x:c>
+      <x:c r="E121" s="19" t="str">
+        <x:v>실제 메일 제공자·DNS·사서함 상태가 없는데 주소만 미리 생성하면 송수신 성공으로 오인하고, NAS 권한과 회사 직책을 혼동할 수 있음.</x:v>
+      </x:c>
+      <x:c r="F121" s="19" t="str">
+        <x:v>제공자 미선택, Cloudflare DNS 쓰기 권한 부재, PTR 없음. 기존 계정은 조직 분류 정보가 없음.</x:v>
+      </x:c>
+      <x:c r="G121" s="19" t="str">
+        <x:v>제어면을 메일 제공자와 분리하고 fail-closed 상태로 구현. 일회용 해시 초대, 도메인 필터, 부서·직책, 예정 주소, 실시간 갱신, 초대 취소를 추가.</x:v>
+      </x:c>
+      <x:c r="H121" s="19" t="str">
+        <x:v>backend 51개 테스트 파일 0 fail, UI contract 122 source, production bundle·PDF.js 4.8.69, node syntax, diff-check. 운영 배포 후 추가 검증 예정.</x:v>
+      </x:c>
+      <x:c r="I121" s="19" t="str">
+        <x:v>외부 송수신·MFA·DKIM/SPF/DMARC는 아직 실행된 기능이 아니다. 제공자 가입·DNS 권한 후 연결해야 한다.</x:v>
+      </x:c>
+      <x:c r="J121" s="19" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="K121" s="19" t="str">
+        <x:v>backend/organizationDirectory.js; backend/index.js; frontend/src/components/OrganizationMailSettings.js; frontend/src/components/Signup.js; backend/tests/organizationDirectory.test.js; docs/programs/NAS_MAIL_SPEC.xlsx</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6130,6 +6165,17 @@
         <x:v>삭제·복구뿐 아니라 다른 부분도 같은 원칙을 적용해 단순 조회가 선택 UI나 변경 실행으로 바뀌지 않게 해 달라는 요청.</x:v>
       </x:c>
     </x:row>
+    <x:row r="108">
+      <x:c r="A108" s="19" t="str">
+        <x:v>2026-10-15</x:v>
+      </x:c>
+      <x:c r="B108" s="19" t="str">
+        <x:v>Cresero 조직 메일·가입 구성</x:v>
+      </x:c>
+      <x:c r="C108" s="19" t="str">
+        <x:v>모든 직책의 @cresero.com 메일 초기값, 회사 내·외부 가입 분리, 명부·보안 설정을 NAS 관리자 화면에 구성해 나중에 사용자가 수정할 수 있게 해달라는 요청.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6909,6 +6955,23 @@
       </x:c>
       <x:c r="E60" s="19" t="str">
         <x:v>차단 사용자·연결 해제 PC·노트 목록은 모두 텍스트 조회로 끝났고 새 선택·실행 UI를 만들지 않았다. 조회와 실행의 분리는 삭제·복구 전용 하드코딩이 아니라 공통 런타임·응답 정책으로 적용된다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="61">
+      <x:c r="A61" s="19" t="str">
+        <x:v>2026-10-15 Cresero 조직·메일 제어면</x:v>
+      </x:c>
+      <x:c r="B61" s="19" t="str">
+        <x:v>조직 정책·부서·직책·초대·명부·예정 메일을 실제 제공자와 분리하여 구현했다.</x:v>
+      </x:c>
+      <x:c r="C61" s="19" t="str">
+        <x:v>artifact-tool 기존 행 스타일 보존·재열기·수식 오류·문자 깨짐·렌더; backend 51 files; UI 122 sources; production/PDF.js</x:v>
+      </x:c>
+      <x:c r="D61" s="19" t="str">
+        <x:v>로컬 검증 통과 / 운영 배포 전</x:v>
+      </x:c>
+      <x:c r="E61" s="19" t="str">
+        <x:v>외부 메일 제공자·Cloudflare DNS 쓰기 권한·MFA 구현은 보류 항목으로 분리했다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7283,6 +7346,41 @@
         <x:v>2026-09-07</x:v>
       </x:c>
     </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
+        <x:v>PENDING-CRESERO-MAIL-PROVIDER-2026-10-15</x:v>
+      </x:c>
+      <x:c r="B11" t="str">
+        <x:v>2026-10-15</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>사용자 조치 대기</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>cresero.com 실제 사서함, 송수신, MFA, SPF/DKIM/DMARC, NAS 웹메일 연결</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>메일 제공자 계정·요금제·관리 API 인증정보가 없고 Cloudflare 인증에 DNS 쓰기 범위가 없음. 서버 IP에 PTR도 없어 직접 발송 서버는 안전하지 않음.</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>포트 25 outbound 가능, nginx가 443 사용, 메일 포트·제공자는 미구성. 제어면은 UNCONFIGURED에서 fail-closed.</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>사용자가 선택한 메일 제공자 가입·결제, API 키/관리자 위임, Cloudflare DNS Edit 재인증</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>제공자 샌드박스에서 사용자 1명 생성·정지·비밀번호 초기화·송수신·SPF/DKIM/DMARC 검증 후 점진 배포</x:v>
+      </x:c>
+      <x:c r="J11" t="str">
+        <x:v>PATCH-ORG-MAIL-CONTROL-2026-10-15; docs/programs/NAS_MAIL_SPEC.xlsx</x:v>
+      </x:c>
+      <x:c r="K11" t="str">
+        <x:v>2026-10-15</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="C2:C500">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="보류"/>
@@ -9729,6 +9827,20 @@
         <x:v>변경 권한은 실제 실행 명령으로만 만든다. 누구에게 알려줘·말해줘는 채팅 전송으로 별도 식별한다. 선택 프레임은 승인된 변경 도구와 호환되는 최신 조회 결과에만 결속한다. 휴지통만 저장 메시지와 최신 trash를 결정적으로 재대조하고, 다른 선택은 표시 문자열을 새 대화로 보내 관련 조회 도구가 다시 검증한다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="166">
+      <x:c r="A166" s="19" t="str">
+        <x:v>DNB-ORG-MAIL-BOUNDARY</x:v>
+      </x:c>
+      <x:c r="B166" s="19" t="str">
+        <x:v>조직·메일 계정 보안 경계</x:v>
+      </x:c>
+      <x:c r="C166" s="19" t="str">
+        <x:v>NAS MASTER/MANAGER/USER 권한과 회사 직책을 같은 값으로 간주하지 말 것. 기존 계정을 자동으로 내부 임직원으로 승격하지 말 것. 메일 제공자가 연결되기 전에 주소를 사용 가능으로 표시하지 말 것.</x:v>
+      </x:c>
+      <x:c r="D166" s="19" t="str">
+        <x:v>기존 계정은 UNCLASSIFIED/REVIEW_REQUIRED로 등록하고 마스터가 분류한다. 내부 초대는 마스터만 발급·취소하며 일회용 토큰은 SHA-256 해시만 저장한다. 외부 가입 개방은 이메일 본인 확인 제공자 ACTIVE 후에만 허용한다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -12091,6 +12203,23 @@
         <x:v>AI-AGENT, AI-AGENT-TRASH-RESTORE, FILE, CHAT, NOTI, NOTE-STUDIO, WIN-PAIR, SHARE, MEET, USER-MGMT</x:v>
       </x:c>
     </x:row>
+    <x:row r="139">
+      <x:c r="A139" s="19" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="B139" s="19" t="str">
+        <x:v>조직 명부·cresero.com 메일 제어면</x:v>
+      </x:c>
+      <x:c r="C139" s="19" t="str">
+        <x:v>관리 기반 구현·로컬 검증 완료 / 외부 제공자·DNS 연결 보류</x:v>
+      </x:c>
+      <x:c r="D139" s="19" t="str">
+        <x:v>내부·외부·서비스 계정 분리, 부서·직책, 일회용 초대, 도메인 허용·차단, 계정별 예정 메일 주소, 제공자 상태를 하나의 관리 화면에서 관리한다.</x:v>
+      </x:c>
+      <x:c r="E139" s="19" t="str">
+        <x:v>AUTH, USER-MANAGEMENT, STORAGE-QUOTA, Settings, Code_Map, API_Routes, Data_Files, NAS_MAIL_SPEC.xlsx</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -14990,6 +15119,20 @@
         <x:v>새 목록 도구나 변경 도구를 추가할 때 선택 호환 관계와 조회 문장 회귀를 함께 등록하지 않으면 선택 UI를 자동 노출하지 않는다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="207">
+      <x:c r="A207" s="19" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="B207" s="19" t="str">
+        <x:v>separates_authorization_from</x:v>
+      </x:c>
+      <x:c r="C207" s="19" t="str">
+        <x:v>NAS ROLE / COMPANY POSITION / MAIL PROVIDER</x:v>
+      </x:c>
+      <x:c r="D207" s="19" t="str">
+        <x:v>대표이사·CTO 같은 회사 직책이 NAS MASTER 권한을 자동 부여하지 않으며, 메일 제공자 상태가 실제 사서함 상태의 정본이다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -22003,6 +22146,76 @@
       </x:c>
       <x:c r="D500" s="19" t="str">
         <x:v>알려줘를 전역 실행 어미로 사용하지 않는다. 외부 사용자에게 알려줘만 채팅 전송 의도로 유지하며, 선택 UI는 승인 작업과 source tool 호환성을 검사한다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="501">
+      <x:c r="A501" s="19" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="B501" s="19" t="str">
+        <x:v>backend/organizationDirectory.js</x:v>
+      </x:c>
+      <x:c r="C501" s="19" t="str">
+        <x:v>조직 정책·명부·초대·메일 주소·감사 이력을 원자적 JSON으로 관리.</x:v>
+      </x:c>
+      <x:c r="D501" s="19" t="str">
+        <x:v>원문 초대 토큰·비밀번호·제공자 인증정보 저장 금지</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="502">
+      <x:c r="A502" s="19" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="B502" s="19" t="str">
+        <x:v>backend/index.js</x:v>
+      </x:c>
+      <x:c r="C502" s="19" t="str">
+        <x:v>공개 가입 정책과 매니저/마스터 조직 관리 API, 회원가입·승인·삭제 연동.</x:v>
+      </x:c>
+      <x:c r="D502" s="19" t="str">
+        <x:v>내부 초대·구조 변경은 MASTER 확인</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="503">
+      <x:c r="A503" s="19" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="B503" s="19" t="str">
+        <x:v>frontend/src/components/OrganizationMailSettings.js</x:v>
+      </x:c>
+      <x:c r="C503" s="19" t="str">
+        <x:v>정책, 부서·직책, 일회용 초대·취소, 명부·메일 상태 관리 UI.</x:v>
+      </x:c>
+      <x:c r="D503" s="19" t="str">
+        <x:v>제공자 미연결 시 실제 송수신 가능 표시 금지</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="504">
+      <x:c r="A504" s="19" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="B504" s="19" t="str">
+        <x:v>frontend/src/components/Signup.js</x:v>
+      </x:c>
+      <x:c r="C504" s="19" t="str">
+        <x:v>내부·외부 가입 분기와 초대 링크 수신.</x:v>
+      </x:c>
+      <x:c r="D504" s="19" t="str">
+        <x:v>URL의 초대 토큰은 로드 즉시 history에서 제거</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="505">
+      <x:c r="A505" s="19" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="B505" s="19" t="str">
+        <x:v>backend/tests/organizationDirectory.test.js</x:v>
+      </x:c>
+      <x:c r="C505" s="19" t="str">
+        <x:v>초대·권한·충돌·예약어·구조·정지 회귀 검증.</x:v>
+      </x:c>
+      <x:c r="D505" s="19" t="str">
+        <x:v>외부 유료 API 호출 없음</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -25452,6 +25665,153 @@
       </x:c>
       <x:c r="E201" s="24" t="str">
         <x:v>표시 이름·kind revision 갱신</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="202">
+      <x:c r="A202" s="24" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="B202" s="24" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C202" s="24" t="str">
+        <x:v>/api/organization/signup-policy</x:v>
+      </x:c>
+      <x:c r="D202" s="24" t="str">
+        <x:v>backend/index.js</x:v>
+      </x:c>
+      <x:c r="E202" s="24" t="str"/>
+      <x:c r="F202" t="str">
+        <x:v>공개 가입 유형·초대 필요 여부만 반환</x:v>
+      </x:c>
+      <x:c r="G202" t="str">
+        <x:v>인증 없음/비밀 정보 제외</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="203">
+      <x:c r="A203" s="24" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="B203" s="24" t="str">
+        <x:v>GET</x:v>
+      </x:c>
+      <x:c r="C203" s="24" t="str">
+        <x:v>/api/organization/admin</x:v>
+      </x:c>
+      <x:c r="D203" s="24" t="str">
+        <x:v>backend/index.js</x:v>
+      </x:c>
+      <x:c r="E203" s="24" t="str"/>
+      <x:c r="F203" t="str">
+        <x:v>조직 명부·정책·초대·감사 상태</x:v>
+      </x:c>
+      <x:c r="G203" t="str">
+        <x:v>MANAGER 이상/토큰 해시 제외</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="204">
+      <x:c r="A204" s="24" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="B204" s="24" t="str">
+        <x:v>PUT</x:v>
+      </x:c>
+      <x:c r="C204" s="24" t="str">
+        <x:v>/api/organization/policy</x:v>
+      </x:c>
+      <x:c r="D204" s="24" t="str">
+        <x:v>backend/index.js</x:v>
+      </x:c>
+      <x:c r="E204" s="24" t="str"/>
+      <x:c r="F204" t="str">
+        <x:v>가입·메일 발급 정책</x:v>
+      </x:c>
+      <x:c r="G204" t="str">
+        <x:v>MASTER</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="205">
+      <x:c r="A205" s="24" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="B205" s="24" t="str">
+        <x:v>PUT</x:v>
+      </x:c>
+      <x:c r="C205" s="24" t="str">
+        <x:v>/api/organization/structure</x:v>
+      </x:c>
+      <x:c r="D205" s="24" t="str">
+        <x:v>backend/index.js</x:v>
+      </x:c>
+      <x:c r="E205" s="24" t="str"/>
+      <x:c r="F205" t="str">
+        <x:v>부서·직책 구조 저장</x:v>
+      </x:c>
+      <x:c r="G205" t="str">
+        <x:v>MASTER/사용 중 ID 삭제 거부</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="206">
+      <x:c r="A206" s="24" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="B206" s="24" t="str">
+        <x:v>POST</x:v>
+      </x:c>
+      <x:c r="C206" s="24" t="str">
+        <x:v>/api/organization/invitations</x:v>
+      </x:c>
+      <x:c r="D206" s="24" t="str">
+        <x:v>backend/index.js</x:v>
+      </x:c>
+      <x:c r="E206" s="24" t="str"/>
+      <x:c r="F206" t="str">
+        <x:v>일회용 초대 발급</x:v>
+      </x:c>
+      <x:c r="G206" t="str">
+        <x:v>내부=MASTER, 외부=MANAGER 이상</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="207">
+      <x:c r="A207" s="24" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="B207" s="24" t="str">
+        <x:v>DELETE</x:v>
+      </x:c>
+      <x:c r="C207" s="24" t="str">
+        <x:v>/api/organization/invitations/:invitationId</x:v>
+      </x:c>
+      <x:c r="D207" s="24" t="str">
+        <x:v>backend/index.js</x:v>
+      </x:c>
+      <x:c r="E207" s="24" t="str"/>
+      <x:c r="F207" t="str">
+        <x:v>미사용 초대 취소</x:v>
+      </x:c>
+      <x:c r="G207" t="str">
+        <x:v>내부=MASTER, 외부=MANAGER 이상</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="208">
+      <x:c r="A208" s="24" t="str">
+        <x:v>ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="B208" s="24" t="str">
+        <x:v>PUT</x:v>
+      </x:c>
+      <x:c r="C208" s="24" t="str">
+        <x:v>/api/organization/users/:userUid</x:v>
+      </x:c>
+      <x:c r="D208" s="24" t="str">
+        <x:v>backend/index.js</x:v>
+      </x:c>
+      <x:c r="E208" s="24" t="str"/>
+      <x:c r="F208" t="str">
+        <x:v>계정 유형·부서·직책·예정 메일 수정</x:v>
+      </x:c>
+      <x:c r="G208" t="str">
+        <x:v>MASTER</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -27276,6 +27636,20 @@
         <x:v>장치별 마지막 화면 상태와 계정 최신 fallback. 디렉터리 0700, 파일 0600, 임시 파일+rename. 비밀번호·token·cookie·credential 키는 저장 거부.</x:v>
       </x:c>
     </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="24" t="str">
+        <x:v>backend/data/organization_directory.json</x:v>
+      </x:c>
+      <x:c r="B26" s="24" t="str">
+        <x:v>운영 시 생성</x:v>
+      </x:c>
+      <x:c r="C26" s="24" t="str">
+        <x:v>조직 정책·명부·초대 해시·예정 메일·감사 이력</x:v>
+      </x:c>
+      <x:c r="D26" s="24" t="str">
+        <x:v>Git 제외. 디렉터리 0700/파일 0600, 원문 토큰·비밀번호·외부 제공자 키 저장 금지.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
docs: record Cresero mail deployment verification
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R3b26ba2f62414bc7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Ra6590b597851469d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R52be0925cc82467d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Rc3f63732f2da409b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R32b40bf68cd24299"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R6b5ba280dc124096"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Raf706b1eb5654cae"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R88bb5117dc48414f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R527a92dbba6c4389"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rf40c27fe23ac4606"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R42195d1e47394805"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R26cfe267efa3428c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R3dd73f86d78e4e23"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R52685421fc1a424e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R077ecc3477ec4cea"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rdd87e9b8888c439f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R8dc33a9d17514609"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R6ed947517c6f43f2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R0c26c50b19ae4a39"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R03fd6388646a465c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Re33104784f554d7b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Rab37e0a1e0a746b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Rf213b8eb9b5a452a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Re1a0825ab8f645f5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Recbb7a1dd9664d2a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R5dc461d8dbaf423a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R4076e0bf06134e86"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R9ba8c4b9661e438d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R9da215029bbd4a45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Rca1b70ba1cd741c9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4941,7 +4941,7 @@
         <x:v>2026-10-15</x:v>
       </x:c>
       <x:c r="C121" s="19" t="str">
-        <x:v>로컬 구현·검증 완료 / 운영 배포·외부 연결 전</x:v>
+        <x:v>운영 배포·검증 완료 / 외부 제공자·DNS 연결 보류</x:v>
       </x:c>
       <x:c r="D121" s="19" t="str">
         <x:v>사용자@cresero.com 메일, 직책별 초기 계정, 회사 내·외부 회원가입과 명부·보안 설정을 알아서 구성.</x:v>
@@ -4956,7 +4956,7 @@
         <x:v>제어면을 메일 제공자와 분리하고 fail-closed 상태로 구현. 일회용 해시 초대, 도메인 필터, 부서·직책, 예정 주소, 실시간 갱신, 초대 취소를 추가.</x:v>
       </x:c>
       <x:c r="H121" s="19" t="str">
-        <x:v>backend 51개 테스트 파일 0 fail, UI contract 122 source, production bundle·PDF.js 4.8.69, node syntax, diff-check. 운영 배포 후 추가 검증 예정.</x:v>
+        <x:v>Windows·NAS backend 51 test files 0 fail, UI contract 122 source, Linux production/PDF.js build, PM2 online, 필수 서비스 6개 active, 공개 policy·site·bundle HTTP 200, 비인증 admin 403, 25 members=25 identities, browser 가입 UI·내외부 분기·console error 0</x:v>
       </x:c>
       <x:c r="I121" s="19" t="str">
         <x:v>외부 송수신·MFA·DKIM/SPF/DMARC는 아직 실행된 기능이 아니다. 제공자 가입·DNS 권한 후 연결해야 한다.</x:v>
@@ -6968,7 +6968,7 @@
         <x:v>artifact-tool 기존 행 스타일 보존·재열기·수식 오류·문자 깨짐·렌더; backend 51 files; UI 122 sources; production/PDF.js</x:v>
       </x:c>
       <x:c r="D61" s="19" t="str">
-        <x:v>로컬 검증 통과 / 운영 배포 전</x:v>
+        <x:v>운영 배포·검증 통과 / 실제 메일 제공자 연결 전</x:v>
       </x:c>
       <x:c r="E61" s="19" t="str">
         <x:v>외부 메일 제공자·Cloudflare DNS 쓰기 권한·MFA 구현은 보류 항목으로 분리했다.</x:v>

</xml_diff>

<commit_message>
feat: reserve Cresero addresses for NAS signups
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rdd87e9b8888c439f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R8dc33a9d17514609"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R6ed947517c6f43f2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R0c26c50b19ae4a39"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R03fd6388646a465c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Re33104784f554d7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Rab37e0a1e0a746b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Rf213b8eb9b5a452a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Re1a0825ab8f645f5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Recbb7a1dd9664d2a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R5dc461d8dbaf423a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R4076e0bf06134e86"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R9ba8c4b9661e438d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R9da215029bbd4a45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Rca1b70ba1cd741c9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R06199fb0d0ea4ba3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R2d24519cd3644d0e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="Rca9d757306054812"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R853580f869944c67"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R61b99b2f8df24911"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Re9aea4ed734c4ab4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R775985c42f144c40"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Redc6166fb3074cff"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rdc53cd16d27f40e6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Re984f3e676ed499c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R1739e48342e6422f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="Rdc2f91ae8693495a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="Rcfeddf81a83d4853"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="Rfde27a8c55ca4b91"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R3f03a3d979a8479a"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4968,6 +4968,39 @@
         <x:v>backend/organizationDirectory.js; backend/index.js; frontend/src/components/OrganizationMailSettings.js; frontend/src/components/Signup.js; backend/tests/organizationDirectory.test.js; docs/programs/NAS_MAIL_SPEC.xlsx</x:v>
       </x:c>
     </x:row>
+    <x:row r="122">
+      <x:c r="A122" s="19" t="str">
+        <x:v>PATCH-ORG-MAIL-ID-AUTO-2026-10-16</x:v>
+      </x:c>
+      <x:c r="B122" s="19" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="C122" s="19" t="str">
+        <x:v>구현·로컬 전체 회귀 완료 / 운영 배포·외부 제공자 연결 대기</x:v>
+      </x:c>
+      <x:c r="D122" s="19" t="str">
+        <x:v>앞으로 회원가입 ID와 같은 @cresero.com 이메일 주소를 자동으로 만들고 기존 Cresero 주소와 혼란이 없게 하며, 앞서 만든 계정도 NAS 계정과 연결해 달라는 요청.</x:v>
+      </x:c>
+      <x:c r="E122" s="19" t="str">
+        <x:v>NAS 로그인 ID·가입 대기·조직 identity·공용 주소가 서로 다른 목록이라 승인 대기 중 주소 선점과 대소문자/예약어 충돌을 한 번에 막지 못했다. 실제 메일 제공자는 UNCONFIGURED라 사서함 생성 완료를 주장할 수도 없다.</x:v>
+      </x:c>
+      <x:c r="F122" s="19" t="str">
+        <x:v>가입 ID를 소문자 이메일형 이름공간으로 제한하고 signup request와 mailReservations를 userUid로 결속했다. 승인 시 identity로 승격, 거절 시 해제하며 기존 NAS 계정은 안전한 ID만 PLANNED로 백필한다. 점 포함 ID의 개인 저장공간 경로도 허용하되 선행·후행·연속 점은 차단한다. 기존 Cresero 서비스 계정 비밀번호는 복사하지 않고 후속 SSO/활성화 연결 대상으로 분리했다.</x:v>
+      </x:c>
+      <x:c r="G122" s="19" t="str">
+        <x:v>organizationDirectory 및 storageCapacity 단위 시험, Windows backend 51 test files 0 fail(환경 의존 skip 유지), UI contract 122 source, production build main.8c853416.js, react-pdf 9.2.1/PDF.js 4.8.69, JavaScript 구문·diff check 통과.</x:v>
+      </x:c>
+      <x:c r="H122" s="19" t="str">
+        <x:v>운영 배포와 실제 회원가입 화면 E2E, 기존 NAS 데이터 백필 집계, 외부 메일 제공자의 기존 주소 목록 동기화, Cresero Event Studio 기존 계정의 SSO 기반 NAS 활성화는 후속 검증이 필요하다.</x:v>
+      </x:c>
+      <x:c r="I122" s="19" t="str">
+        <x:v>ORG-MAIL-ID-AUTO</x:v>
+      </x:c>
+      <x:c r="J122" s="19" t="str">
+        <x:v>backend/organizationDirectory.js; backend/index.js; backend/storageQuota.js; frontend/src/components/Signup.js; frontend/src/components/OrganizationMailSettings.js; backend/tests/organizationDirectory.test.js; backend/tests/storageCapacity.test.js</x:v>
+      </x:c>
+      <x:c r="K122" s="19" t="str"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6176,6 +6209,17 @@
         <x:v>모든 직책의 @cresero.com 메일 초기값, 회사 내·외부 가입 분리, 명부·보안 설정을 NAS 관리자 화면에 구성해 나중에 사용자가 수정할 수 있게 해달라는 요청.</x:v>
       </x:c>
     </x:row>
+    <x:row r="109">
+      <x:c r="A109" s="19" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="B109" s="19" t="str">
+        <x:v>회원가입 ID와 Cresero 메일·NAS 계정 자동 결속</x:v>
+      </x:c>
+      <x:c r="C109" s="19" t="str">
+        <x:v>회원가입 때 입력한 ID로 id@cresero.com 주소를 자동 준비하고 기존 Cresero 주소와 중복되지 않게 하며, 기존 Cresero 계정도 NAS 계정과 연결해 달라는 요청.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6972,6 +7016,23 @@
       </x:c>
       <x:c r="E61" s="19" t="str">
         <x:v>외부 메일 제공자·Cloudflare DNS 쓰기 권한·MFA 구현은 보류 항목으로 분리했다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="62">
+      <x:c r="A62" s="19" t="str">
+        <x:v>2026-10-16 가입 ID 기반 Cresero 주소 예약</x:v>
+      </x:c>
+      <x:c r="B62" s="19" t="str">
+        <x:v>가입 요청 단계의 주소 예약, 승인 결속, 거절 해제, 기존 NAS 사용자 안전 백필과 가입 화면 주소 미리보기를 구현했다.</x:v>
+      </x:c>
+      <x:c r="C62" s="19" t="str">
+        <x:v>organizationDirectory 단위 시험; Windows backend 51 test files 0 fail; UI contract 122 source; production/PDF.js build; JavaScript 구문·diff check 통과.</x:v>
+      </x:c>
+      <x:c r="D62" s="19" t="str">
+        <x:v>로컬 구현 검증 완료 / 운영 배포·실화면·외부 제공자 동기화 대기</x:v>
+      </x:c>
+      <x:c r="E62" s="19" t="str">
+        <x:v>provider UNCONFIGURED에서는 주소를 PLANNED로만 표시한다. 공용/시스템 주소는 개인 NAS 계정으로 만들지 않으며 기존 Cresero 비밀번호 해시는 복사하지 않는다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7354,31 +7415,31 @@
         <x:v>2026-10-15</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>사용자 조치 대기</x:v>
+        <x:v>가입 주소 예약 구현·실제 제공자/기존 계정 SSO 대기</x:v>
       </x:c>
       <x:c r="D11" t="str">
         <x:v>ORG-MAIL-CONTROL</x:v>
       </x:c>
       <x:c r="E11" t="str">
-        <x:v>cresero.com 실제 사서함, 송수신, MFA, SPF/DKIM/DMARC, NAS 웹메일 연결</x:v>
+        <x:v>cresero.com 실제 사서함·송수신·MFA·SPF/DKIM/DMARC·NAS 웹메일과 Cresero 기존 계정의 NAS SSO 활성화</x:v>
       </x:c>
       <x:c r="F11" t="str">
-        <x:v>메일 제공자 계정·요금제·관리 API 인증정보가 없고 Cloudflare 인증에 DNS 쓰기 범위가 없음. 서버 IP에 PTR도 없어 직접 발송 서버는 안전하지 않음.</x:v>
+        <x:v>메일 제공자 계정·요금제·관리 API 인증정보가 없고, Cresero Event Studio와 NAS는 서로 다른 비밀번호 해시·세션을 사용한다. 비밀번호 복사나 동일 ID 자동 병합은 계정 탈취 위험이 있어 금지한다.</x:v>
       </x:c>
       <x:c r="G11" t="str">
-        <x:v>포트 25 outbound 가능, nginx가 443 사용, 메일 포트·제공자는 미구성. 제어면은 UNCONFIGURED에서 fail-closed.</x:v>
+        <x:v>신규 NAS 가입 ID의 @cresero.com 예약·승인 결속·거절 해제와 기존 NAS 안전 백필은 구현됐다. 외부 제공자는 UNCONFIGURED이고 Event Studio 기존 계정 명단의 검증된 연결은 아직 없다.</x:v>
       </x:c>
       <x:c r="H11" t="str">
-        <x:v>사용자가 선택한 메일 제공자 가입·결제, API 키/관리자 위임, Cloudflare DNS Edit 재인증</x:v>
+        <x:v>메일 제공자 가입·관리 OAuth와 DNS 권한, Cresero↔NAS SSO 서명키·계정 소유권 검증 흐름 확정</x:v>
       </x:c>
       <x:c r="I11" t="str">
-        <x:v>제공자 샌드박스에서 사용자 1명 생성·정지·비밀번호 초기화·송수신·SPF/DKIM/DMARC 검증 후 점진 배포</x:v>
+        <x:v>테스트 계정 1개로 Cresero 로그인→NAS 최초 활성화→20GiB 루트 생성→메일 사서함 프로비저닝→중복/충돌/정지/복구를 검증한 뒤 기존 계정을 일괄 이관한다.</x:v>
       </x:c>
       <x:c r="J11" t="str">
-        <x:v>PATCH-ORG-MAIL-CONTROL-2026-10-15; docs/programs/NAS_MAIL_SPEC.xlsx</x:v>
+        <x:v>PATCH-ORG-MAIL-CONTROL-2026-10-15; PATCH-ORG-MAIL-ID-AUTO-2026-10-16; docs/programs/NAS_MAIL_SPEC.xlsx</x:v>
       </x:c>
       <x:c r="K11" t="str">
-        <x:v>2026-10-15</x:v>
+        <x:v>2026-10-16</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9841,6 +9902,20 @@
         <x:v>기존 계정은 UNCLASSIFIED/REVIEW_REQUIRED로 등록하고 마스터가 분류한다. 내부 초대는 마스터만 발급·취소하며 일회용 토큰은 SHA-256 해시만 저장한다. 외부 가입 개방은 이메일 본인 확인 제공자 ACTIVE 후에만 허용한다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="167">
+      <x:c r="A167" s="19" t="str">
+        <x:v>DNB-ORG-MAIL-ID-NAMESPACE</x:v>
+      </x:c>
+      <x:c r="B167" s="19" t="str">
+        <x:v>NAS 로그인 ID와 Cresero 메일 주소 이름공간</x:v>
+      </x:c>
+      <x:c r="C167" s="19" t="str">
+        <x:v>가입 ID와 메일 주소를 따로 중복 검사하거나 승인 뒤에 주소를 배정하면 승인 대기 중 선점, 대소문자 중복, 공용 주소 충돌이 생긴다. 실제 제공자가 연결되지 않았는데 ACTIVE 사서함으로 표시하지 말 것.</x:v>
+      </x:c>
+      <x:c r="D167" s="19" t="str">
+        <x:v>신규 ID는 소문자 영문·숫자·점만 허용하고 가입 요청 단계에서 id@cresero.com을 원자적으로 예약한다. NAS 사용자·가입 대기·개인 주소·공용/시스템 주소·예약 목록을 한 번에 검사한다. 제공자 UNCONFIGURED에서는 PLANNED만 사용하고 공용 주소는 사람 NAS 계정으로 만들지 않는다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -12220,6 +12295,23 @@
         <x:v>AUTH, USER-MANAGEMENT, STORAGE-QUOTA, Settings, Code_Map, API_Routes, Data_Files, NAS_MAIL_SPEC.xlsx</x:v>
       </x:c>
     </x:row>
+    <x:row r="140">
+      <x:c r="A140" s="19" t="str">
+        <x:v>ORG-MAIL-ID-AUTO</x:v>
+      </x:c>
+      <x:c r="B140" s="19" t="str">
+        <x:v>가입 ID 기반 Cresero 메일 주소 자동 예약</x:v>
+      </x:c>
+      <x:c r="C140" s="19" t="str">
+        <x:v>구현·로컬 전체 회귀 완료 / 운영 배포·외부 사서함 생성 대기</x:v>
+      </x:c>
+      <x:c r="D140" s="19" t="str">
+        <x:v>회원가입 ID를 소문자로 정규화하고 같은 id@cresero.com 주소를 승인 전 예약한다. 승인 시 조직 identity에 결속하며 거절 시 예약을 해제한다. 기존 NAS 계정은 충돌 없는 이메일형 ID만 PLANNED 주소로 연결하고 예약어·한글·형식 불일치는 REVIEW_REQUIRED로 유지한다.</x:v>
+      </x:c>
+      <x:c r="E140" s="19" t="str">
+        <x:v>ORG-MAIL-CONTROL, AUTH, STORAGE-QUOTA, Code_Map, API_Routes, Data_Files</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -15133,6 +15225,20 @@
         <x:v>대표이사·CTO 같은 회사 직책이 NAS MASTER 권한을 자동 부여하지 않으며, 메일 제공자 상태가 실제 사서함 상태의 정본이다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="208">
+      <x:c r="A208" s="19" t="str">
+        <x:v>ORG-MAIL-ID-AUTO</x:v>
+      </x:c>
+      <x:c r="B208" s="19" t="str">
+        <x:v>AUTH / ORG-MAIL-CONTROL / STORAGE-QUOTA</x:v>
+      </x:c>
+      <x:c r="C208" s="19" t="str">
+        <x:v>가입 요청 생성·승인·거절과 메일 주소 예약 수명주기를 결속한다. 실제 메일 제공자 상태가 ACTIVE가 아니면 주소는 PLANNED이며 외부 송수신을 주장하지 않는다.</x:v>
+      </x:c>
+      <x:c r="D208" s="19" t="str">
+        <x:v>회원가입 ID 형식, 공용 주소 예약어, 가입 대기 주소, 기존 사용자 identity, 20GiB 용량 예약을 함께 회귀 검증한다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -22216,6 +22322,76 @@
       </x:c>
       <x:c r="D505" s="19" t="str">
         <x:v>외부 유료 API 호출 없음</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="506">
+      <x:c r="A506" s="19" t="str">
+        <x:v>ORG-MAIL-ID-AUTO</x:v>
+      </x:c>
+      <x:c r="B506" s="19" t="str">
+        <x:v>backend/organizationDirectory.js</x:v>
+      </x:c>
+      <x:c r="C506" s="19" t="str">
+        <x:v>메일 주소 이름공간 검사, 가입 중 주소 예약·해제, 승인 결속, 기존 NAS 사용자 안전 백필</x:v>
+      </x:c>
+      <x:c r="D506" s="19" t="str">
+        <x:v>mailReservations; assertSignupAddressAvailable; reserveSignupAddress; releaseSignupAddress; reconcileExistingUserMailboxes</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="507">
+      <x:c r="A507" s="19" t="str">
+        <x:v>ORG-MAIL-ID-AUTO</x:v>
+      </x:c>
+      <x:c r="B507" s="19" t="str">
+        <x:v>backend/index.js</x:v>
+      </x:c>
+      <x:c r="C507" s="19" t="str">
+        <x:v>가입 ID 소문자 정규화, 계정·메일 통합 중복 확인, 승인·거절 수명주기 연결</x:v>
+      </x:c>
+      <x:c r="D507" s="19" t="str">
+        <x:v>/api/signup-request; /api/users/check-identity; /api/users/approve; /api/users/reject</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="508">
+      <x:c r="A508" s="19" t="str">
+        <x:v>ORG-MAIL-ID-AUTO</x:v>
+      </x:c>
+      <x:c r="B508" s="19" t="str">
+        <x:v>frontend/src/components/Signup.js</x:v>
+      </x:c>
+      <x:c r="C508" s="19" t="str">
+        <x:v>입력 ID와 자동 예약될 @cresero.com 주소를 한 화면에서 안내하고 충돌 원인을 표시</x:v>
+      </x:c>
+      <x:c r="D508" s="19" t="str">
+        <x:v>checkIdentity; reservedMailAddress; lowercase input normalization</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="509">
+      <x:c r="A509" s="19" t="str">
+        <x:v>ORG-MAIL-ID-AUTO</x:v>
+      </x:c>
+      <x:c r="B509" s="19" t="str">
+        <x:v>frontend/src/components/OrganizationMailSettings.js</x:v>
+      </x:c>
+      <x:c r="C509" s="19" t="str">
+        <x:v>내부 사용자 전용으로 오해되던 정책명을 승인된 전체 사용자 주소 자동 준비로 교정</x:v>
+      </x:c>
+      <x:c r="D509" s="19" t="str">
+        <x:v>autoIssueSignupMailbox policy switch</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="510">
+      <x:c r="A510" s="19" t="str">
+        <x:v>ORG-MAIL-ID-AUTO</x:v>
+      </x:c>
+      <x:c r="B510" s="19" t="str">
+        <x:v>backend/storageQuota.js; backend/tests/storageCapacity.test.js</x:v>
+      </x:c>
+      <x:c r="C510" s="19" t="str">
+        <x:v>이메일형 점 포함 로그인 ID의 개인 저장공간을 허용하되 선행·후행·연속 점과 경로 탈출 차단</x:v>
+      </x:c>
+      <x:c r="D510" s="19" t="str">
+        <x:v>isSafeLoginId; getCanonicalUserRoot</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: add root NAS connection bootstrap
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R06199fb0d0ea4ba3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R2d24519cd3644d0e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="Rca9d757306054812"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R853580f869944c67"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R61b99b2f8df24911"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Re9aea4ed734c4ab4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R775985c42f144c40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Redc6166fb3074cff"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rdc53cd16d27f40e6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Re984f3e676ed499c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R1739e48342e6422f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="Rdc2f91ae8693495a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="Rcfeddf81a83d4853"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="Rfde27a8c55ca4b91"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R3f03a3d979a8479a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf71fde14c9924347"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R5ce29b6461d74e2e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R16d440a0bd314ee4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Re8e628c77bbe4306"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R92e5467b4f6f44ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Rd02ae936ae454255"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R1e24cd44e175403a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R158fd17d6b364f77"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R55f4cfc95a6f4143"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rea7e5c513b6649b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R14b8fd44ee254f89"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R5037e2cfcc4c46e8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R55aa5a53798f4a9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R09970257e02a4555"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R74e9441268b547d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1048,6 +1048,20 @@
         <x:v>전력은 PSU 정격이나 CPU TDP로 추정하지 않는다. NAS에서 power*_input 또는 신뢰 가능한 UPS/스마트 플러그 연동이 생길 때만 표시한다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="29">
+      <x:c r="A29" t="str">
+        <x:v>Tailscale 상태 스냅샷</x:v>
+      </x:c>
+      <x:c r="B29" t="str">
+        <x:v>2026-10-16 · NAS chanyoung</x:v>
+      </x:c>
+      <x:c r="C29" t="str">
+        <x:v>Tailscale offline · node key expired · 100.80.39.112:22 실패 / LAN 192.168.45.30 SSH 성공</x:v>
+      </x:c>
+      <x:c r="D29" t="str">
+        <x:v>상태는 시간에 따라 바뀌므로 AI_CONNECTION_BOOTSTRAP.md의 명령으로 다시 확인한다. LAN 대체 SSH는 같은 사설망에서만 사용하고 HostKeyAlias=100.80.39.112와 host key 검증을 유지한다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5001,6 +5015,41 @@
       </x:c>
       <x:c r="K122" s="19" t="str"/>
     </x:row>
+    <x:row r="123">
+      <x:c r="A123" s="19" t="str">
+        <x:v>PATCH-AI-CONNECTION-BOOTSTRAP-2026-10-16</x:v>
+      </x:c>
+      <x:c r="B123" s="19" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="C123" s="19" t="str">
+        <x:v>완료 · 연결 문서·기록 검증 완료</x:v>
+      </x:c>
+      <x:c r="D123" s="19" t="str">
+        <x:v>다른 ChatGPT가 Tailscale 연결 기준을 다시 알아내지 않도록 Git 최상단에 비공개로 연결 정보를 기입하는 방식을 검토하고 적용해 달라는 요청.</x:v>
+      </x:c>
+      <x:c r="E123" s="19" t="str">
+        <x:v>기존 상세 연결 문서는 docs 아래에 있어 새 대화가 경로를 먼저 알지 못하면 놓칠 수 있었다. 반대로 credential을 Git에 넣으면 private 저장소라도 복제와 기록에 오래 남는다.</x:v>
+      </x:c>
+      <x:c r="F123" s="19" t="str">
+        <x:v>2026-10-16 실제 확인에서 Windows Tailscale은 로그인 상태였지만 NAS 노드는 35일 오프라인이고 node key가 만료되어 Tailscale SSH가 실패했다. 같은 LAN SSH는 정상 동작했다.</x:v>
+      </x:c>
+      <x:c r="G123" s="19" t="str">
+        <x:v>루트 AI_CONNECTION_BOOTSTRAP.md와 로컬 전용 예시를 추가하고 AGENTS.md 필독 순서에 연결했다. AI_CONNECTION_LOCAL.private.md는 gitignore에 등록했다. 추적 문서에는 비밀이 아닌 식별 정보·검증 명령·날짜 있는 상태만 기록한다.</x:v>
+      </x:c>
+      <x:c r="H123" s="19" t="str">
+        <x:v>tailscale status, tailscale ping, Tailscale TCP 22 실패를 확인했다. HostKeyAlias를 유지한 LAN SSH에서 whoami=limchanyoung, hostname=chanyoung, 기대 branch와 clean worktree를 확인했다. 변경 파일 비밀값 검사와 Git diff 검증을 수행한다.</x:v>
+      </x:c>
+      <x:c r="I123" s="19" t="str">
+        <x:v>Tailscale NAS node key 재인증은 NAS 로컬 화면 또는 별도 관리 경로가 필요하다. 스냅샷은 시간이 지나면 stale이므로 새 작업에서 다시 검사해야 한다.</x:v>
+      </x:c>
+      <x:c r="J123" s="19" t="str">
+        <x:v>AI-CONNECTION-BOOTSTRAP</x:v>
+      </x:c>
+      <x:c r="K123" s="19" t="str">
+        <x:v>AI_CONNECTION_BOOTSTRAP.md; AI_CONNECTION_LOCAL.example.md; AGENTS.md; .gitignore; docs/NAS_PROJECT_LOG.xlsx</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6218,6 +6267,17 @@
       </x:c>
       <x:c r="C109" s="19" t="str">
         <x:v>회원가입 때 입력한 ID로 id@cresero.com 주소를 자동 준비하고 기존 Cresero 주소와 중복되지 않게 하며, 기존 Cresero 계정도 NAS 계정과 연결해 달라는 요청.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="110">
+      <x:c r="A110" s="19" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="B110" s="19" t="str">
+        <x:v>Git 루트 NAS 연결 인수인계</x:v>
+      </x:c>
+      <x:c r="C110" s="19" t="str">
+        <x:v>다른 ChatGPT가 Tailscale 연결 기준을 매번 다시 알아내지 않도록 Git 최상단에서 바로 찾을 수 있게 비공개 연결 정보를 정리하는 방식을 검토하고 적용해 달라는 요청.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9916,6 +9976,20 @@
         <x:v>신규 ID는 소문자 영문·숫자·점만 허용하고 가입 요청 단계에서 id@cresero.com을 원자적으로 예약한다. NAS 사용자·가입 대기·개인 주소·공용/시스템 주소·예약 목록을 한 번에 검사한다. 제공자 UNCONFIGURED에서는 PLANNED만 사용하고 공용 주소는 사람 NAS 계정으로 만들지 않는다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="168">
+      <x:c r="A168" s="19" t="str">
+        <x:v>DNB-AI-CONNECTION-BOOTSTRAP-2026-10-16</x:v>
+      </x:c>
+      <x:c r="B168" s="19" t="str">
+        <x:v>Git 최상단 AI 연결 안내와 비밀정보 경계</x:v>
+      </x:c>
+      <x:c r="C168" s="19" t="str">
+        <x:v>비공개 Git 저장소라도 비밀번호, SSH 개인키, Tailscale auth key, API key, 쿠키, 세션 URL, Agent/DPAPI token을 연결 안내서에 저장하지 말 것. 날짜가 지난 Tailscale 상태를 현재 상태로 단정하지 말 것.</x:v>
+      </x:c>
+      <x:c r="D168" s="19" t="str">
+        <x:v>루트 AI_CONNECTION_BOOTSTRAP.md에는 비밀이 아닌 장치·주소·경로·검증 명령만 기록한다. 장치별 메모는 Git에서 제외된 AI_CONNECTION_LOCAL.private.md에 두되 그곳에도 credential은 넣지 않는다. 매 작업에서 status, ping, TCP 22, SSH를 다시 확인한다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -12312,6 +12386,23 @@
         <x:v>ORG-MAIL-CONTROL, AUTH, STORAGE-QUOTA, Code_Map, API_Routes, Data_Files</x:v>
       </x:c>
     </x:row>
+    <x:row r="141">
+      <x:c r="A141" s="19" t="str">
+        <x:v>AI-CONNECTION-BOOTSTRAP</x:v>
+      </x:c>
+      <x:c r="B141" s="19" t="str">
+        <x:v>새 ChatGPT/Codex용 Git 루트 연결 인덱스</x:v>
+      </x:c>
+      <x:c r="C141" s="19" t="str">
+        <x:v>완료 · 2026-10-16 실연결 상태 기록</x:v>
+      </x:c>
+      <x:c r="D141" s="19" t="str">
+        <x:v>저장소 루트에서 NAS 식별 정보, Tailscale·SSH 판단 순서, LAN 대체 경로, 사용자 승인 경계와 비밀정보 금지를 바로 찾는다. 상태 스냅샷은 날짜를 표시하고 매 작업에서 다시 검증한다.</x:v>
+      </x:c>
+      <x:c r="E141" s="19" t="str">
+        <x:v>AI_CONNECTION_BOOTSTRAP.md, AGENTS.md, Network_Config, Do_Not_Break, Patch_Log</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -15237,6 +15328,20 @@
       </x:c>
       <x:c r="D208" s="19" t="str">
         <x:v>회원가입 ID 형식, 공용 주소 예약어, 가입 대기 주소, 기존 사용자 identity, 20GiB 용량 예약을 함께 회귀 검증한다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="209">
+      <x:c r="A209" s="19" t="str">
+        <x:v>AI-CONNECTION-BOOTSTRAP</x:v>
+      </x:c>
+      <x:c r="B209" s="19" t="str">
+        <x:v>guards_and_routes</x:v>
+      </x:c>
+      <x:c r="C209" s="19" t="str">
+        <x:v>AI-RELAY / NET-TUNNEL / DEPLOY-PM2</x:v>
+      </x:c>
+      <x:c r="D209" s="19" t="str">
+        <x:v>새 대화는 루트 연결 인덱스에서 현재 네트워크를 직접 검증한 뒤 상세 handoff와 relay를 읽는다. 공개 사이트 200, Tailscale, SSH, NAS live worktree는 서로 별도로 확인한다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
ops: record Tailscale node reauthentication
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rf71fde14c9924347"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R5ce29b6461d74e2e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R16d440a0bd314ee4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Re8e628c77bbe4306"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R92e5467b4f6f44ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Rd02ae936ae454255"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R1e24cd44e175403a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R158fd17d6b364f77"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R55f4cfc95a6f4143"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rea7e5c513b6649b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R14b8fd44ee254f89"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R5037e2cfcc4c46e8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R55aa5a53798f4a9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R09970257e02a4555"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R74e9441268b547d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1ebcbf50421143ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R1d6a1b151e4843e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R5ead6044937d423d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R412f90b55afb4002"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="Radc4dfebd48f48b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R8e9b818044244da7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R1b846ade45254d1b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Ra8b74936784a4354"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R92ef280b76f845df"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R905356d034324b2c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Rfdc8e634f4aa441c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R88f5cdf5753f4e30"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R95827a571dd14a9e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="Recd3d43e830245bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R01740b331a584497"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1056,10 +1056,10 @@
         <x:v>2026-10-16 · NAS chanyoung</x:v>
       </x:c>
       <x:c r="C29" t="str">
-        <x:v>Tailscale offline · node key expired · 100.80.39.112:22 실패 / LAN 192.168.45.30 SSH 성공</x:v>
+        <x:v>node key 재인증 완료 · 100.80.39.112 · ping/TCP 22/SSH 성공</x:v>
       </x:c>
       <x:c r="D29" t="str">
-        <x:v>상태는 시간에 따라 바뀌므로 AI_CONNECTION_BOOTSTRAP.md의 명령으로 다시 확인한다. LAN 대체 SSH는 같은 사설망에서만 사용하고 HostKeyAlias=100.80.39.112와 host key 검증을 유지한다.</x:v>
+        <x:v>tailscaled enabled+active. immutable /etc/resolv.conf 때문에 Tailscale DNS health 경고가 남지만 NetworkManager DNS 조회와 backend/public HTTP는 정상이다. DNS 설정은 이번 작업에서 변경하지 않았다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -5050,6 +5050,41 @@
         <x:v>AI_CONNECTION_BOOTSTRAP.md; AI_CONNECTION_LOCAL.example.md; AGENTS.md; .gitignore; docs/NAS_PROJECT_LOG.xlsx</x:v>
       </x:c>
     </x:row>
+    <x:row r="124">
+      <x:c r="A124" s="19" t="str">
+        <x:v>PATCH-TAILSCALE-NODE-REAUTH-2026-10-16</x:v>
+      </x:c>
+      <x:c r="B124" s="19" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="C124" s="19" t="str">
+        <x:v>완료 · Tailscale·SSH 실검증</x:v>
+      </x:c>
+      <x:c r="D124" s="19" t="str">
+        <x:v>NAS 본체 쪽 Tailscale 재인증이 필요하다는 상태를 확인하고 복구해 달라는 요청.</x:v>
+      </x:c>
+      <x:c r="E124" s="19" t="str">
+        <x:v>tailscaled 서비스는 실행 중이었지만 장치가 Logged out이고 node key가 만료되어 Tailscale IP ping과 TCP 22가 실패했다.</x:v>
+      </x:c>
+      <x:c r="F124" s="19" t="str">
+        <x:v>NAS 시계와 NTP는 정상이었고 기존 사용자 프로필은 남아 있었다. LAN SSH로 접근 가능한 상태에서 공식 장치 로그인 URL을 발급했다.</x:v>
+      </x:c>
+      <x:c r="G124" s="19" t="str">
+        <x:v>기존 Tailnet 계정으로 장치를 재인증해 원래 100.80.39.112를 복구했다. credential은 저장하지 않았고 tailscaled enabled+active를 유지했다.</x:v>
+      </x:c>
+      <x:c r="H124" s="19" t="str">
+        <x:v>Windows status에서 chanyoung online, ping 약 1ms, TCP 22 true, ssh nas 성공. NAS에서 사용자·호스트·IP·branch·clean worktree, backend/public HTTP 200, 필수 서비스 active를 확인했다.</x:v>
+      </x:c>
+      <x:c r="I124" s="19" t="str">
+        <x:v>immutable /etc/resolv.conf 때문에 Tailscale DNS health 경고가 남아 있다. 일반 DNS는 정상이라 이번 작업에서는 DNS 구성과 immutable 속성을 변경하지 않았다.</x:v>
+      </x:c>
+      <x:c r="J124" s="19" t="str">
+        <x:v>AI-CONNECTION-BOOTSTRAP</x:v>
+      </x:c>
+      <x:c r="K124" s="19" t="str">
+        <x:v>AI_CONNECTION_BOOTSTRAP.md; docs/AI_MUST_READ_OTHER_PC_TAILSCALE_HANDOFF.md; AI_MUST_READ_PROJECT_RELAY.md; docs/NAS_PROJECT_LOG.xlsx</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6278,6 +6313,17 @@
       </x:c>
       <x:c r="C110" s="19" t="str">
         <x:v>다른 ChatGPT가 Tailscale 연결 기준을 매번 다시 알아내지 않도록 Git 최상단에서 바로 찾을 수 있게 비공개 연결 정보를 정리하는 방식을 검토하고 적용해 달라는 요청.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="111">
+      <x:c r="A111" s="19" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="B111" s="19" t="str">
+        <x:v>NAS Tailscale node key 재인증</x:v>
+      </x:c>
+      <x:c r="C111" s="19" t="str">
+        <x:v>NAS 본체 쪽 Tailscale 재인증이 필요하다는 상태를 확인하고 기존 Tailnet과 SSH 접근을 복구해 달라는 요청.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -9990,6 +10036,20 @@
         <x:v>루트 AI_CONNECTION_BOOTSTRAP.md에는 비밀이 아닌 장치·주소·경로·검증 명령만 기록한다. 장치별 메모는 Git에서 제외된 AI_CONNECTION_LOCAL.private.md에 두되 그곳에도 credential은 넣지 않는다. 매 작업에서 status, ping, TCP 22, SSH를 다시 확인한다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="169">
+      <x:c r="A169" s="19" t="str">
+        <x:v>DNB-TAILSCALE-DNS-IMMUTABLE-2026-10-16</x:v>
+      </x:c>
+      <x:c r="B169" s="19" t="str">
+        <x:v>Tailscale 재인증과 NAS DNS 경고 분리</x:v>
+      </x:c>
+      <x:c r="C169" s="19" t="str">
+        <x:v>node key 재인증과 /etc/resolv.conf DNS health 경고를 같은 문제로 보고 immutable 속성이나 NetworkManager DNS를 즉시 변경하지 말 것.</x:v>
+      </x:c>
+      <x:c r="D169" s="19" t="str">
+        <x:v>먼저 status·ping·TCP 22·SSH와 일반 DNS 조회를 각각 검증한다. 접속이 복구되고 일반 DNS가 정상이라면 경고를 비차단 상태로 기록하고, DNS 변경은 기존 네트워크 설계를 확인한 별도 작업에서만 수행한다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -12394,10 +12454,10 @@
         <x:v>새 ChatGPT/Codex용 Git 루트 연결 인덱스</x:v>
       </x:c>
       <x:c r="C141" s="19" t="str">
-        <x:v>완료 · 2026-10-16 실연결 상태 기록</x:v>
+        <x:v>완료 · NAS Tailscale 재인증·SSH 실검증</x:v>
       </x:c>
       <x:c r="D141" s="19" t="str">
-        <x:v>저장소 루트에서 NAS 식별 정보, Tailscale·SSH 판단 순서, LAN 대체 경로, 사용자 승인 경계와 비밀정보 금지를 바로 찾는다. 상태 스냅샷은 날짜를 표시하고 매 작업에서 다시 검증한다.</x:v>
+        <x:v>저장소 루트에서 NAS 식별 정보, Tailscale·SSH 판단 순서, LAN 대체 경로, 사용자 승인 경계와 비밀정보 금지를 바로 찾는다. 2026-10-16 NAS node key를 재인증해 기존 IP의 ping·TCP 22·SSH를 복구했고 상태는 매 작업에서 다시 검증한다.</x:v>
       </x:c>
       <x:c r="E141" s="19" t="str">
         <x:v>AI_CONNECTION_BOOTSTRAP.md, AGENTS.md, Network_Config, Do_Not_Break, Patch_Log</x:v>

</xml_diff>

<commit_message>
Connect Cresero employee identities and expose account status in NAS profiles
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1ebcbf50421143ec"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R1d6a1b151e4843e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R5ead6044937d423d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R412f90b55afb4002"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="Radc4dfebd48f48b2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R8e9b818044244da7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R1b846ade45254d1b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="Ra8b74936784a4354"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R92ef280b76f845df"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R905356d034324b2c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Rfdc8e634f4aa441c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R88f5cdf5753f4e30"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R95827a571dd14a9e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="Recd3d43e830245bb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R01740b331a584497"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rbbd124866f4548af"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Rb4b132e8fcbc4582"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R31c709d3a3ae4caf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R5fcee42180eb46e5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R1c0555a116394725"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R6516d3aed6074722"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R010d388087dc41d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R5e438b9c959c4d61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Re9a1ef4d96f44640"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R0a1574c6f94f49b0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R343dcb8927bf4594"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R442c607d381c40a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R14f3ab6629644eb8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R83e7a351a6474a45"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R997c360461c34d7d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5085,6 +5085,35 @@
         <x:v>AI_CONNECTION_BOOTSTRAP.md; docs/AI_MUST_READ_OTHER_PC_TAILSCALE_HANDOFF.md; AI_MUST_READ_PROJECT_RELAY.md; docs/NAS_PROJECT_LOG.xlsx</x:v>
       </x:c>
     </x:row>
+    <x:row r="125">
+      <x:c r="A125" s="19" t="str">
+        <x:v>PATCH-CRESERO-IDENTITY-20261016</x:v>
+      </x:c>
+      <x:c r="B125" s="19" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="C125" s="19" t="str">
+        <x:v>운영 연결·계정 이전 검증</x:v>
+      </x:c>
+      <x:c r="D125" s="19" t="str">
+        <x:v>기존 NAS 계정을 Cresero에 연결하고 초기 비밀번호 변경, 프로필 이메일·연결 버튼과 메일 프로젝트를 준비해 달라는 요청. 비밀번호 원문 제외.</x:v>
+      </x:c>
+      <x:c r="E125" s="19" t="str">
+        <x:v>NAS와 회사 계정의 연결 및 직원 구분 부재</x:v>
+      </x:c>
+      <x:c r="F125" s="19" t="str">
+        <x:v>Tailscale 재인증 후 NAS 고유 UID 기준으로 승인 회원을 확인</x:v>
+      </x:c>
+      <x:c r="G125" s="19" t="str">
+        <x:v>기존 25개 아이디를 Cresero 일반 계정으로 이전. 지정 직원 5개만 회사 주소와 기존 NAS UID 연결. 초기 비밀번호 변경 전 서비스 제한. NAS 프로필 연결 상태·메일 진입 추가.</x:v>
+      </x:c>
+      <x:c r="H125" s="19" t="str">
+        <x:v>Cresero 단위 검사 27개, NAS backend 180 pass·6 skip, UI contract 122, production build 및 HTTP 검증</x:v>
+      </x:c>
+      <x:c r="I125" s="19" t="str">
+        <x:v>NAS 비밀번호·역할·파일 경로 보존. admin 메일은 시스템 예약어를 피해 staff.admin. 실제 메일 제공자·메일 도메인·송수신은 미설정.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6324,6 +6353,17 @@
       </x:c>
       <x:c r="C111" s="19" t="str">
         <x:v>NAS 본체 쪽 Tailscale 재인증이 필요하다는 상태를 확인하고 기존 Tailnet과 SSH 접근을 복구해 달라는 요청.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="112">
+      <x:c r="A112" s="19" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="B112" s="19" t="str">
+        <x:v>Cresero/NAS 계정 연결·직원 이메일</x:v>
+      </x:c>
+      <x:c r="C112" s="19" t="str">
+        <x:v>기존 NAS 계정까지 연결하고 지정 초기 비밀번호(원문 제외)와 변경 기능을 구성. 직원은 dntdlzz, admin, cksdudstudy, cksdudproject, cmoe. NAS 프로필에 연결 버튼 또는 이메일 표시. Cresero 이메일 프로젝트 준비, 도메인은 추후 결정. 겹치는 계정은 통합.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7521,28 +7561,28 @@
         <x:v>2026-10-15</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>가입 주소 예약 구현·실제 제공자/기존 계정 SSO 대기</x:v>
+        <x:v>도메인·메일 제공자 선택 대기</x:v>
       </x:c>
       <x:c r="D11" t="str">
-        <x:v>ORG-MAIL-CONTROL</x:v>
+        <x:v>AUTH-CRESERO-IDENTITY / ORG-MAIL-CONTROL</x:v>
       </x:c>
       <x:c r="E11" t="str">
-        <x:v>cresero.com 실제 사서함·송수신·MFA·SPF/DKIM/DMARC·NAS 웹메일과 Cresero 기존 계정의 NAS SSO 활성화</x:v>
+        <x:v>Cresero 직원 이메일 송수신</x:v>
       </x:c>
       <x:c r="F11" t="str">
-        <x:v>메일 제공자 계정·요금제·관리 API 인증정보가 없고, Cresero Event Studio와 NAS는 서로 다른 비밀번호 해시·세션을 사용한다. 비밀번호 복사나 동일 ID 자동 병합은 계정 탈취 위험이 있어 금지한다.</x:v>
+        <x:v>메일 제공자와 서비스 도메인이 아직 미정</x:v>
       </x:c>
       <x:c r="G11" t="str">
-        <x:v>신규 NAS 가입 ID의 @cresero.com 예약·승인 결속·거절 해제와 기존 NAS 안전 백필은 구현됐다. 외부 제공자는 UNCONFIGURED이고 Event Studio 기존 계정 명단의 검증된 연결은 아직 없다.</x:v>
+        <x:v>직원 주소 예약과 메일 공간·NAS 프로필 연결 구현. 실제 사서함 송수신은 비활성.</x:v>
       </x:c>
       <x:c r="H11" t="str">
-        <x:v>메일 제공자 가입·관리 OAuth와 DNS 권한, Cresero↔NAS SSO 서명키·계정 소유권 검증 흐름 확정</x:v>
+        <x:v>사용자가 메일 도메인·제공자·비용 확정 및 제공자 연결</x:v>
       </x:c>
       <x:c r="I11" t="str">
-        <x:v>테스트 계정 1개로 Cresero 로그인→NAS 최초 활성화→20GiB 루트 생성→메일 사서함 프로비저닝→중복/충돌/정지/복구를 검증한 뒤 기존 계정을 일괄 이관한다.</x:v>
+        <x:v>제공자 앱 등록, 테스트 사서함 1개, 실제 송수신·권한·오프라인 검증</x:v>
       </x:c>
       <x:c r="J11" t="str">
-        <x:v>PATCH-ORG-MAIL-CONTROL-2026-10-15; PATCH-ORG-MAIL-ID-AUTO-2026-10-16; docs/programs/NAS_MAIL_SPEC.xlsx</x:v>
+        <x:v>PATCH-CRESERO-IDENTITY-20261016</x:v>
       </x:c>
       <x:c r="K11" t="str">
         <x:v>2026-10-16</x:v>
@@ -10050,6 +10090,20 @@
         <x:v>먼저 status·ping·TCP 22·SSH와 일반 DNS 조회를 각각 검증한다. 접속이 복구되고 일반 DNS가 정상이라면 경고를 비차단 상태로 기록하고, DNS 변경은 기존 네트워크 설계를 확인한 별도 작업에서만 수행한다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="170">
+      <x:c r="A170" s="19" t="str">
+        <x:v>DNB-CRESERO-IDENTITY-20261016</x:v>
+      </x:c>
+      <x:c r="B170" s="19" t="str">
+        <x:v>회사 계정·기존 NAS 연결</x:v>
+      </x:c>
+      <x:c r="C170" s="19" t="str">
+        <x:v>NAS UID 없이 닉네임만으로 계정을 합치거나, NAS MASTER를 회사 총관리자로 자동 복사하지 않는다. 임시 비밀번호 원문을 Git·문서·로그에 기록하지 않는다.</x:v>
+      </x:c>
+      <x:c r="D170" s="19" t="str">
+        <x:v>지정 직원만 연결하고 기존 계정의 UID·비밀번호·역할·파일 루트를 보존한다. 초기 비밀번호 변경 후 이용. 직원 주소 예약과 실제 메일 송수신을 구분한다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -12463,6 +12517,23 @@
         <x:v>AI_CONNECTION_BOOTSTRAP.md, AGENTS.md, Network_Config, Do_Not_Break, Patch_Log</x:v>
       </x:c>
     </x:row>
+    <x:row r="142">
+      <x:c r="A142" s="19" t="str">
+        <x:v>AUTH-CRESERO-IDENTITY</x:v>
+      </x:c>
+      <x:c r="B142" s="19" t="str">
+        <x:v>Cresero 계정·직원 NAS 연결</x:v>
+      </x:c>
+      <x:c r="C142" s="19" t="str">
+        <x:v>운영 적용·메일 제공자 대기</x:v>
+      </x:c>
+      <x:c r="D142" s="19" t="str">
+        <x:v>NAS UID를 공통 계정에 매핑하고 일반 회원과 지정 직원을 분리한다. 기존 NAS 권한·비밀번호·저장공간 유지. 메일함은 제공자 연결 전 비활성.</x:v>
+      </x:c>
+      <x:c r="E142" s="19" t="str">
+        <x:v>AUTH-SESSION, AUTH-ROLE, ORG-MAIL-CONTROL, Code_Map, 보류 작업</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -15404,6 +15475,20 @@
         <x:v>새 대화는 루트 연결 인덱스에서 현재 네트워크를 직접 검증한 뒤 상세 handoff와 relay를 읽는다. 공개 사이트 200, Tailscale, SSH, NAS live worktree는 서로 별도로 확인한다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="210">
+      <x:c r="A210" s="19" t="str">
+        <x:v>AUTH-CRESERO-IDENTITY</x:v>
+      </x:c>
+      <x:c r="B210" s="19" t="str">
+        <x:v>separates_authorization_from</x:v>
+      </x:c>
+      <x:c r="C210" s="19" t="str">
+        <x:v>AUTH-ROLE / ORG-MAIL-CONTROL</x:v>
+      </x:c>
+      <x:c r="D210" s="19" t="str">
+        <x:v>NAS MASTER/MANAGER를 회사 관리자·직원으로 자동 승격하지 않는다. 사용자 지정 직원만 주소 연결. 메일 PLANNED와 실제 송수신 구분.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -22557,6 +22642,20 @@
       </x:c>
       <x:c r="D510" s="19" t="str">
         <x:v>isSafeLoginId; getCanonicalUserRoot</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="511">
+      <x:c r="A511" s="19" t="str">
+        <x:v>AUTH-CRESERO-IDENTITY</x:v>
+      </x:c>
+      <x:c r="B511" s="19" t="str">
+        <x:v>backend/cresero-provisioner.cjs; backend/index.js; frontend/src/components/TopBar.js</x:v>
+      </x:c>
+      <x:c r="C511" s="19" t="str">
+        <x:v>30초 대기열 처리·기존 UID 연결·1회 NAS/Cresero 인증 티켓·프로필 이메일 표시</x:v>
+      </x:c>
+      <x:c r="D511" s="19" t="str">
+        <x:v>비밀값은 환경에만 저장. 기존 NAS 로그인·가입·비밀번호·역할·개인 루트 보존.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
Harden Cresero startup reconciliation and record full service QA
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rbbd124866f4548af"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Rb4b132e8fcbc4582"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R31c709d3a3ae4caf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R5fcee42180eb46e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R1c0555a116394725"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R6516d3aed6074722"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R010d388087dc41d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R5e438b9c959c4d61"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Re9a1ef4d96f44640"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R0a1574c6f94f49b0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R343dcb8927bf4594"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R442c607d381c40a9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R14f3ab6629644eb8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R83e7a351a6474a45"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R997c360461c34d7d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rcf8c4a16bc704d18"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R9006975352be42fa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R60e1244c6bdd4cbe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Rfd6548727a3e46ca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="Rc5d475177aec41e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R5a448d775c2a41d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R7722226863de4fb7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R7019b06bc3a042e4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R3f869eaa53c74f08"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R27ff0c3252b64562"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Rc9994f2803b44cbb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R48913d63ee6e405d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R8a40ed4f2e3f4b7e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R1ac3a528961d4fde"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Ra70387052416403f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5114,6 +5114,35 @@
         <x:v>NAS 비밀번호·역할·파일 경로 보존. admin 메일은 시스템 예약어를 피해 staff.admin. 실제 메일 제공자·메일 도메인·송수신은 미설정.</x:v>
       </x:c>
     </x:row>
+    <x:row r="126">
+      <x:c r="A126" s="19" t="str">
+        <x:v>PATCH-CRESERO-QA-20261016</x:v>
+      </x:c>
+      <x:c r="B126" s="19" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="C126" s="19" t="str">
+        <x:v>완료·실제 사용자 SSO 확인 필요</x:v>
+      </x:c>
+      <x:c r="D126" s="19" t="str">
+        <x:v>ㄴ싹다 돌려봐 이상한점없는지 말이야.</x:v>
+      </x:c>
+      <x:c r="E126" s="19" t="str">
+        <x:v>정상 로그인 반복 제한, NAS 시작 시 일시적 명부 오류 전파, 역할별 메뉴 혼동, 퀴즈 거절 요청 뒤 스트림 오류</x:v>
+      </x:c>
+      <x:c r="F126" s="19" t="str">
+        <x:v>로그인 성공에도 실패 카운터 누적; 명부 초기화 예외 미격리; 외부 운영자와 내부 관리 화면 혼용; 거절된 요청 본문 미소비</x:v>
+      </x:c>
+      <x:c r="G126" s="19" t="str">
+        <x:v>로그인 성공 시 실패 카운터 해제, 직원 명부 재조정 실패 격리 및 30초 재시도, 내부 관리·고객 운영자·직원 메일 메뉴 분리, 퀴즈 계정 API의 외부 출처 거절 전에 본문 정리. NAS .env 소유자를 원래 개발 계정으로 복구하고 0600 유지.</x:v>
+      </x:c>
+      <x:c r="H126" s="19" t="str">
+        <x:v>회사/NAS 29개 단위 검사, NAS 189 pass·6 skip, 퀴즈 로그인 65·계정 연결/복구 78·QR 98, 타입 검사·production build·역할별 브라우저 검사. NAS 25명 비밀번호·권한·저장 경로 보존 및 직원 5명 연결 재확인.</x:v>
+      </x:c>
+      <x:c r="I126" s="19" t="str">
+        <x:v>기존 PC 전용 fixture가 필요한 퀴즈 4개 검사는 미실행. Google/Meta 앱 및 실제 메일 제공자 미설정. 사용자 직접 초기 비밀번호 변경 후 실제 SSO 클릭 확인 필요.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6364,6 +6393,17 @@
       </x:c>
       <x:c r="C112" s="19" t="str">
         <x:v>기존 NAS 계정까지 연결하고 지정 초기 비밀번호(원문 제외)와 변경 기능을 구성. 직원은 dntdlzz, admin, cksdudstudy, cksdudproject, cmoe. NAS 프로필에 연결 버튼 또는 이메일 표시. Cresero 이메일 프로젝트 준비, 도메인은 추후 결정. 겹치는 계정은 통합.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="113">
+      <x:c r="A113" s="19" t="str">
+        <x:v>2026-10-16</x:v>
+      </x:c>
+      <x:c r="B113" s="19" t="str">
+        <x:v>Cresero·퀴즈·NAS 전체 회귀 점검</x:v>
+      </x:c>
+      <x:c r="C113" s="19" t="str">
+        <x:v>ㄴ싹다 돌려봐 이상한점없는지 말이야.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10104,6 +10144,20 @@
         <x:v>지정 직원만 연결하고 기존 계정의 UID·비밀번호·역할·파일 루트를 보존한다. 초기 비밀번호 변경 후 이용. 직원 주소 예약과 실제 메일 송수신을 구분한다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="171">
+      <x:c r="A171" s="19" t="str">
+        <x:v>DNB-CRESERO-QA-20261016</x:v>
+      </x:c>
+      <x:c r="B171" s="19" t="str">
+        <x:v>계정 연동 장애 격리와 환경 소유권</x:v>
+      </x:c>
+      <x:c r="C171" s="19" t="str">
+        <x:v>조직 명부 일시 오류 때문에 NAS 서버 시작이 중단되면 안 된다. 환경 파일 원자 교체 시 uid/gid를 root로 바꾸지 않는다. 로그인 성공을 실패 제한에 누적하지 않는다.</x:v>
+      </x:c>
+      <x:c r="D171" s="19" t="str">
+        <x:v>직원별 초기화 예외를 격리하고 30초 폴링에서 재시도한다. .env는 기존 소유자와 0600을 보존한다. NAS 기존 비밀번호·권한·root와 지정 직원 5명만 연결하는 경계를 회귀 검사한다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
fix: open master file manager at NAS root
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rcf8c4a16bc704d18"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R9006975352be42fa"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R60e1244c6bdd4cbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Rfd6548727a3e46ca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="Rc5d475177aec41e7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R5a448d775c2a41d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R7722226863de4fb7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R7019b06bc3a042e4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R3f869eaa53c74f08"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R27ff0c3252b64562"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Rc9994f2803b44cbb"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R48913d63ee6e405d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R8a40ed4f2e3f4b7e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R1ac3a528961d4fde"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Ra70387052416403f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc1d9e61638f84040"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R37936e911ac34fa2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R59ddd41b73164149"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R8ad96b236bf04036"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R3304baf877f44445"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Ra827ca83c5b446d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R744fed1e3e9b49d1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R8ff1897965554fd5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Ref4d14f2686e4eee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rdd15d244be0b4b3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R6d18f0dd57f94b4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R38104778145c4426"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="Rfe8b1a35d6754339"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="Rc6bbbb58aaab4cfd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R267fe787048d42d8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5143,6 +5143,41 @@
         <x:v>기존 PC 전용 fixture가 필요한 퀴즈 4개 검사는 미실행. Google/Meta 앱 및 실제 메일 제공자 미설정. 사용자 직접 초기 비밀번호 변경 후 실제 SSO 클릭 확인 필요.</x:v>
       </x:c>
     </x:row>
+    <x:row r="127">
+      <x:c r="A127" s="19" t="str">
+        <x:v>PATCH-MASTER-ROOT-ENTRY-20261030</x:v>
+      </x:c>
+      <x:c r="B127" s="19" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
+      <x:c r="C127" s="19" t="str">
+        <x:v>부분 확인 · 로컬 검증 완료 / 운영 배포 대기</x:v>
+      </x:c>
+      <x:c r="D127" s="19" t="str">
+        <x:v>기본 경로가 루트로 들어가지게 해 그냥</x:v>
+      </x:c>
+      <x:c r="E127" s="19" t="str">
+        <x:v>마스터가 파일관리자를 다시 열어도 계정별로 저장된 이전 하위 경로가 복원되어 NAS 전체 루트가 기본 화면으로 보이지 않았다.</x:v>
+      </x:c>
+      <x:c r="F127" s="19" t="str">
+        <x:v>계정별 마지막 파일관리자 경로 복원 정책이 역할과 무관하게 모든 계정에 동일 적용됐다.</x:v>
+      </x:c>
+      <x:c r="G127" s="19" t="str">
+        <x:v>MASTER 일반 진입·브라우저 복원·계정 전환에서는 /를 선택하는 공통 정책을 추가하고 플랫폼과 상단 파일관리자 진입에 적용했다. 목적지가 명시된 알림·최근 작업·폴더 열기는 변경하지 않았다.</x:v>
+      </x:c>
+      <x:c r="H127" s="19" t="str">
+        <x:v>fileManagerEntryPolicy 및 계정별 경로 테스트 6개 통과, DISABLE_ESLINT_PLUGIN=true production build 성공, git diff --check 통과. 현재 PC에서 NAS SSH 연결이 확인되지 않아 운영 실화면은 미검증.</x:v>
+      </x:c>
+      <x:c r="I127" s="19" t="str">
+        <x:v>일반 사용자·매니저의 마지막 경로 복원, 개인 quota와 Windows NAS Drive 개인 루트를 유지한다. NAS 연결 후 fast-forward·build·PM2 재시작 및 MASTER/USER 실제 진입을 회귀 검증한다.</x:v>
+      </x:c>
+      <x:c r="J127" s="19" t="str">
+        <x:v>NAS-MASTER-ROOT-ENTRY</x:v>
+      </x:c>
+      <x:c r="K127" s="19" t="str">
+        <x:v>frontend/src/utils/fileManagerEntryPolicy.js; frontend/src/contexts/WindowContext.js; frontend/src/components/ServicePlatform.js; frontend/src/components/TopBar.js</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6406,6 +6441,17 @@
         <x:v>ㄴ싹다 돌려봐 이상한점없는지 말이야.</x:v>
       </x:c>
     </x:row>
+    <x:row r="114">
+      <x:c r="A114" s="19" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
+      <x:c r="B114" s="19" t="str">
+        <x:v>마스터 파일관리자 기본 진입을 NAS 루트로 변경</x:v>
+      </x:c>
+      <x:c r="C114" s="19" t="str">
+        <x:v>기본 경로가 루트로 들어가지게 해 그냥</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7219,6 +7265,23 @@
       </x:c>
       <x:c r="E62" s="19" t="str">
         <x:v>provider UNCONFIGURED에서는 주소를 PLANNED로만 표시한다. 공용/시스템 주소는 개인 NAS 계정으로 만들지 않으며 기존 Cresero 비밀번호 해시는 복사하지 않는다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="63">
+      <x:c r="A63" s="19" t="str">
+        <x:v>2026-10-30 마스터 파일관리자 루트 기본 진입</x:v>
+      </x:c>
+      <x:c r="B63" s="19" t="str">
+        <x:v>MASTER 일반 진입과 저장 상태 복원은 /로 초기화하고 일반 사용자·매니저 및 명시적 목적지 이동은 보존했다.</x:v>
+      </x:c>
+      <x:c r="C63" s="19" t="str">
+        <x:v>정책·계정 경로 단위 테스트 6개; production build; git diff --check; artifact-tool 재계산·오류 검색·변경 행 렌더·문자 깨짐 검사</x:v>
+      </x:c>
+      <x:c r="D63" s="19" t="str">
+        <x:v>로컬 검증 완료 / NAS 운영 배포·실화면 검증 대기</x:v>
+      </x:c>
+      <x:c r="E63" s="19" t="str">
+        <x:v>현재 작업 PC는 ssh nas alias가 없고 100.80.39.112:22 직접 연결도 확인되지 않았다. 연결 가능한 환경에서 배포 후 MASTER와 USER를 각각 검증한다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7628,6 +7691,41 @@
         <x:v>2026-10-16</x:v>
       </x:c>
     </x:row>
+    <x:row r="12">
+      <x:c r="A12" s="19" t="str">
+        <x:v>PENDING-MASTER-ROOT-DEPLOY-20261030</x:v>
+      </x:c>
+      <x:c r="B12" s="19" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
+      <x:c r="C12" s="19" t="str">
+        <x:v>로컬 구현 완료·운영 배포 대기</x:v>
+      </x:c>
+      <x:c r="D12" s="19" t="str">
+        <x:v>NAS-MASTER-ROOT-ENTRY</x:v>
+      </x:c>
+      <x:c r="E12" s="19" t="str">
+        <x:v>마스터 파일관리자 기본 진입을 NAS 루트 /로 적용하고 실제 역할별 화면을 확인한다.</x:v>
+      </x:c>
+      <x:c r="F12" s="19" t="str">
+        <x:v>현재 작업 PC에서 SSH alias nas가 없고 Tailscale IP 100.80.39.112의 TCP 22 직접 연결도 확인되지 않아 운영 NAS에 반영할 수 없다.</x:v>
+      </x:c>
+      <x:c r="G12" s="19" t="str">
+        <x:v>공통 진입 정책 구현, 단위 테스트 6개와 production build 완료. 일반 사용자·매니저·명시적 목적지 경로 보존.</x:v>
+      </x:c>
+      <x:c r="H12" s="19" t="str">
+        <x:v>NAS가 켜져 있고 이 PC의 Tailscale·SSH 키 또는 LAN SSH 경로가 복구됨</x:v>
+      </x:c>
+      <x:c r="I12" s="19" t="str">
+        <x:v>NAS worktree 상태 확인 후 대상 commit fast-forward, frontend build, pm2-root 재시작, MASTER는 /mnt/nas 루트·USER는 개인 루트·알림 목적지는 지정 폴더로 열리는지 확인한다.</x:v>
+      </x:c>
+      <x:c r="J12" s="19" t="str">
+        <x:v>PATCH-MASTER-ROOT-ENTRY-20261030 / AI_MUST_READ_PROJECT_RELAY.md</x:v>
+      </x:c>
+      <x:c r="K12" s="19" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:conditionalFormatting sqref="C2:C500">
     <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="보류"/>
@@ -10158,6 +10256,20 @@
         <x:v>직원별 초기화 예외를 격리하고 30초 폴링에서 재시도한다. .env는 기존 소유자와 0600을 보존한다. NAS 기존 비밀번호·권한·root와 지정 직원 5명만 연결하는 경계를 회귀 검사한다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="172">
+      <x:c r="A172" s="19" t="str">
+        <x:v>DNB-MASTER-ROOT-ENTRY-20261030</x:v>
+      </x:c>
+      <x:c r="B172" s="19" t="str">
+        <x:v>마스터 웹 파일관리자 기본 경로</x:v>
+      </x:c>
+      <x:c r="C172" s="19" t="str">
+        <x:v>마스터의 웹 파일관리자 기본 진입을 NAS 루트로 바꾸더라도 일반 사용자·매니저의 계정별 마지막 경로, 개인 quota, Windows NAS Drive 동기화 루트를 전체 NAS로 확대하지 않는다.</x:v>
+      </x:c>
+      <x:c r="D172" s="19" t="str">
+        <x:v>파일 관리자 아이콘 진입과 저장 경로 복원에서만 MASTER를 /로 초기화한다. 알림·최근 작업·특정 폴더 열기의 명시적 목적지는 유지하고 서버의 기존 resolveInside·role 검사를 계속 사용한다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -12588,6 +12700,23 @@
         <x:v>AUTH-SESSION, AUTH-ROLE, ORG-MAIL-CONTROL, Code_Map, 보류 작업</x:v>
       </x:c>
     </x:row>
+    <x:row r="143">
+      <x:c r="A143" s="19" t="str">
+        <x:v>NAS-MASTER-ROOT-ENTRY</x:v>
+      </x:c>
+      <x:c r="B143" s="19" t="str">
+        <x:v>마스터 파일관리자 루트 기본 진입</x:v>
+      </x:c>
+      <x:c r="C143" s="19" t="str">
+        <x:v>로컬 구현·테스트 완료 / 운영 배포 대기</x:v>
+      </x:c>
+      <x:c r="D143" s="19" t="str">
+        <x:v>MASTER가 웹 파일관리자를 일반 진입하면 /에서 시작하고 서버에서 /mnt/nas로 해석된다. 일반 사용자·매니저의 마지막 경로 복원과 개인 PC 동기화·quota 경계는 유지한다.</x:v>
+      </x:c>
+      <x:c r="E143" s="19" t="str">
+        <x:v>AUTH-ROLE, STORAGE-QUOTA, NAS-PC-SYNC, Relation_Map, Code_Map, Patch_Log</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -15543,6 +15672,20 @@
         <x:v>NAS MASTER/MANAGER를 회사 관리자·직원으로 자동 승격하지 않는다. 사용자 지정 직원만 주소 연결. 메일 PLANNED와 실제 송수신 구분.</x:v>
       </x:c>
     </x:row>
+    <x:row r="211">
+      <x:c r="A211" s="19" t="str">
+        <x:v>NAS-MASTER-ROOT-ENTRY</x:v>
+      </x:c>
+      <x:c r="B211" s="19" t="str">
+        <x:v>uses_without_expanding</x:v>
+      </x:c>
+      <x:c r="C211" s="19" t="str">
+        <x:v>AUTH-ROLE / STORAGE-QUOTA / NAS-PC-SYNC</x:v>
+      </x:c>
+      <x:c r="D211" s="19" t="str">
+        <x:v>웹 파일관리자 일반 진입만 MASTER의 /로 초기화한다. 목적지 지정 이동은 보존하며 /mnt/nas 전체 접근을 개인 quota 또는 Windows Drive 전체 동기화 권한으로 전파하지 않는다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -22710,6 +22853,20 @@
       </x:c>
       <x:c r="D511" s="19" t="str">
         <x:v>비밀값은 환경에만 저장. 기존 NAS 로그인·가입·비밀번호·역할·개인 루트 보존.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="512">
+      <x:c r="A512" s="19" t="str">
+        <x:v>NAS-MASTER-ROOT-ENTRY</x:v>
+      </x:c>
+      <x:c r="B512" s="19" t="str">
+        <x:v>frontend/src/utils/fileManagerEntryPolicy.js; frontend/src/contexts/WindowContext.js; frontend/src/components/ServicePlatform.js; frontend/src/components/TopBar.js</x:v>
+      </x:c>
+      <x:c r="C512" s="19" t="str">
+        <x:v>MASTER 기본 경로 / 정책, 저장 경로 복원, 플랫폼·상단 파일관리자 진입에 공통 적용</x:v>
+      </x:c>
+      <x:c r="D512" s="19" t="str">
+        <x:v>알림·최근 작업·특정 폴더 열기의 명시적 경로는 덮어쓰지 않는다. USER/MANAGER 마지막 경로와 PC 동기화 개인 루트 유지.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>

<commit_message>
docs: record Zephyrus G14 Tailscale setup
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rc1d9e61638f84040"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R37936e911ac34fa2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R59ddd41b73164149"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R8ad96b236bf04036"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R3304baf877f44445"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Ra827ca83c5b446d4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R744fed1e3e9b49d1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R8ff1897965554fd5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Ref4d14f2686e4eee"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rdd15d244be0b4b3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R6d18f0dd57f94b4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R38104778145c4426"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="Rfe8b1a35d6754339"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="Rc6bbbb58aaab4cfd"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R267fe787048d42d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re572a0bbbd0a482c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R43d1cd4be0734236"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R362c933b0449424a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Ra38bc37e78a744ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R9665907e49164557"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Rd3ebd8545d48424b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Re36d822f4f3b429a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R6c6836e92b654bc6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rdd89f020ecf640c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rec441ab60f04462d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Reb781e20cdd842d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R461556fdea7e43fe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="Rb154572646fc41d3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R82deee41e85a4c12"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R7e64b31e6407493f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1062,6 +1062,20 @@
         <x:v>tailscaled enabled+active. immutable /etc/resolv.conf 때문에 Tailscale DNS health 경고가 남지만 NetworkManager DNS 조회와 backend/public HTTP는 정상이다. DNS 설정은 이번 작업에서 변경하지 않았다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="19" t="str">
+        <x:v>Zephyrus G14 작업 PC Tailscale</x:v>
+      </x:c>
+      <x:c r="B30" s="19" t="str">
+        <x:v>zephyrus-g14-laptop · 100.86.38.22</x:v>
+      </x:c>
+      <x:c r="C30" s="19" t="str">
+        <x:v>Tailscale 1.104.4 · 서비스 Running/Automatic · Tailnet online · DNSName zephyrus-g14-laptop.tailf3e023.ts.net</x:v>
+      </x:c>
+      <x:c r="D30" s="19" t="str">
+        <x:v>NAS chanyoung(100.80.39.112) ping은 DERP(tok) 경유 성공, direct 미성립. SSH는 도달했으나 새 PC의 known_hosts에 NAS host key가 없어 검증 실패로 중단했다. host key 확인을 끄지 않는다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5178,6 +5192,41 @@
         <x:v>frontend/src/utils/fileManagerEntryPolicy.js; frontend/src/contexts/WindowContext.js; frontend/src/components/ServicePlatform.js; frontend/src/components/TopBar.js</x:v>
       </x:c>
     </x:row>
+    <x:row r="128">
+      <x:c r="A128" s="19" t="str">
+        <x:v>PATCH-ZEPHYRUS-G14-TAILSCALE-20261030</x:v>
+      </x:c>
+      <x:c r="B128" s="19" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
+      <x:c r="C128" s="19" t="str">
+        <x:v>완료 · Tailscale 설치/등록/명명 · SSH host key 대조 대기</x:v>
+      </x:c>
+      <x:c r="D128" s="19" t="str">
+        <x:v>테일스케일을 내 pc에 설치좀해줘 알아서 그럼 / 지금 로그인한 장비 노트북을 제피러스 g14 노트북으로 설정해줘</x:v>
+      </x:c>
+      <x:c r="E128" s="19" t="str">
+        <x:v>새 작업 PC에 Tailscale이 없어 NAS Tailnet과 SSH에 접근할 수 없었고, 로그인 뒤 기본 장비명이 desktop-2u175f8로 표시됐다.</x:v>
+      </x:c>
+      <x:c r="F128" s="19" t="str">
+        <x:v>Windows에 Tailscale 패키지가 미설치였고 이 PC가 기존 Tailnet 장치로 등록되지 않았다.</x:v>
+      </x:c>
+      <x:c r="G128" s="19" t="str">
+        <x:v>winget 공식 Tailscale.Tailscale 1.104.4를 설치하고 사용자가 공식 로그인 페이지에서 인증했다. Tailscale hostname을 zephyrus-g14-laptop으로 설정했다. Windows 자체 컴퓨터 이름은 변경하지 않았다.</x:v>
+      </x:c>
+      <x:c r="H128" s="19" t="str">
+        <x:v>서비스 Running/Automatic, Self HostName zephyrus-g14-laptop, DNSName zephyrus-g14-laptop.tailf3e023.ts.net, IPv4 100.86.38.22, Online=true. NAS ping 2회 성공.</x:v>
+      </x:c>
+      <x:c r="I128" s="19" t="str">
+        <x:v>NAS ping은 DERP(tok) 경유이며 direct는 미성립이다. SSH host key 검증을 끄지 말고 신뢰된 기존 PC 또는 NAS 콘솔에서 지문을 대조한 뒤 known_hosts와 ssh nas alias를 설정한다.</x:v>
+      </x:c>
+      <x:c r="J128" s="19" t="str">
+        <x:v>AI-CONNECTION-BOOTSTRAP / NET-TAILSCALE</x:v>
+      </x:c>
+      <x:c r="K128" s="19" t="str">
+        <x:v>AI_MUST_READ_PROJECT_RELAY.md; Network_Config; 보류 작업</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6452,6 +6501,17 @@
         <x:v>기본 경로가 루트로 들어가지게 해 그냥</x:v>
       </x:c>
     </x:row>
+    <x:row r="115">
+      <x:c r="A115" s="19" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
+      <x:c r="B115" s="19" t="str">
+        <x:v>Zephyrus G14 작업 PC Tailscale 설치·장비명 설정</x:v>
+      </x:c>
+      <x:c r="C115" s="19" t="str">
+        <x:v>테일스케일을 내 pc에 설치좀해줘 알아서 그럼. 로그인한 장비 노트북을 제피러스 g14 노트북으로 설정해줘.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7282,6 +7342,23 @@
       </x:c>
       <x:c r="E63" s="19" t="str">
         <x:v>현재 작업 PC는 ssh nas alias가 없고 100.80.39.112:22 직접 연결도 확인되지 않았다. 연결 가능한 환경에서 배포 후 MASTER와 USER를 각각 검증한다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="64">
+      <x:c r="A64" s="19" t="str">
+        <x:v>2026-10-30 Zephyrus G14 Tailscale 설치·등록</x:v>
+      </x:c>
+      <x:c r="B64" s="19" t="str">
+        <x:v>공식 패키지 설치, 사용자 인증, 장비명·서비스·Tailnet online 및 NAS ping을 확인하고 SSH host key 미등록 상태를 별도 보류로 유지했다.</x:v>
+      </x:c>
+      <x:c r="C64" s="19" t="str">
+        <x:v>Tailscale version/status/status --json/ip/ping; Windows service; artifact-tool 재계산·오류 검색·변경 행 렌더·문자 깨짐 검사</x:v>
+      </x:c>
+      <x:c r="D64" s="19" t="str">
+        <x:v>Tailscale 작업 완료 / NAS SSH host key 대조·배포 대기</x:v>
+      </x:c>
+      <x:c r="E64" s="19" t="str">
+        <x:v>비밀번호·OTP·인증 토큰은 기록하지 않았다. SSH StrictHostKeyChecking을 우회하지 않았다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7699,7 +7776,7 @@
         <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="C12" s="19" t="str">
-        <x:v>로컬 구현 완료·운영 배포 대기</x:v>
+        <x:v>Tailscale 복구 완료·SSH host key 확인 대기</x:v>
       </x:c>
       <x:c r="D12" s="19" t="str">
         <x:v>NAS-MASTER-ROOT-ENTRY</x:v>
@@ -7708,19 +7785,19 @@
         <x:v>마스터 파일관리자 기본 진입을 NAS 루트 /로 적용하고 실제 역할별 화면을 확인한다.</x:v>
       </x:c>
       <x:c r="F12" s="19" t="str">
-        <x:v>현재 작업 PC에서 SSH alias nas가 없고 Tailscale IP 100.80.39.112의 TCP 22 직접 연결도 확인되지 않아 운영 NAS에 반영할 수 없다.</x:v>
+        <x:v>Tailscale 설치·Tailnet 등록·NAS ping은 복구됐다. 다만 새 PC known_hosts에 NAS host key가 없어 SSH 검증 단계에서 중단됐다.</x:v>
       </x:c>
       <x:c r="G12" s="19" t="str">
-        <x:v>공통 진입 정책 구현, 단위 테스트 6개와 production build 완료. 일반 사용자·매니저·명시적 목적지 경로 보존.</x:v>
+        <x:v>공통 진입 정책 구현과 테스트·build 완료. 이 PC는 zephyrus-g14-laptop(100.86.38.22)으로 online이고 NAS 100.80.39.112 ping 성공. SSH host key 검증은 우회하지 않았다.</x:v>
       </x:c>
       <x:c r="H12" s="19" t="str">
-        <x:v>NAS가 켜져 있고 이 PC의 Tailscale·SSH 키 또는 LAN SSH 경로가 복구됨</x:v>
+        <x:v>신뢰된 기존 PC 또는 NAS 콘솔에서 100.80.39.112의 SSH fingerprint를 대조하고 이 PC known_hosts에 승인 등록, SSH 공개키/alias 구성</x:v>
       </x:c>
       <x:c r="I12" s="19" t="str">
-        <x:v>NAS worktree 상태 확인 후 대상 commit fast-forward, frontend build, pm2-root 재시작, MASTER는 /mnt/nas 루트·USER는 개인 루트·알림 목적지는 지정 폴더로 열리는지 확인한다.</x:v>
+        <x:v>ssh nas로 NAS worktree 상태 확인 후 29021d1 fast-forward, frontend build, pm2-root 재시작, MASTER는 /mnt/nas 루트·USER는 개인 루트·알림 목적지는 지정 폴더로 열리는지 확인한다.</x:v>
       </x:c>
       <x:c r="J12" s="19" t="str">
-        <x:v>PATCH-MASTER-ROOT-ENTRY-20261030 / AI_MUST_READ_PROJECT_RELAY.md</x:v>
+        <x:v>PATCH-MASTER-ROOT-ENTRY-20261030 / PATCH-ZEPHYRUS-G14-TAILSCALE-20261030 / AI_MUST_READ_PROJECT_RELAY.md</x:v>
       </x:c>
       <x:c r="K12" s="19" t="str">
         <x:v>2026-10-30</x:v>

</xml_diff>

<commit_message>
docs: record Zephyrus SSH bootstrap blocker
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Re572a0bbbd0a482c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R43d1cd4be0734236"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R362c933b0449424a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Ra38bc37e78a744ba"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R9665907e49164557"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Rd3ebd8545d48424b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Re36d822f4f3b429a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R6c6836e92b654bc6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rdd89f020ecf640c5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rec441ab60f04462d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Reb781e20cdd842d9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R461556fdea7e43fe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="Rb154572646fc41d3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R82deee41e85a4c12"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R7e64b31e6407493f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R8c76698ff8944f8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Rb1c98d414b9d4556"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="Re0eddd87b3f34ac0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Rb183a608b3484ef9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="Rcbf4722540fc479f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Re370feb3dbd14a64"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Rc81bd8e0346d4bca"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R88beb41430594d3a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R1c0524a6895a43d2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R221b9c929dce4724"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Rb58e6b4b309c4080"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R6cabee5fcb0e4d70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R1cc22fad70bb4bfe"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R9d247bfaebc94761"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R23c0e972eb8b48e7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5227,6 +5227,41 @@
         <x:v>AI_MUST_READ_PROJECT_RELAY.md; Network_Config; 보류 작업</x:v>
       </x:c>
     </x:row>
+    <x:row r="129">
+      <x:c r="A129" s="19" t="str">
+        <x:v>PATCH-ZEPHYRUS-G14-SSH-BOOTSTRAP-20261030</x:v>
+      </x:c>
+      <x:c r="B129" s="19" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
+      <x:c r="C129" s="19" t="str">
+        <x:v>부분 확인 · 로컬 SSH 준비 완료 / NAS 공개키 등록 필요</x:v>
+      </x:c>
+      <x:c r="D129" s="19" t="str">
+        <x:v>어 전부다 해줄래?</x:v>
+      </x:c>
+      <x:c r="E129" s="19" t="str">
+        <x:v>새 노트북에서 NAS 배포까지 진행하려 했으나 NAS가 등록되지 않은 공개키를 거부했다.</x:v>
+      </x:c>
+      <x:c r="F129" s="19" t="str">
+        <x:v>NAS sshd는 publickey만 허용하고 이 노트북의 신규 키가 /home/limchanyoung/.ssh/authorized_keys에 아직 없다. Tailscale SSH도 서버에서 활성화되지 않았다.</x:v>
+      </x:c>
+      <x:c r="G129" s="19" t="str">
+        <x:v>승인된 NAS host key를 known_hosts에 등록하고 전용 ED25519 키와 ssh nas alias를 생성했다. 비밀번호 인증·Tailscale SSH·SMB·웹 API 대안을 확인했으나 안전한 서버측 키 등록 경로가 없어서 우회하지 않았다.</x:v>
+      </x:c>
+      <x:c r="H129" s="19" t="str">
+        <x:v>NAS host key 고정, 로컬 키 fingerprint SHA256:/yS8T5iWaLLUmMUAadIkUoTM8pUKh/EtcE5Hh5Fkfrw, ssh nas가 해당 키를 선택함. 일반·비밀번호 SSH는 모두 서버에서 publickey 거부.</x:v>
+      </x:c>
+      <x:c r="I129" s="19" t="str">
+        <x:v>NAS 콘솔 또는 이미 승인된 PC에서 공개키를 authorized_keys에 한 번 등록해야 한다. 개인키 원문을 Git·로그·채팅에 노출하지 않는다. 등록 뒤 895e359 배포와 역할별 검증을 재개한다.</x:v>
+      </x:c>
+      <x:c r="J129" s="19" t="str">
+        <x:v>AI-CONNECTION-BOOTSTRAP / NAS-MASTER-ROOT-ENTRY</x:v>
+      </x:c>
+      <x:c r="K129" s="19" t="str">
+        <x:v>AI_MUST_READ_PROJECT_RELAY.md; C:/Users/user/.ssh/config; 보류 작업</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6512,6 +6547,17 @@
         <x:v>테일스케일을 내 pc에 설치좀해줘 알아서 그럼. 로그인한 장비 노트북을 제피러스 g14 노트북으로 설정해줘.</x:v>
       </x:c>
     </x:row>
+    <x:row r="116">
+      <x:c r="A116" s="19" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
+      <x:c r="B116" s="19" t="str">
+        <x:v>Zephyrus G14 NAS SSH·배포 전체 진행</x:v>
+      </x:c>
+      <x:c r="C116" s="19" t="str">
+        <x:v>어 전부다 해줄래?</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7359,6 +7405,23 @@
       </x:c>
       <x:c r="E64" s="19" t="str">
         <x:v>비밀번호·OTP·인증 토큰은 기록하지 않았다. SSH StrictHostKeyChecking을 우회하지 않았다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="65">
+      <x:c r="A65" s="19" t="str">
+        <x:v>2026-10-30 Zephyrus G14 SSH bootstrap</x:v>
+      </x:c>
+      <x:c r="B65" s="19" t="str">
+        <x:v>NAS host key, 로컬 전용 ED25519 키와 ssh nas alias를 준비하고 서버가 publickey-only이며 신규 키 미등록으로 차단됨을 확인했다.</x:v>
+      </x:c>
+      <x:c r="C65" s="19" t="str">
+        <x:v>ssh strict host verification; publickey·password·keyboard-interactive·Tailscale SSH·SMB 경로 확인; artifact-tool 재계산·오류 검색·변경 행 렌더</x:v>
+      </x:c>
+      <x:c r="D65" s="19" t="str">
+        <x:v>로컬 준비 완료 / NAS authorized_keys 1회 등록 대기</x:v>
+      </x:c>
+      <x:c r="E65" s="19" t="str">
+        <x:v>host key 검증과 서버 인증을 우회하지 않았다. 개인키는 로컬 사용자 .ssh에만 존재하며 공개키만 기록했다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7776,28 +7839,28 @@
         <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="C12" s="19" t="str">
-        <x:v>Tailscale 복구 완료·SSH host key 확인 대기</x:v>
+        <x:v>로컬 SSH 준비 완료·NAS 공개키 등록 대기</x:v>
       </x:c>
       <x:c r="D12" s="19" t="str">
-        <x:v>NAS-MASTER-ROOT-ENTRY</x:v>
+        <x:v>NAS-MASTER-ROOT-ENTRY / AI-CONNECTION-BOOTSTRAP</x:v>
       </x:c>
       <x:c r="E12" s="19" t="str">
-        <x:v>마스터 파일관리자 기본 진입을 NAS 루트 /로 적용하고 실제 역할별 화면을 확인한다.</x:v>
+        <x:v>마스터 파일관리자 기본 진입을 NAS 루트 /로 배포하고 실제 역할별 화면을 확인한다.</x:v>
       </x:c>
       <x:c r="F12" s="19" t="str">
-        <x:v>Tailscale 설치·Tailnet 등록·NAS ping은 복구됐다. 다만 새 PC known_hosts에 NAS host key가 없어 SSH 검증 단계에서 중단됐다.</x:v>
+        <x:v>Tailscale·host key·로컬 ssh nas alias는 준비됐다. NAS sshd가 publickey-only이고 신규 노트북 공개키가 authorized_keys에 없어 서버 로그인만 차단된다.</x:v>
       </x:c>
       <x:c r="G12" s="19" t="str">
-        <x:v>공통 진입 정책 구현과 테스트·build 완료. 이 PC는 zephyrus-g14-laptop(100.86.38.22)으로 online이고 NAS 100.80.39.112 ping 성공. SSH host key 검증은 우회하지 않았다.</x:v>
+        <x:v>zephyrus-g14-laptop online, NAS ping 성공, NAS host key 고정, 전용 ED25519 키와 alias 생성. 비밀번호·Tailscale SSH·SMB·웹 API 우회 경로 없음.</x:v>
       </x:c>
       <x:c r="H12" s="19" t="str">
-        <x:v>신뢰된 기존 PC 또는 NAS 콘솔에서 100.80.39.112의 SSH fingerprint를 대조하고 이 PC known_hosts에 승인 등록, SSH 공개키/alias 구성</x:v>
+        <x:v>NAS 로컬 콘솔 또는 기존 승인 PC에서 공개키를 /home/limchanyoung/.ssh/authorized_keys에 중복 없이 1회 등록</x:v>
       </x:c>
       <x:c r="I12" s="19" t="str">
-        <x:v>ssh nas로 NAS worktree 상태 확인 후 29021d1 fast-forward, frontend build, pm2-root 재시작, MASTER는 /mnt/nas 루트·USER는 개인 루트·알림 목적지는 지정 폴더로 열리는지 확인한다.</x:v>
+        <x:v>ssh nas 연결 즉시 live worktree dirty 상태 확인·보존, 895e359 fast-forward, frontend build, pm2-root 재시작·save, 필수 서비스·HTTP·MASTER/USER 경로 회귀 검증</x:v>
       </x:c>
       <x:c r="J12" s="19" t="str">
-        <x:v>PATCH-MASTER-ROOT-ENTRY-20261030 / PATCH-ZEPHYRUS-G14-TAILSCALE-20261030 / AI_MUST_READ_PROJECT_RELAY.md</x:v>
+        <x:v>PATCH-MASTER-ROOT-ENTRY-20261030 / PATCH-ZEPHYRUS-G14-TAILSCALE-20261030 / PATCH-ZEPHYRUS-G14-SSH-BOOTSTRAP-20261030</x:v>
       </x:c>
       <x:c r="K12" s="19" t="str">
         <x:v>2026-10-30</x:v>

</xml_diff>

<commit_message>
docs: record master root deployment verification
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R8c76698ff8944f8a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Rb1c98d414b9d4556"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="Re0eddd87b3f34ac0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="Rb183a608b3484ef9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="Rcbf4722540fc479f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="Re370feb3dbd14a64"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Rc81bd8e0346d4bca"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R88beb41430594d3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="R1c0524a6895a43d2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="R221b9c929dce4724"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Rb58e6b4b309c4080"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R6cabee5fcb0e4d70"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R1cc22fad70bb4bfe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R9d247bfaebc94761"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R23c0e972eb8b48e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1fdd1e66635c409d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R3813f273aa154cb1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R3f8d3de0306846c8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R4fd7ebf45829431d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R8c90559dea6a4f2d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R13a5da0ca9dc4707"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Raf0963475d3a422b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R35ed3933f16146ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rb3c447e1c8eb44c0"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rf9146c5e519146b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R065e5f43a18c4385"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R0dd7fbc9f2c64c5f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R6c4921af1f374d3f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R4be21ec93e3e4c21"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R77f3e98ee5d241cd"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1076,6 +1076,20 @@
         <x:v>NAS chanyoung(100.80.39.112) ping은 DERP(tok) 경유 성공, direct 미성립. SSH는 도달했으나 새 PC의 known_hosts에 NAS host key가 없어 검증 실패로 중단했다. host key 확인을 끄지 않는다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="19" t="str">
+        <x:v>마스터 루트 정책 운영 배포</x:v>
+      </x:c>
+      <x:c r="B31" s="19" t="str">
+        <x:v>cc81a95 · main.1a342207.js</x:v>
+      </x:c>
+      <x:c r="C31" s="19" t="str">
+        <x:v>PM2 online · 필수 6서비스 enabled+active · localhost/public HTTP 200</x:v>
+      </x:c>
+      <x:c r="D31" s="19" t="str">
+        <x:v>build/live index SHA-256 4dc9ab63638cd9998a637b75099c88082b4dc4ee091887982e9d0638712325a2. 배포 전 /var/www/html과 build는 /home/limchanyoung/msp-backups/master-root-entry-20261030-predeploy에 보존.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -5262,6 +5276,41 @@
         <x:v>AI_MUST_READ_PROJECT_RELAY.md; C:/Users/user/.ssh/config; 보류 작업</x:v>
       </x:c>
     </x:row>
+    <x:row r="130">
+      <x:c r="A130" s="19" t="str">
+        <x:v>PATCH-MASTER-ROOT-ENTRY-DEPLOY-20261030</x:v>
+      </x:c>
+      <x:c r="B130" s="19" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
+      <x:c r="C130" s="19" t="str">
+        <x:v>완료 · 운영 배포·실화면 검증</x:v>
+      </x:c>
+      <x:c r="D130" s="19" t="str">
+        <x:v>어 이제 깃에 다 반영해줬대. 자세히 읽어보고 이제 시작해봐</x:v>
+      </x:c>
+      <x:c r="E130" s="19" t="str">
+        <x:v>G14 SSH 키 등록 뒤 보류된 마스터 파일관리자 루트 기본 진입 변경을 NAS에 배포하고 실제 동작을 검증해야 했다.</x:v>
+      </x:c>
+      <x:c r="F130" s="19" t="str">
+        <x:v>NAS는 8549065로 원격보다 9개 커밋 뒤였고 운영 정적 bundle은 이전 build였다.</x:v>
+      </x:c>
+      <x:c r="G130" s="19" t="str">
+        <x:v>G14 ssh nas 재검증 후 clean worktree를 cc81a95까지 fast-forward했다. 테스트·build 통과 뒤 기존 운영 파일을 백업하고 frontend/build를 /var/www/html에 동기화했으며 PM2 재시작·save를 수행했다.</x:v>
+      </x:c>
+      <x:c r="H130" s="19" t="str">
+        <x:v>프런트 6 tests, UI contract 124, production/PDF.js build, backend 경계 7 tests 통과. build/live hash 일치. PM2 online, 6서비스 enabled+active, localhost/public 200. 실제 마스터 화면에서 서버 전체 저장소 / 및 하위 폴더 뒤 루트 복귀 확인.</x:v>
+      </x:c>
+      <x:c r="I130" s="19" t="str">
+        <x:v>일반 사용자·매니저 기억 경로와 개인 quota·Windows Drive는 확대하지 않는다. Tailscale SSH 자동 연결은 별도 보안 작업이다. rollback은 predeploy 백업을 사용한다.</x:v>
+      </x:c>
+      <x:c r="J130" s="19" t="str">
+        <x:v>NAS-MASTER-ROOT-ENTRY / AI-CONNECTION-BOOTSTRAP</x:v>
+      </x:c>
+      <x:c r="K130" s="19" t="str">
+        <x:v>frontend/src/utils/fileManagerEntryPolicy.js; frontend/src/contexts/WindowContext.js; frontend/src/components/ServicePlatform.js; frontend/src/components/TopBar.js</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6558,6 +6607,17 @@
         <x:v>어 전부다 해줄래?</x:v>
       </x:c>
     </x:row>
+    <x:row r="117">
+      <x:c r="A117" s="19" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
+      <x:c r="B117" s="19" t="str">
+        <x:v>Git 반영 확인 후 마스터 루트 정책 NAS 배포 재개</x:v>
+      </x:c>
+      <x:c r="C117" s="19" t="str">
+        <x:v>어 이제 깃에 다 반영해줬대. 자세히 읽어보고 이제 시작해봐</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7422,6 +7482,23 @@
       </x:c>
       <x:c r="E65" s="19" t="str">
         <x:v>host key 검증과 서버 인증을 우회하지 않았다. 개인키는 로컬 사용자 .ssh에만 존재하며 공개키만 기록했다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="66">
+      <x:c r="A66" s="19" t="str">
+        <x:v>2026-10-30 마스터 루트 정책 운영 배포</x:v>
+      </x:c>
+      <x:c r="B66" s="19" t="str">
+        <x:v>SSH 복구, NAS fast-forward, 테스트·build·정적 파일 배포·PM2 재시작과 마스터 실화면 검증을 완료했다.</x:v>
+      </x:c>
+      <x:c r="C66" s="19" t="str">
+        <x:v>frontend 6 tests; UI contract 124; production/PDF.js build; backend storage 7 tests; build/live SHA-256; PM2/services/HTTP; Chrome master root UI</x:v>
+      </x:c>
+      <x:c r="D66" s="19" t="str">
+        <x:v>운영 배포·실화면 검증 완료</x:v>
+      </x:c>
+      <x:c r="E66" s="19" t="str">
+        <x:v>일반 사용자·매니저 경로와 개인 quota/PC Drive 경계는 코드·서버 테스트로 유지했다. 운영 rollback 백업 위치를 기록했다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -7839,7 +7916,7 @@
         <x:v>2026-10-30</x:v>
       </x:c>
       <x:c r="C12" s="19" t="str">
-        <x:v>로컬 SSH 준비 완료·NAS 공개키 등록 대기</x:v>
+        <x:v>완료 · 운영 배포·실화면 검증</x:v>
       </x:c>
       <x:c r="D12" s="19" t="str">
         <x:v>NAS-MASTER-ROOT-ENTRY / AI-CONNECTION-BOOTSTRAP</x:v>
@@ -7848,19 +7925,19 @@
         <x:v>마스터 파일관리자 기본 진입을 NAS 루트 /로 배포하고 실제 역할별 화면을 확인한다.</x:v>
       </x:c>
       <x:c r="F12" s="19" t="str">
-        <x:v>Tailscale·host key·로컬 ssh nas alias는 준비됐다. NAS sshd가 publickey-only이고 신규 노트북 공개키가 authorized_keys에 없어 서버 로그인만 차단된다.</x:v>
+        <x:v>해결됨. G14 공개키 등록과 ssh nas 연결이 복구되어 NAS 배포를 수행했다.</x:v>
       </x:c>
       <x:c r="G12" s="19" t="str">
-        <x:v>zephyrus-g14-laptop online, NAS ping 성공, NAS host key 고정, 전용 ED25519 키와 alias 생성. 비밀번호·Tailscale SSH·SMB·웹 API 우회 경로 없음.</x:v>
+        <x:v>NAS cc81a95, main.1a342207.js, build/live hash 일치, PM2 online, 6서비스 enabled+active, localhost/public 200. 마스터 화면에서 /와 루트 복귀 확인. 경계 테스트 7개 통과.</x:v>
       </x:c>
       <x:c r="H12" s="19" t="str">
-        <x:v>NAS 로컬 콘솔 또는 기존 승인 PC에서 공개키를 /home/limchanyoung/.ssh/authorized_keys에 중복 없이 1회 등록</x:v>
+        <x:v>완료</x:v>
       </x:c>
       <x:c r="I12" s="19" t="str">
-        <x:v>ssh nas 연결 즉시 live worktree dirty 상태 확인·보존, 895e359 fast-forward, frontend build, pm2-root 재시작·save, 필수 서비스·HTTP·MASTER/USER 경로 회귀 검증</x:v>
+        <x:v>후속 변경 시 MASTER 일반 진입과 명시적 목적지 이동을 구분하고 USER/MANAGER 마지막 경로·개인 quota·Windows Drive를 회귀 검증한다.</x:v>
       </x:c>
       <x:c r="J12" s="19" t="str">
-        <x:v>PATCH-MASTER-ROOT-ENTRY-20261030 / PATCH-ZEPHYRUS-G14-TAILSCALE-20261030 / PATCH-ZEPHYRUS-G14-SSH-BOOTSTRAP-20261030</x:v>
+        <x:v>PATCH-MASTER-ROOT-ENTRY-DEPLOY-20261030 / AI_MUST_READ_PROJECT_RELAY.md</x:v>
       </x:c>
       <x:c r="K12" s="19" t="str">
         <x:v>2026-10-30</x:v>
@@ -12848,10 +12925,10 @@
         <x:v>마스터 파일관리자 루트 기본 진입</x:v>
       </x:c>
       <x:c r="C143" s="19" t="str">
-        <x:v>로컬 구현·테스트 완료 / 운영 배포 대기</x:v>
+        <x:v>운영 배포·실화면·역할 경계 검증 완료</x:v>
       </x:c>
       <x:c r="D143" s="19" t="str">
-        <x:v>MASTER가 웹 파일관리자를 일반 진입하면 /에서 시작하고 서버에서 /mnt/nas로 해석된다. 일반 사용자·매니저의 마지막 경로 복원과 개인 PC 동기화·quota 경계는 유지한다.</x:v>
+        <x:v>MASTER가 웹 파일관리자를 일반 진입하면 /에서 시작하고 서버에서 /mnt/nas로 해석된다. 실제 마스터 화면에서 하위 users 폴더 진입 뒤 파일 관리자 버튼으로 / 복귀를 확인했다. 일반 사용자·매니저 마지막 경로와 개인 PC 동기화·quota 경계는 유지한다.</x:v>
       </x:c>
       <x:c r="E143" s="19" t="str">
         <x:v>AUTH-ROLE, STORAGE-QUOTA, NAS-PC-SYNC, Relation_Map, Code_Map, Patch_Log</x:v>

</xml_diff>

<commit_message>
docs: record account workspace switching
</commit_message>
<xml_diff>
--- a/docs/NAS_PROJECT_LOG.xlsx
+++ b/docs/NAS_PROJECT_LOG.xlsx
@@ -2,21 +2,21 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R1fdd1e66635c409d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="R3813f273aa154cb1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R3f8d3de0306846c8"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R4fd7ebf45829431d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="R8c90559dea6a4f2d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R13a5da0ca9dc4707"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="Raf0963475d3a422b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R35ed3933f16146ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rb3c447e1c8eb44c0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rf9146c5e519146b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="R065e5f43a18c4385"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R0dd7fbc9f2c64c5f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R6c4921af1f374d3f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="R4be21ec93e3e4c21"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="R77f3e98ee5d241cd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R4478a09bdcd94a8a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Memory_Process" sheetId="2" r:id="Ra52a95daf9e14baa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Do_Not_Break" sheetId="3" r:id="R4cb211ae5fc04675"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Feature_Index" sheetId="4" r:id="R492a402b7729423a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Relation_Map" sheetId="5" r:id="Re6943d0e44c24463"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Code_Map" sheetId="6" r:id="R2086c7498e9549ec"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="API_Routes" sheetId="7" r:id="R30fa7446ce094fee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Socket_Events" sheetId="8" r:id="R41fe45fc866344d6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data_Files" sheetId="9" r:id="Rb4e38c508a33463e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Network_Config" sheetId="10" r:id="Rdeaebcaa11484a28"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office_Viewers" sheetId="11" r:id="Rc8ef491bf9644a57"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Patch_Log" sheetId="12" r:id="R640241e8b77d4e6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Request_Archive" sheetId="13" r:id="R3e53d3f048644d20"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Generated_Check" sheetId="14" r:id="Rb4226c9bae714bcc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="보류 작업" sheetId="15" r:id="Rbe666c1b437b4c39"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -5311,6 +5311,41 @@
         <x:v>frontend/src/utils/fileManagerEntryPolicy.js; frontend/src/contexts/WindowContext.js; frontend/src/components/ServicePlatform.js; frontend/src/components/TopBar.js</x:v>
       </x:c>
     </x:row>
+    <x:row r="131">
+      <x:c r="A131" s="25" t="str">
+        <x:v>PATCH-FILE-WORKSPACE-STORAGE-TOGGLE-20261030</x:v>
+      </x:c>
+      <x:c r="B131" s="25" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
+      <x:c r="C131" s="25" t="str">
+        <x:v>완료 · 운영 배포·자동 회귀 검증</x:v>
+      </x:c>
+      <x:c r="D131" s="25" t="str">
+        <x:v>파일 작업공간에 반영이 되게해줘 뭔가 on off 처럼 이제 좋은생각났는데 다른 권한의 계정들도 각 계정공간(내 계정공간) 현재 경로 사용량을 파일 작업공간에 표시되는 기본값이 되게 해줘. 창이 열리는게 아니라 이해했지?</x:v>
+      </x:c>
+      <x:c r="E131" s="25" t="str">
+        <x:v>마스터 저장공간 바로가리가 window 모드에서는 별도 폴더 창을 열었고, 다른 역할에는 계정공간 전환 상태가 없었다. 현재 경로 사용량도 포커스된 부동 창에 따라 바뀔 수 있었다.</x:v>
+      </x:c>
+      <x:c r="F131" s="25" t="str">
+        <x:v>이전 구현이 open mode에 따라 navigate 또는 openFolderWindow로 분기했고, 기본 경로 정책은 마스터만 /로 고정하고 나머지는 기억 경로를 복원했다.</x:v>
+      </x:c>
+      <x:c r="G131" s="25" t="str">
+        <x:v>모든 역할에 내 계정공간 선택 상태를 추가하고 저장공간 버튼은 항상 중앙 fileManagerPath만 전환하게 했다. MASTER만 전체 경로 선택을 표시한다. 현재 경로 사용량·동기화 폴링을 중앙 경로에 결속하고 계정별 기본 경로 정책을 MASTER /, MANAGER/globalAccess 개인 경로, USER 개인 root로 정리했다.</x:v>
+      </x:c>
+      <x:c r="H131" s="25" t="str">
+        <x:v>로컬·NAS 정책 5 tests, UI contract 124 source, production build, PDF.js 호환 통과. NAS ff-only 02730b1, build/live index SHA-256 일치, 운영 bundle main.4c0081c3.js, 필수 6서비스 active+enabled, PM2 online, localhost/public HTTP 200.</x:v>
+      </x:c>
+      <x:c r="I131" s="25" t="str">
+        <x:v>서버 role·resolveInside·quota·Windows Drive 개인 root를 확대하지 않는다. 역할별 실제 클릭 화면은 다음 사용자 세션에서 확인하되 자동 정책/빌드/운영 정적 배포 검증은 완료했다. rollback은 file-workspace-toggle-20261030-predeploy 백업을 사용한다.</x:v>
+      </x:c>
+      <x:c r="J131" s="25" t="str">
+        <x:v>NAS-MASTER-ROOT-ENTRY / AUTH-ROLE / STORAGE-QUOTA</x:v>
+      </x:c>
+      <x:c r="K131" s="25" t="str">
+        <x:v>frontend/src/components/NAS.js; frontend/src/utils/fileManagerEntryPolicy.js; frontend/src/contexts/WindowContext.js</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -6618,6 +6653,17 @@
         <x:v>어 이제 깃에 다 반영해줬대. 자세히 읽어보고 이제 시작해봐</x:v>
       </x:c>
     </x:row>
+    <x:row r="118">
+      <x:c r="A118" s="25" t="str">
+        <x:v>2026-10-30</x:v>
+      </x:c>
+      <x:c r="B118" s="25" t="str">
+        <x:v>계정별 파일 작업공간 기본값과 저장공간 토글</x:v>
+      </x:c>
+      <x:c r="C118" s="25" t="str">
+        <x:v>파일 작업공간에 반영이 되게해줘 뭔가 on off 처럼 이제 좋은생각났는데 다른 권한의 계정들도 각 계정공간(내 계정공간) 현재 경로 사용량을 파일 작업공간에 표시되는 기본값이 되게 해줘. 창이 열리는게 아니라 이해했지?</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -7499,6 +7545,23 @@
       </x:c>
       <x:c r="E66" s="19" t="str">
         <x:v>일반 사용자·매니저 경로와 개인 quota/PC Drive 경계는 코드·서버 테스트로 유지했다. 운영 rollback 백업 위치를 기록했다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="67">
+      <x:c r="A67" s="25" t="str">
+        <x:v>2026-10-30 계정별 파일 작업공간 전환</x:v>
+      </x:c>
+      <x:c r="B67" s="25" t="str">
+        <x:v>별도 창 없는 중앙 작업공간 토글, 역할별 계정공간 기본값, 마스터 전용 전체 경로 상태와 현재 경로 사용량 결속을 확인했다.</x:v>
+      </x:c>
+      <x:c r="C67" s="25" t="str">
+        <x:v>local/NAS 5 policy tests; UI contract 124; production/PDF.js build; ff-only deploy; build/live SHA-256; PM2/services/HTTP</x:v>
+      </x:c>
+      <x:c r="D67" s="25" t="str">
+        <x:v>운영 배포·자동 회귀 검증 완료</x:v>
+      </x:c>
+      <x:c r="E67" s="25" t="str">
+        <x:v>MASTER /, MANAGER/globalAccess /users/&lt;id&gt;, USER 서버 개인 root 경계를 유지한다. 실제 역할별 브라우저 클릭 확인은 다음 사용자 세션에서 수행 가능하다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -10474,17 +10537,17 @@
       </x:c>
     </x:row>
     <x:row r="172">
-      <x:c r="A172" s="19" t="str">
+      <x:c r="A172" s="25" t="str">
         <x:v>DNB-MASTER-ROOT-ENTRY-20261030</x:v>
       </x:c>
-      <x:c r="B172" s="19" t="str">
-        <x:v>마스터 웹 파일관리자 기본 경로</x:v>
-      </x:c>
-      <x:c r="C172" s="19" t="str">
-        <x:v>마스터의 웹 파일관리자 기본 진입을 NAS 루트로 바꾸더라도 일반 사용자·매니저의 계정별 마지막 경로, 개인 quota, Windows NAS Drive 동기화 루트를 전체 NAS로 확대하지 않는다.</x:v>
-      </x:c>
-      <x:c r="D172" s="19" t="str">
-        <x:v>파일 관리자 아이콘 진입과 저장 경로 복원에서만 MASTER를 /로 초기화한다. 알림·최근 작업·특정 폴더 열기의 명시적 목적지는 유지하고 서버의 기존 resolveInside·role 검사를 계속 사용한다.</x:v>
+      <x:c r="B172" s="25" t="str">
+        <x:v>계정별 파일 작업공간과 마스터 전체 경로</x:v>
+      </x:c>
+      <x:c r="C172" s="25" t="str">
+        <x:v>저장공간 바로가기는 새 폴더 창을 띄우지 않고 중앙 파일 작업공간만 전환해야 한다. 모든 계정의 기본 작업공간은 자기 계정공간이며, MASTER만 전체 NAS 루트 전환을 표시한다. 웹 전환을 개인 quota나 Windows NAS Drive 전체 동기화 권한으로 확대하지 않는다.</x:v>
+      </x:c>
+      <x:c r="D172" s="25" t="str">
+        <x:v>일반 USER의 /는 서버가 개인 root로 매핑한다. MANAGER/globalAccess는 /users/&lt;loginId&gt; 개인 경로를 기본값으로 사용하고 MASTER 기본값은 기존 요구대로 /를 유지하되 내 계정공간 버튼을 제공한다. 서버 resolveInside·최신 계정 role 검사를 유지하고 계정 전환 시 UI·경로·사용량을 함께 재평가한다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -12918,19 +12981,19 @@
       </x:c>
     </x:row>
     <x:row r="143">
-      <x:c r="A143" s="19" t="str">
+      <x:c r="A143" s="25" t="str">
         <x:v>NAS-MASTER-ROOT-ENTRY</x:v>
       </x:c>
-      <x:c r="B143" s="19" t="str">
-        <x:v>마스터 파일관리자 루트 기본 진입</x:v>
-      </x:c>
-      <x:c r="C143" s="19" t="str">
-        <x:v>운영 배포·실화면·역할 경계 검증 완료</x:v>
-      </x:c>
-      <x:c r="D143" s="19" t="str">
-        <x:v>MASTER가 웹 파일관리자를 일반 진입하면 /에서 시작하고 서버에서 /mnt/nas로 해석된다. 실제 마스터 화면에서 하위 users 폴더 진입 뒤 파일 관리자 버튼으로 / 복귀를 확인했다. 일반 사용자·매니저 마지막 경로와 개인 PC 동기화·quota 경계는 유지한다.</x:v>
-      </x:c>
-      <x:c r="E143" s="19" t="str">
+      <x:c r="B143" s="25" t="str">
+        <x:v>계정별 파일 작업공간 전환과 마스터 전체 경로</x:v>
+      </x:c>
+      <x:c r="C143" s="25" t="str">
+        <x:v>운영 배포·자동 회귀 검증 완료</x:v>
+      </x:c>
+      <x:c r="D143" s="25" t="str">
+        <x:v>Storage 블록의 내 계정공간/현재 경로 사용량이 중앙 파일 작업공간을 직접 전환한다. 모든 역할에 내 계정공간 상태를 표시하고 MASTER만 전체 경로 상태를 표시한다. MASTER 기본 진입 /, MANAGER·globalAccess 개인 /users/&lt;id&gt;, USER 서버 개인 root 매핑을 사용한다.</x:v>
+      </x:c>
+      <x:c r="E143" s="25" t="str">
         <x:v>AUTH-ROLE, STORAGE-QUOTA, NAS-PC-SYNC, Relation_Map, Code_Map, Patch_Log</x:v>
       </x:c>
     </x:row>
@@ -15890,17 +15953,17 @@
       </x:c>
     </x:row>
     <x:row r="211">
-      <x:c r="A211" s="19" t="str">
+      <x:c r="A211" s="25" t="str">
         <x:v>NAS-MASTER-ROOT-ENTRY</x:v>
       </x:c>
-      <x:c r="B211" s="19" t="str">
-        <x:v>uses_without_expanding</x:v>
-      </x:c>
-      <x:c r="C211" s="19" t="str">
+      <x:c r="B211" s="25" t="str">
+        <x:v>switches_workspace_without_expanding</x:v>
+      </x:c>
+      <x:c r="C211" s="25" t="str">
         <x:v>AUTH-ROLE / STORAGE-QUOTA / NAS-PC-SYNC</x:v>
       </x:c>
-      <x:c r="D211" s="19" t="str">
-        <x:v>웹 파일관리자 일반 진입만 MASTER의 /로 초기화한다. 목적지 지정 이동은 보존하며 /mnt/nas 전체 접근을 개인 quota 또는 Windows Drive 전체 동기화 권한으로 전파하지 않는다.</x:v>
+      <x:c r="D211" s="25" t="str">
+        <x:v>저장공간 버튼은 floating window를 만들지 않고 fileManagerPath를 전환한다. 모든 계정은 자기 공간을 기본으로 보며 MASTER만 전체 경로 UI를 가진다. 서버 권한·개인 quota·PC 동기화 경계는 기존대로 유지한다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -23073,17 +23136,17 @@
       </x:c>
     </x:row>
     <x:row r="512">
-      <x:c r="A512" s="19" t="str">
+      <x:c r="A512" s="25" t="str">
         <x:v>NAS-MASTER-ROOT-ENTRY</x:v>
       </x:c>
-      <x:c r="B512" s="19" t="str">
-        <x:v>frontend/src/utils/fileManagerEntryPolicy.js; frontend/src/contexts/WindowContext.js; frontend/src/components/ServicePlatform.js; frontend/src/components/TopBar.js</x:v>
-      </x:c>
-      <x:c r="C512" s="19" t="str">
-        <x:v>MASTER 기본 경로 / 정책, 저장 경로 복원, 플랫폼·상단 파일관리자 진입에 공통 적용</x:v>
-      </x:c>
-      <x:c r="D512" s="19" t="str">
-        <x:v>알림·최근 작업·특정 폴더 열기의 명시적 경로는 덮어쓰지 않는다. USER/MANAGER 마지막 경로와 PC 동기화 개인 루트 유지.</x:v>
+      <x:c r="B512" s="25" t="str">
+        <x:v>frontend/src/components/NAS.js; frontend/src/utils/fileManagerEntryPolicy.js; frontend/src/utils/fileManagerEntryPolicy.test.js; frontend/src/contexts/WindowContext.js; frontend/scripts/verify-ui-contract.mjs</x:v>
+      </x:c>
+      <x:c r="C512" s="25" t="str">
+        <x:v>중앙 파일 작업공간의 계정공간/전체 경로 토글, 계정별 기본 경로, 현재 경로 사용량, 계정 전환 반응 및 UI 계약 검증</x:v>
+      </x:c>
+      <x:c r="D512" s="25" t="str">
+        <x:v>MASTER 전체 경로만 별도 노출. USER의 /는 개인 root 의미이며 MANAGER/globalAccess 개인 경로를 /users/&lt;id&gt;로 계산한다. 새 창을 만들거나 PC 동기화 root를 넓히지 않는다.</x:v>
       </x:c>
     </x:row>
   </x:sheetData>

</xml_diff>